<commit_message>
Updated all code files to read new updated coin names
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E6D26BA-42D4-498B-B372-86587DE8D97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A571C446-F3B5-4CAD-94AF-6199012B7FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="23385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="632">
   <si>
     <t>Opponent</t>
   </si>
@@ -1353,9 +1353,6 @@
     <t>pikachu gold</t>
   </si>
   <si>
-    <t>pikachu gold 1</t>
-  </si>
-  <si>
     <t>pikachu gold 10</t>
   </si>
   <si>
@@ -1918,6 +1915,21 @@
   </si>
   <si>
     <t>Diglett Brown</t>
+  </si>
+  <si>
+    <t>Pikachu Gold</t>
+  </si>
+  <si>
+    <t>pikachu gold 11</t>
+  </si>
+  <si>
+    <t>Pidgeotto Silver</t>
+  </si>
+  <si>
+    <t>Caterpie Green</t>
+  </si>
+  <si>
+    <t>Tentacool Blue</t>
   </si>
 </sst>
 </file>
@@ -2265,7 +2277,7 @@
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Coin"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Granted By" dataDxfId="0">
-      <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(A2, opponents_table!C:C, opponents_table!A:A, "", 0), "")</calculatedColumnFormula>
+      <calculatedColumnFormula>_xlfn.XLOOKUP(A2, opponents_table!C:C, opponents_table!A:A, "", 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2892,7 +2904,7 @@
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>15</v>
@@ -2909,7 +2921,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>15</v>
@@ -2926,7 +2938,7 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>15</v>
@@ -2943,7 +2955,7 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>15</v>
@@ -2966,7 +2978,7 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>15</v>
@@ -2989,7 +3001,7 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>15</v>
@@ -3006,7 +3018,7 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>15</v>
@@ -3029,7 +3041,7 @@
         <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>15</v>
@@ -3046,7 +3058,7 @@
         <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>15</v>
@@ -3065,6 +3077,9 @@
       <c r="B18" t="s">
         <v>33</v>
       </c>
+      <c r="C18" t="s">
+        <v>627</v>
+      </c>
       <c r="G18" s="2" t="s">
         <v>15</v>
       </c>
@@ -3083,7 +3098,7 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>15</v>
@@ -3111,6 +3126,9 @@
       <c r="B20" t="s">
         <v>37</v>
       </c>
+      <c r="C20" t="s">
+        <v>631</v>
+      </c>
       <c r="G20" s="2" t="s">
         <v>15</v>
       </c>
@@ -3151,6 +3169,9 @@
       <c r="B22" t="s">
         <v>41</v>
       </c>
+      <c r="C22" t="s">
+        <v>629</v>
+      </c>
       <c r="G22" s="2" t="s">
         <v>15</v>
       </c>
@@ -3170,6 +3191,9 @@
       </c>
       <c r="B23" t="s">
         <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>630</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>15</v>
@@ -4314,7 +4338,7 @@
         <v>200</v>
       </c>
       <c r="B2" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A2, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A2, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4323,7 +4347,7 @@
         <v>201</v>
       </c>
       <c r="B3" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A3, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A3, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4332,7 +4356,7 @@
         <v>202</v>
       </c>
       <c r="B4" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A4, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A4, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4341,7 +4365,7 @@
         <v>203</v>
       </c>
       <c r="B5" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A5, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A5, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4350,7 +4374,7 @@
         <v>204</v>
       </c>
       <c r="B6" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A6, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A6, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4359,7 +4383,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A7, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A7, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4368,7 +4392,7 @@
         <v>206</v>
       </c>
       <c r="B8" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A8, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A8, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4377,7 +4401,7 @@
         <v>207</v>
       </c>
       <c r="B9" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A9, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A9, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4386,7 +4410,7 @@
         <v>208</v>
       </c>
       <c r="B10" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A10, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A10, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4395,7 +4419,7 @@
         <v>209</v>
       </c>
       <c r="B11" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A11, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A11, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4404,7 +4428,7 @@
         <v>210</v>
       </c>
       <c r="B12" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A12, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A12, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4413,7 +4437,7 @@
         <v>211</v>
       </c>
       <c r="B13" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A13, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A13, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4422,7 +4446,7 @@
         <v>212</v>
       </c>
       <c r="B14" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A14, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A14, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4431,7 +4455,7 @@
         <v>213</v>
       </c>
       <c r="B15" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A15, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A15, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4440,7 +4464,7 @@
         <v>214</v>
       </c>
       <c r="B16" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A16, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A16, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4449,7 +4473,7 @@
         <v>215</v>
       </c>
       <c r="B17" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A17, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A17, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4458,7 +4482,7 @@
         <v>216</v>
       </c>
       <c r="B18" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A18, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A18, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4467,7 +4491,7 @@
         <v>217</v>
       </c>
       <c r="B19" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A19, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A19, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4476,7 +4500,7 @@
         <v>218</v>
       </c>
       <c r="B20" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A20, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A20, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4485,7 +4509,7 @@
         <v>219</v>
       </c>
       <c r="B21" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A21, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A21, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4494,7 +4518,7 @@
         <v>220</v>
       </c>
       <c r="B22" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A22, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A22, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4503,7 +4527,7 @@
         <v>221</v>
       </c>
       <c r="B23" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A23, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A23, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4512,7 +4536,7 @@
         <v>222</v>
       </c>
       <c r="B24" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A24, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A24, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4521,7 +4545,7 @@
         <v>223</v>
       </c>
       <c r="B25" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A25, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A25, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4530,7 +4554,7 @@
         <v>224</v>
       </c>
       <c r="B26" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A26, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A26, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Gardener Callum</v>
       </c>
     </row>
@@ -4539,7 +4563,7 @@
         <v>225</v>
       </c>
       <c r="B27" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A27, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A27, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4548,8 +4572,8 @@
         <v>226</v>
       </c>
       <c r="B28" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A28, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
-        <v/>
+        <f>_xlfn.XLOOKUP(A28, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
+        <v>Bug Catcher Alex</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -4557,7 +4581,7 @@
         <v>227</v>
       </c>
       <c r="B29" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A29, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A29, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4566,7 +4590,7 @@
         <v>228</v>
       </c>
       <c r="B30" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A30, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A30, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4575,7 +4599,7 @@
         <v>229</v>
       </c>
       <c r="B31" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A31, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A31, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4584,7 +4608,7 @@
         <v>230</v>
       </c>
       <c r="B32" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A32, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A32, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4593,7 +4617,7 @@
         <v>231</v>
       </c>
       <c r="B33" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A33, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A33, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4602,7 +4626,7 @@
         <v>232</v>
       </c>
       <c r="B34" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A34, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A34, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4611,7 +4635,7 @@
         <v>233</v>
       </c>
       <c r="B35" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A35, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A35, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4620,7 +4644,7 @@
         <v>234</v>
       </c>
       <c r="B36" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A36, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A36, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4629,7 +4653,7 @@
         <v>235</v>
       </c>
       <c r="B37" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A37, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A37, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4638,7 +4662,7 @@
         <v>236</v>
       </c>
       <c r="B38" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A38, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A38, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4647,7 +4671,7 @@
         <v>237</v>
       </c>
       <c r="B39" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A39, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A39, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4656,7 +4680,7 @@
         <v>238</v>
       </c>
       <c r="B40" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A40, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A40, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4665,7 +4689,7 @@
         <v>239</v>
       </c>
       <c r="B41" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A41, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A41, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4674,7 +4698,7 @@
         <v>240</v>
       </c>
       <c r="B42" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A42, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A42, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4683,7 +4707,7 @@
         <v>241</v>
       </c>
       <c r="B43" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A43, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A43, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4692,7 +4716,7 @@
         <v>242</v>
       </c>
       <c r="B44" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A44, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A44, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4701,7 +4725,7 @@
         <v>243</v>
       </c>
       <c r="B45" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A45, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A45, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4710,7 +4734,7 @@
         <v>244</v>
       </c>
       <c r="B46" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A46, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A46, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4719,7 +4743,7 @@
         <v>245</v>
       </c>
       <c r="B47" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A47, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A47, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4728,7 +4752,7 @@
         <v>246</v>
       </c>
       <c r="B48" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A48, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A48, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4737,7 +4761,7 @@
         <v>247</v>
       </c>
       <c r="B49" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A49, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A49, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4746,7 +4770,7 @@
         <v>248</v>
       </c>
       <c r="B50" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A50, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A50, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4755,7 +4779,7 @@
         <v>249</v>
       </c>
       <c r="B51" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A51, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A51, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4764,7 +4788,7 @@
         <v>250</v>
       </c>
       <c r="B52" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A52, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A52, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4773,7 +4797,7 @@
         <v>251</v>
       </c>
       <c r="B53" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A53, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A53, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4782,7 +4806,7 @@
         <v>252</v>
       </c>
       <c r="B54" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A54, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A54, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4791,7 +4815,7 @@
         <v>253</v>
       </c>
       <c r="B55" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A55, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A55, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4800,7 +4824,7 @@
         <v>254</v>
       </c>
       <c r="B56" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A56, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A56, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4809,7 +4833,7 @@
         <v>255</v>
       </c>
       <c r="B57" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A57, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A57, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4818,7 +4842,7 @@
         <v>256</v>
       </c>
       <c r="B58" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A58, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A58, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4827,7 +4851,7 @@
         <v>257</v>
       </c>
       <c r="B59" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A59, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A59, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4836,7 +4860,7 @@
         <v>258</v>
       </c>
       <c r="B60" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A60, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A60, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4845,7 +4869,7 @@
         <v>259</v>
       </c>
       <c r="B61" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A61, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A61, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4854,7 +4878,7 @@
         <v>260</v>
       </c>
       <c r="B62" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A62, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A62, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4863,7 +4887,7 @@
         <v>261</v>
       </c>
       <c r="B63" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A63, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A63, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4872,7 +4896,7 @@
         <v>262</v>
       </c>
       <c r="B64" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A64, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A64, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4881,7 +4905,7 @@
         <v>263</v>
       </c>
       <c r="B65" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A65, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A65, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4890,7 +4914,7 @@
         <v>264</v>
       </c>
       <c r="B66" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A66, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A66, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4899,7 +4923,7 @@
         <v>265</v>
       </c>
       <c r="B67" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A67, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A67, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4908,7 +4932,7 @@
         <v>266</v>
       </c>
       <c r="B68" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A68, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A68, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4917,7 +4941,7 @@
         <v>267</v>
       </c>
       <c r="B69" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A69, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A69, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4926,7 +4950,7 @@
         <v>268</v>
       </c>
       <c r="B70" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A70, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A70, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Beach Kid Timothy</v>
       </c>
     </row>
@@ -4935,7 +4959,7 @@
         <v>269</v>
       </c>
       <c r="B71" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A71, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A71, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4944,7 +4968,7 @@
         <v>270</v>
       </c>
       <c r="B72" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A72, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A72, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4953,7 +4977,7 @@
         <v>271</v>
       </c>
       <c r="B73" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A73, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A73, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4962,7 +4986,7 @@
         <v>272</v>
       </c>
       <c r="B74" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A74, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A74, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4971,7 +4995,7 @@
         <v>273</v>
       </c>
       <c r="B75" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A75, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A75, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4980,7 +5004,7 @@
         <v>274</v>
       </c>
       <c r="B76" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A76, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A76, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4989,7 +5013,7 @@
         <v>275</v>
       </c>
       <c r="B77" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A77, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A77, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -4998,7 +5022,7 @@
         <v>276</v>
       </c>
       <c r="B78" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A78, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A78, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5007,7 +5031,7 @@
         <v>277</v>
       </c>
       <c r="B79" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A79, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A79, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5016,7 +5040,7 @@
         <v>278</v>
       </c>
       <c r="B80" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A80, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A80, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Schoolboy Adam</v>
       </c>
     </row>
@@ -5025,7 +5049,7 @@
         <v>279</v>
       </c>
       <c r="B81" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A81, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A81, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5034,7 +5058,7 @@
         <v>280</v>
       </c>
       <c r="B82" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A82, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A82, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5043,7 +5067,7 @@
         <v>281</v>
       </c>
       <c r="B83" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A83, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A83, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5052,7 +5076,7 @@
         <v>282</v>
       </c>
       <c r="B84" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A84, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A84, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5061,7 +5085,7 @@
         <v>283</v>
       </c>
       <c r="B85" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A85, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A85, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5070,7 +5094,7 @@
         <v>284</v>
       </c>
       <c r="B86" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A86, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A86, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5079,7 +5103,7 @@
         <v>285</v>
       </c>
       <c r="B87" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A87, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A87, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5088,7 +5112,7 @@
         <v>286</v>
       </c>
       <c r="B88" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A88, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A88, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5097,7 +5121,7 @@
         <v>287</v>
       </c>
       <c r="B89" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A89, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A89, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5106,7 +5130,7 @@
         <v>288</v>
       </c>
       <c r="B90" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A90, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A90, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Painter Jericho</v>
       </c>
     </row>
@@ -5115,7 +5139,7 @@
         <v>289</v>
       </c>
       <c r="B91" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A91, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A91, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5124,7 +5148,7 @@
         <v>290</v>
       </c>
       <c r="B92" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A92, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A92, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5133,7 +5157,7 @@
         <v>291</v>
       </c>
       <c r="B93" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A93, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A93, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5142,7 +5166,7 @@
         <v>292</v>
       </c>
       <c r="B94" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A94, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A94, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5151,7 +5175,7 @@
         <v>293</v>
       </c>
       <c r="B95" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A95, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A95, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5160,7 +5184,7 @@
         <v>294</v>
       </c>
       <c r="B96" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A96, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A96, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5169,7 +5193,7 @@
         <v>295</v>
       </c>
       <c r="B97" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A97, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A97, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5178,7 +5202,7 @@
         <v>296</v>
       </c>
       <c r="B98" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A98, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A98, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5187,7 +5211,7 @@
         <v>297</v>
       </c>
       <c r="B99" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A99, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A99, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5196,7 +5220,7 @@
         <v>298</v>
       </c>
       <c r="B100" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A100, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A100, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5205,7 +5229,7 @@
         <v>299</v>
       </c>
       <c r="B101" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A101, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A101, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5214,7 +5238,7 @@
         <v>300</v>
       </c>
       <c r="B102" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A102, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A102, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5223,7 +5247,7 @@
         <v>301</v>
       </c>
       <c r="B103" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A103, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A103, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5232,7 +5256,7 @@
         <v>302</v>
       </c>
       <c r="B104" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A104, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A104, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5241,7 +5265,7 @@
         <v>303</v>
       </c>
       <c r="B105" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A105, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A105, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5250,7 +5274,7 @@
         <v>304</v>
       </c>
       <c r="B106" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A106, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A106, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5259,7 +5283,7 @@
         <v>305</v>
       </c>
       <c r="B107" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A107, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A107, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5268,7 +5292,7 @@
         <v>306</v>
       </c>
       <c r="B108" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A108, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A108, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5277,7 +5301,7 @@
         <v>307</v>
       </c>
       <c r="B109" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A109, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A109, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5286,7 +5310,7 @@
         <v>308</v>
       </c>
       <c r="B110" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A110, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A110, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5295,7 +5319,7 @@
         <v>309</v>
       </c>
       <c r="B111" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A111, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A111, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5304,7 +5328,7 @@
         <v>310</v>
       </c>
       <c r="B112" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A112, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A112, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5313,7 +5337,7 @@
         <v>311</v>
       </c>
       <c r="B113" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A113, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A113, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5322,7 +5346,7 @@
         <v>312</v>
       </c>
       <c r="B114" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A114, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A114, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5331,7 +5355,7 @@
         <v>313</v>
       </c>
       <c r="B115" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A115, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A115, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5340,7 +5364,7 @@
         <v>314</v>
       </c>
       <c r="B116" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A116, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A116, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5349,7 +5373,7 @@
         <v>315</v>
       </c>
       <c r="B117" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A117, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A117, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5358,7 +5382,7 @@
         <v>316</v>
       </c>
       <c r="B118" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A118, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A118, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5367,7 +5391,7 @@
         <v>317</v>
       </c>
       <c r="B119" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A119, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A119, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5376,7 +5400,7 @@
         <v>318</v>
       </c>
       <c r="B120" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A120, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A120, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5385,7 +5409,7 @@
         <v>319</v>
       </c>
       <c r="B121" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A121, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A121, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5394,7 +5418,7 @@
         <v>320</v>
       </c>
       <c r="B122" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A122, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A122, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5403,7 +5427,7 @@
         <v>321</v>
       </c>
       <c r="B123" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A123, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A123, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5412,7 +5436,7 @@
         <v>322</v>
       </c>
       <c r="B124" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A124, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A124, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5421,7 +5445,7 @@
         <v>323</v>
       </c>
       <c r="B125" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A125, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A125, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5430,7 +5454,7 @@
         <v>324</v>
       </c>
       <c r="B126" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A126, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A126, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5439,7 +5463,7 @@
         <v>325</v>
       </c>
       <c r="B127" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A127, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A127, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Gambler Mick</v>
       </c>
     </row>
@@ -5448,7 +5472,7 @@
         <v>326</v>
       </c>
       <c r="B128" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A128, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A128, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5457,7 +5481,7 @@
         <v>327</v>
       </c>
       <c r="B129" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A129, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A129, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5466,7 +5490,7 @@
         <v>328</v>
       </c>
       <c r="B130" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A130, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A130, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5475,7 +5499,7 @@
         <v>329</v>
       </c>
       <c r="B131" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A131, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A131, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5484,7 +5508,7 @@
         <v>330</v>
       </c>
       <c r="B132" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A132, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A132, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5493,7 +5517,7 @@
         <v>331</v>
       </c>
       <c r="B133" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A133, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A133, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5502,7 +5526,7 @@
         <v>332</v>
       </c>
       <c r="B134" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A134, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A134, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5511,7 +5535,7 @@
         <v>333</v>
       </c>
       <c r="B135" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A135, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A135, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5520,7 +5544,7 @@
         <v>334</v>
       </c>
       <c r="B136" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A136, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A136, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5529,7 +5553,7 @@
         <v>335</v>
       </c>
       <c r="B137" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A137, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A137, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5538,7 +5562,7 @@
         <v>336</v>
       </c>
       <c r="B138" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A138, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A138, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5547,7 +5571,7 @@
         <v>337</v>
       </c>
       <c r="B139" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A139, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A139, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5556,7 +5580,7 @@
         <v>338</v>
       </c>
       <c r="B140" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A140, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A140, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5565,7 +5589,7 @@
         <v>339</v>
       </c>
       <c r="B141" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A141, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A141, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5574,7 +5598,7 @@
         <v>340</v>
       </c>
       <c r="B142" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A142, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A142, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5583,7 +5607,7 @@
         <v>341</v>
       </c>
       <c r="B143" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A143, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A143, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5592,7 +5616,7 @@
         <v>342</v>
       </c>
       <c r="B144" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A144, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A144, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5601,7 +5625,7 @@
         <v>343</v>
       </c>
       <c r="B145" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A145, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A145, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5610,7 +5634,7 @@
         <v>344</v>
       </c>
       <c r="B146" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A146, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A146, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5619,7 +5643,7 @@
         <v>345</v>
       </c>
       <c r="B147" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A147, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A147, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5628,7 +5652,7 @@
         <v>346</v>
       </c>
       <c r="B148" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A148, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A148, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5637,7 +5661,7 @@
         <v>347</v>
       </c>
       <c r="B149" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A149, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A149, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5646,7 +5670,7 @@
         <v>348</v>
       </c>
       <c r="B150" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A150, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A150, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5655,7 +5679,7 @@
         <v>349</v>
       </c>
       <c r="B151" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A151, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A151, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5664,7 +5688,7 @@
         <v>350</v>
       </c>
       <c r="B152" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A152, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A152, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5673,7 +5697,7 @@
         <v>351</v>
       </c>
       <c r="B153" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A153, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A153, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5682,7 +5706,7 @@
         <v>352</v>
       </c>
       <c r="B154" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A154, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A154, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5691,7 +5715,7 @@
         <v>353</v>
       </c>
       <c r="B155" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A155, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A155, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5700,7 +5724,7 @@
         <v>354</v>
       </c>
       <c r="B156" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A156, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A156, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5709,7 +5733,7 @@
         <v>355</v>
       </c>
       <c r="B157" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A157, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A157, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5718,7 +5742,7 @@
         <v>356</v>
       </c>
       <c r="B158" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A158, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A158, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5727,7 +5751,7 @@
         <v>357</v>
       </c>
       <c r="B159" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A159, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A159, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5736,7 +5760,7 @@
         <v>358</v>
       </c>
       <c r="B160" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A160, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A160, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5745,7 +5769,7 @@
         <v>359</v>
       </c>
       <c r="B161" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A161, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A161, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5754,7 +5778,7 @@
         <v>360</v>
       </c>
       <c r="B162" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A162, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A162, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5763,7 +5787,7 @@
         <v>361</v>
       </c>
       <c r="B163" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A163, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A163, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5772,7 +5796,7 @@
         <v>362</v>
       </c>
       <c r="B164" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A164, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A164, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5781,7 +5805,7 @@
         <v>363</v>
       </c>
       <c r="B165" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A165, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A165, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5790,7 +5814,7 @@
         <v>364</v>
       </c>
       <c r="B166" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A166, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A166, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5799,7 +5823,7 @@
         <v>365</v>
       </c>
       <c r="B167" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A167, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A167, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5808,7 +5832,7 @@
         <v>366</v>
       </c>
       <c r="B168" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A168, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A168, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5817,7 +5841,7 @@
         <v>367</v>
       </c>
       <c r="B169" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A169, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A169, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5826,7 +5850,7 @@
         <v>368</v>
       </c>
       <c r="B170" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A170, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A170, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5835,7 +5859,7 @@
         <v>369</v>
       </c>
       <c r="B171" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A171, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A171, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5844,7 +5868,7 @@
         <v>370</v>
       </c>
       <c r="B172" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A172, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A172, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5853,7 +5877,7 @@
         <v>371</v>
       </c>
       <c r="B173" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A173, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A173, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5862,7 +5886,7 @@
         <v>372</v>
       </c>
       <c r="B174" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A174, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A174, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5871,7 +5895,7 @@
         <v>373</v>
       </c>
       <c r="B175" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A175, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A175, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5880,7 +5904,7 @@
         <v>374</v>
       </c>
       <c r="B176" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A176, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A176, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5889,7 +5913,7 @@
         <v>375</v>
       </c>
       <c r="B177" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A177, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A177, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5898,7 +5922,7 @@
         <v>376</v>
       </c>
       <c r="B178" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A178, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A178, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5907,7 +5931,7 @@
         <v>377</v>
       </c>
       <c r="B179" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A179, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A179, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5916,7 +5940,7 @@
         <v>378</v>
       </c>
       <c r="B180" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A180, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A180, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5925,7 +5949,7 @@
         <v>379</v>
       </c>
       <c r="B181" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A181, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A181, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5934,7 +5958,7 @@
         <v>380</v>
       </c>
       <c r="B182" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A182, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A182, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5943,7 +5967,7 @@
         <v>381</v>
       </c>
       <c r="B183" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A183, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A183, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5952,7 +5976,7 @@
         <v>382</v>
       </c>
       <c r="B184" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A184, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A184, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5961,7 +5985,7 @@
         <v>383</v>
       </c>
       <c r="B185" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A185, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A185, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5970,7 +5994,7 @@
         <v>384</v>
       </c>
       <c r="B186" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A186, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A186, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5979,7 +6003,7 @@
         <v>385</v>
       </c>
       <c r="B187" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A187, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A187, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5988,7 +6012,7 @@
         <v>386</v>
       </c>
       <c r="B188" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A188, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A188, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -5997,7 +6021,7 @@
         <v>387</v>
       </c>
       <c r="B189" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A189, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A189, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6006,7 +6030,7 @@
         <v>388</v>
       </c>
       <c r="B190" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A190, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A190, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6015,7 +6039,7 @@
         <v>389</v>
       </c>
       <c r="B191" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A191, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A191, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6024,7 +6048,7 @@
         <v>390</v>
       </c>
       <c r="B192" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A192, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A192, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6033,7 +6057,7 @@
         <v>391</v>
       </c>
       <c r="B193" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A193, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A193, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6042,7 +6066,7 @@
         <v>392</v>
       </c>
       <c r="B194" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A194, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A194, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Fisherman Dave</v>
       </c>
     </row>
@@ -6051,7 +6075,7 @@
         <v>393</v>
       </c>
       <c r="B195" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A195, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A195, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6060,7 +6084,7 @@
         <v>394</v>
       </c>
       <c r="B196" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A196, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A196, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6069,7 +6093,7 @@
         <v>395</v>
       </c>
       <c r="B197" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A197, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A197, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6078,7 +6102,7 @@
         <v>396</v>
       </c>
       <c r="B198" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A198, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A198, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6087,7 +6111,7 @@
         <v>397</v>
       </c>
       <c r="B199" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A199, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A199, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6096,7 +6120,7 @@
         <v>398</v>
       </c>
       <c r="B200" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A200, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A200, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6105,7 +6129,7 @@
         <v>399</v>
       </c>
       <c r="B201" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A201, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A201, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6114,7 +6138,7 @@
         <v>400</v>
       </c>
       <c r="B202" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A202, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A202, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6123,7 +6147,7 @@
         <v>401</v>
       </c>
       <c r="B203" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A203, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A203, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6132,7 +6156,7 @@
         <v>402</v>
       </c>
       <c r="B204" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A204, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A204, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6141,7 +6165,7 @@
         <v>403</v>
       </c>
       <c r="B205" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A205, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A205, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6150,7 +6174,7 @@
         <v>404</v>
       </c>
       <c r="B206" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A206, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A206, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6159,7 +6183,7 @@
         <v>405</v>
       </c>
       <c r="B207" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A207, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A207, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6168,7 +6192,7 @@
         <v>406</v>
       </c>
       <c r="B208" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A208, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A208, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6177,7 +6201,7 @@
         <v>407</v>
       </c>
       <c r="B209" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A209, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A209, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6186,7 +6210,7 @@
         <v>408</v>
       </c>
       <c r="B210" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A210, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A210, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6195,7 +6219,7 @@
         <v>409</v>
       </c>
       <c r="B211" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A211, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A211, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6204,7 +6228,7 @@
         <v>410</v>
       </c>
       <c r="B212" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A212, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A212, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6213,7 +6237,7 @@
         <v>411</v>
       </c>
       <c r="B213" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A213, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A213, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6222,7 +6246,7 @@
         <v>412</v>
       </c>
       <c r="B214" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A214, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A214, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6231,7 +6255,7 @@
         <v>413</v>
       </c>
       <c r="B215" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A215, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A215, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6240,7 +6264,7 @@
         <v>414</v>
       </c>
       <c r="B216" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A216, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A216, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6249,7 +6273,7 @@
         <v>415</v>
       </c>
       <c r="B217" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A217, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A217, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6258,7 +6282,7 @@
         <v>416</v>
       </c>
       <c r="B218" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A218, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A218, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6267,7 +6291,7 @@
         <v>417</v>
       </c>
       <c r="B219" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A219, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A219, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6276,7 +6300,7 @@
         <v>418</v>
       </c>
       <c r="B220" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A220, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A220, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6285,7 +6309,7 @@
         <v>419</v>
       </c>
       <c r="B221" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A221, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A221, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6294,7 +6318,7 @@
         <v>420</v>
       </c>
       <c r="B222" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A222, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A222, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6303,7 +6327,7 @@
         <v>421</v>
       </c>
       <c r="B223" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A223, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A223, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6312,7 +6336,7 @@
         <v>422</v>
       </c>
       <c r="B224" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A224, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A224, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6321,7 +6345,7 @@
         <v>423</v>
       </c>
       <c r="B225" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A225, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A225, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6330,7 +6354,7 @@
         <v>424</v>
       </c>
       <c r="B226" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A226, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A226, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6339,7 +6363,7 @@
         <v>425</v>
       </c>
       <c r="B227" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A227, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A227, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6348,7 +6372,7 @@
         <v>426</v>
       </c>
       <c r="B228" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A228, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A228, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6357,7 +6381,7 @@
         <v>427</v>
       </c>
       <c r="B229" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A229, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A229, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6366,7 +6390,7 @@
         <v>428</v>
       </c>
       <c r="B230" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A230, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A230, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6375,7 +6399,7 @@
         <v>429</v>
       </c>
       <c r="B231" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A231, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A231, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6384,7 +6408,7 @@
         <v>430</v>
       </c>
       <c r="B232" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A232, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A232, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6393,7 +6417,7 @@
         <v>431</v>
       </c>
       <c r="B233" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A233, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A233, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6402,7 +6426,7 @@
         <v>432</v>
       </c>
       <c r="B234" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A234, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A234, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6411,7 +6435,7 @@
         <v>433</v>
       </c>
       <c r="B235" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A235, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A235, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6420,7 +6444,7 @@
         <v>434</v>
       </c>
       <c r="B236" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A236, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A236, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6429,8 +6453,8 @@
         <v>435</v>
       </c>
       <c r="B237" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A237, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
-        <v/>
+        <f>_xlfn.XLOOKUP(A237, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
+        <v>Birdspotter Tamsin</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
@@ -6438,7 +6462,7 @@
         <v>436</v>
       </c>
       <c r="B238" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A238, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A238, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6447,7 +6471,7 @@
         <v>437</v>
       </c>
       <c r="B239" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A239, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A239, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
@@ -6456,1618 +6480,1618 @@
         <v>438</v>
       </c>
       <c r="B240" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A240, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
-        <v/>
+        <f>_xlfn.XLOOKUP(A240, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
+        <v>Beach Kid Evie</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>439</v>
+        <v>628</v>
       </c>
       <c r="B241" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A241, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A241, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B242" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A242, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A242, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B243" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A243, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A243, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B244" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A244, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A244, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B245" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A245, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A245, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B246" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A246, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A246, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B247" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A247, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A247, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B248" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A248, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A248, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B249" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A249, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A249, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B250" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A250, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A250, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B251" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A251, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A251, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B252" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A252, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A252, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B253" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A253, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A253, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B254" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A254, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A254, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B255" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A255, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A255, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B256" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A256, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A256, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B257" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A257, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A257, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Swimmer Jordan</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B258" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A258, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A258, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B259" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A259, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A259, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B260" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A260, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A260, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B261" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A261, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A261, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B262" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A262, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A262, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B263" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A263, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A263, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B264" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A264, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A264, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B265" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A265, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A265, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B266" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A266, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A266, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B267" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A267, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A267, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B268" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A268, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A268, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B269" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A269, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A269, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B270" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A270, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A270, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B271" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A271, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A271, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B272" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A272, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A272, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Youngster Joey</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B273" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A273, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A273, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B274" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A274, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A274, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B275" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A275, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A275, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B276" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A276, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A276, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B277" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A277, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A277, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B278" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A278, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A278, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B279" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A279, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A279, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B280" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A280, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A280, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B281" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A281, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A281, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B282" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A282, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A282, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B283" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A283, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A283, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B284" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A284, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A284, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B285" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A285, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A285, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B286" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A286, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A286, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B287" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A287, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A287, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B288" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A288, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A288, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B289" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A289, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A289, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B290" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A290, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A290, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B291" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A291, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A291, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B292" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A292, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A292, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B293" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A293, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A293, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="294" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B294" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A294, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A294, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="295" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B295" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A295, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A295, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="296" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B296" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A296, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A296, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="297" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B297" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A297, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A297, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="298" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B298" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A298, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A298, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="299" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B299" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A299, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A299, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="300" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B300" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A300, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A300, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="301" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B301" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A301, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A301, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B302" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A302, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A302, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B303" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A303, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A303, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Fisherman John</v>
       </c>
     </row>
     <row r="304" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B304" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A304, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A304, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="305" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B305" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A305, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A305, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="306" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B306" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A306, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A306, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="307" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B307" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A307, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A307, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="308" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B308" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A308, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A308, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="309" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B309" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A309, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A309, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="310" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B310" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A310, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A310, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="311" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B311" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A311, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A311, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="312" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B312" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A312, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A312, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="313" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B313" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A313, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A313, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="314" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B314" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A314, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A314, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="315" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B315" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A315, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A315, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="316" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B316" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A316, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A316, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="317" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B317" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A317, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A317, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="318" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B318" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A318, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A318, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="319" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B319" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A319, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A319, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="320" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B320" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A320, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A320, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B321" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A321, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A321, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="322" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B322" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A322, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A322, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="323" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B323" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A323, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A323, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="324" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B324" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A324, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
-        <v/>
+        <f>_xlfn.XLOOKUP(A324, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
+        <v>Swimmer Todd</v>
       </c>
     </row>
     <row r="325" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B325" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A325, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A325, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="326" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B326" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A326, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A326, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="327" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B327" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A327, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A327, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="328" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B328" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A328, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A328, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="329" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B329" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A329, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A329, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="330" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B330" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A330, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A330, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="331" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B331" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A331, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A331, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="332" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B332" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A332, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A332, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="333" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B333" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A333, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A333, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="334" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B334" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A334, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A334, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="335" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B335" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A335, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A335, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="336" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B336" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A336, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A336, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="337" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B337" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A337, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A337, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="338" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B338" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A338, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A338, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="339" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B339" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A339, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A339, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="340" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B340" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A340, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A340, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="341" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B341" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A341, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A341, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="342" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B342" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A342, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A342, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="343" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B343" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A343, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A343, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="344" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B344" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A344, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A344, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="345" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B345" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A345, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A345, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="346" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B346" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A346, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A346, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="347" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B347" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A347, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A347, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="348" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B348" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A348, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A348, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="349" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B349" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A349, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A349, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v>Engineer Allan</v>
       </c>
     </row>
     <row r="350" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B350" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A350, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A350, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="351" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B351" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A351, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A351, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="352" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B352" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A352, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A352, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="353" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B353" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A353, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A353, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="354" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B354" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A354, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A354, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="355" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B355" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A355, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A355, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="356" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B356" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A356, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A356, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="357" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B357" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A357, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A357, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="358" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B358" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A358, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A358, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="359" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B359" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A359, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A359, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="360" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B360" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A360, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A360, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="361" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B361" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A361, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A361, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="362" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B362" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A362, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A362, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="363" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B363" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A363, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A363, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="364" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B364" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A364, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A364, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="365" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B365" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A365, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A365, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="366" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B366" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A366, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A366, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="367" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B367" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A367, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A367, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="368" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B368" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A368, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A368, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="369" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B369" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A369, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A369, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="370" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B370" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A370, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A370, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="371" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B371" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A371, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A371, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="372" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B372" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A372, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A372, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B373" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A373, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A373, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="374" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B374" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A374, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A374, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="375" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B375" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A375, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A375, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="376" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B376" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A376, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A376, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="377" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B377" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A377, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A377, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B378" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A378, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A378, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="379" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B379" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A379, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A379, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="380" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B380" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A380, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A380, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="381" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B381" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A381, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A381, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="382" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B382" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A382, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A382, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="383" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B383" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A383, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A383, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="384" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B384" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A384, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A384, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="385" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B385" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A385, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A385, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="386" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B386" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A386, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A386, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="387" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B387" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A387, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A387, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B388" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A388, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A388, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B389" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A389, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A389, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="390" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B390" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A390, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A390, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="391" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B391" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A391, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A391, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="392" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B392" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A392, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A392, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="393" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B393" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A393, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A393, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="394" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B394" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A394, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A394, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B395" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A395, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A395, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="396" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B396" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A396, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A396, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="397" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B397" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A397, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A397, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B398" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A398, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A398, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="399" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B399" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A399, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A399, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="400" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B400" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A400, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A400, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="401" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B401" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A401, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A401, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="402" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B402" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A402, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A402, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="403" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B403" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A403, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A403, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="404" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B404" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A404, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A404, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B405" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A405, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A405, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="406" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B406" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A406, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A406, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="407" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B407" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A407, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A407, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="408" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B408" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A408, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A408, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="409" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B409" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A409, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A409, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="410" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B410" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A410, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A410, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="411" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B411" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A411, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A411, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="412" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B412" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A412, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A412, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="413" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B413" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A413, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A413, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="414" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B414" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A414, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A414, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="415" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B415" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A415, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A415, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="416" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B416" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A416, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A416, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="417" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B417" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A417, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A417, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="418" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B418" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A418, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A418, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>
     <row r="419" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B419" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(A419, opponents_table!C:C, opponents_table!A:A, "", 0), "")</f>
+        <f>_xlfn.XLOOKUP(A419, opponents_table!C:C, opponents_table!A:A, "", 0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Started building gym decks
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{66A8ADB5-482C-46D4-8D06-96D08C7FCB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2678B9D-CF21-474D-8E0A-BBDFCF641016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="23385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
     <sheet name="coins_table" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="742">
   <si>
     <t>Opponent</t>
   </si>
@@ -2176,6 +2175,93 @@
   </si>
   <si>
     <t>Tourist Alissa</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Brock</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Misty</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Erika</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Koga</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Sabrina</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Blaine</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Giovanni</t>
+  </si>
+  <si>
+    <t>Gym Hero Brock</t>
+  </si>
+  <si>
+    <t>Gym Hero Misty</t>
+  </si>
+  <si>
+    <t>Gym Hero Lt. Surge</t>
+  </si>
+  <si>
+    <t>Ex Gym Leader Lt. Surge</t>
+  </si>
+  <si>
+    <t>Gym Hero Erika</t>
+  </si>
+  <si>
+    <t>Gym Hero Koga</t>
+  </si>
+  <si>
+    <t>Gym Hero Sabrina</t>
+  </si>
+  <si>
+    <t>Gym Hero Blaine</t>
+  </si>
+  <si>
+    <t>Gym Hero Giovanni</t>
+  </si>
+  <si>
+    <t>Brock</t>
+  </si>
+  <si>
+    <t>Misty</t>
+  </si>
+  <si>
+    <t>Lt. Surge</t>
+  </si>
+  <si>
+    <t>Erika</t>
+  </si>
+  <si>
+    <t>Koga</t>
+  </si>
+  <si>
+    <t>Sabrina</t>
+  </si>
+  <si>
+    <t>Blaine</t>
+  </si>
+  <si>
+    <t>Giovanni</t>
+  </si>
+  <si>
+    <t>Pewter Compassion</t>
+  </si>
+  <si>
+    <t>Pewter Crusher</t>
+  </si>
+  <si>
+    <t>Misty's Wrath</t>
+  </si>
+  <si>
+    <t>Dragon Rage</t>
+  </si>
+  <si>
+    <t>Cold Water Warmup</t>
   </si>
 </sst>
 </file>
@@ -2213,7 +2299,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="31">
+  <fills count="32">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2394,6 +2480,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2488,61 +2580,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90"/>
     </xf>
@@ -2652,6 +2689,61 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3038,7 +3130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z101"/>
+  <dimension ref="A1:Z125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -3049,77 +3141,77 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25" t="s">
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25" t="s">
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25" t="s">
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25" t="s">
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69" t="s">
         <v>694</v>
       </c>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25" t="s">
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69" t="s">
         <v>694</v>
       </c>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="25" t="s">
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69" t="s">
         <v>694</v>
       </c>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="25"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
     </row>
     <row r="2" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E2" s="48" t="s">
+      <c r="E2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="54" t="s">
+      <c r="G2" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="72" t="s">
+      <c r="H2" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="75" t="s">
+      <c r="I2" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="78" t="s">
+      <c r="J2" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="57" t="s">
+      <c r="K2" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="L2" s="60" t="s">
+      <c r="L2" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="M2" s="63" t="s">
+      <c r="M2" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="N2" s="66" t="s">
+      <c r="N2" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="O2" s="69" t="s">
+      <c r="O2" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="P2" s="46" t="s">
+      <c r="P2" s="27" t="s">
         <v>121</v>
       </c>
       <c r="Q2" s="18" t="s">
@@ -3151,47 +3243,47 @@
       </c>
     </row>
     <row r="3" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="72" t="s">
         <v>700</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="63" t="s">
         <v>695</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="49">
+      <c r="D3" s="63"/>
+      <c r="E3" s="30">
         <v>4</v>
       </c>
-      <c r="F3" s="52">
+      <c r="F3" s="33">
         <v>4</v>
       </c>
-      <c r="G3" s="55">
+      <c r="G3" s="36">
         <v>0</v>
       </c>
-      <c r="H3" s="73">
+      <c r="H3" s="54">
         <v>6</v>
       </c>
-      <c r="I3" s="76">
+      <c r="I3" s="57">
         <v>4</v>
       </c>
-      <c r="J3" s="79">
+      <c r="J3" s="60">
         <v>3</v>
       </c>
-      <c r="K3" s="58">
+      <c r="K3" s="39">
         <v>6</v>
       </c>
-      <c r="L3" s="61">
+      <c r="L3" s="42">
         <v>4</v>
       </c>
-      <c r="M3" s="64">
+      <c r="M3" s="45">
         <v>4</v>
       </c>
-      <c r="N3" s="67">
+      <c r="N3" s="48">
         <v>7</v>
       </c>
-      <c r="O3" s="70">
+      <c r="O3" s="51">
         <v>0</v>
       </c>
-      <c r="P3" s="47">
+      <c r="P3" s="28">
         <v>0</v>
       </c>
       <c r="Q3" s="17">
@@ -3223,45 +3315,45 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="29"/>
-      <c r="C4" s="33" t="s">
+      <c r="B4" s="73"/>
+      <c r="C4" s="63" t="s">
         <v>696</v>
       </c>
-      <c r="D4" s="33"/>
-      <c r="E4" s="49">
+      <c r="D4" s="63"/>
+      <c r="E4" s="30">
         <v>4</v>
       </c>
-      <c r="F4" s="52">
+      <c r="F4" s="33">
         <v>4</v>
       </c>
-      <c r="G4" s="55">
+      <c r="G4" s="36">
         <v>0</v>
       </c>
-      <c r="H4" s="73">
+      <c r="H4" s="54">
         <v>4</v>
       </c>
-      <c r="I4" s="76">
+      <c r="I4" s="57">
         <v>4</v>
       </c>
-      <c r="J4" s="79">
+      <c r="J4" s="60">
         <v>0</v>
       </c>
-      <c r="K4" s="58">
+      <c r="K4" s="39">
         <v>4</v>
       </c>
-      <c r="L4" s="61">
+      <c r="L4" s="42">
         <v>4</v>
       </c>
-      <c r="M4" s="64">
+      <c r="M4" s="45">
         <v>0</v>
       </c>
-      <c r="N4" s="67">
+      <c r="N4" s="48">
         <v>4</v>
       </c>
-      <c r="O4" s="70">
+      <c r="O4" s="51">
         <v>4</v>
       </c>
-      <c r="P4" s="47">
+      <c r="P4" s="28">
         <v>0</v>
       </c>
       <c r="Q4" s="17">
@@ -3293,45 +3385,45 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="29"/>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="73"/>
+      <c r="C5" s="63" t="s">
         <v>697</v>
       </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="49">
+      <c r="D5" s="63"/>
+      <c r="E5" s="30">
         <v>4</v>
       </c>
-      <c r="F5" s="52">
+      <c r="F5" s="33">
         <v>8</v>
       </c>
-      <c r="G5" s="55">
+      <c r="G5" s="36">
         <v>4</v>
       </c>
-      <c r="H5" s="73">
+      <c r="H5" s="54">
         <v>6</v>
       </c>
-      <c r="I5" s="76">
+      <c r="I5" s="57">
         <v>9</v>
       </c>
-      <c r="J5" s="79">
+      <c r="J5" s="60">
         <v>7</v>
       </c>
-      <c r="K5" s="58">
+      <c r="K5" s="39">
         <v>21</v>
       </c>
-      <c r="L5" s="61">
+      <c r="L5" s="42">
         <v>18</v>
       </c>
-      <c r="M5" s="64">
+      <c r="M5" s="45">
         <v>15</v>
       </c>
-      <c r="N5" s="67">
+      <c r="N5" s="48">
         <v>0</v>
       </c>
-      <c r="O5" s="70">
+      <c r="O5" s="51">
         <v>0</v>
       </c>
-      <c r="P5" s="47">
+      <c r="P5" s="28">
         <v>0</v>
       </c>
       <c r="Q5" s="3">
@@ -3377,13 +3469,13 @@
       <c r="V6" s="15"/>
     </row>
     <row r="7" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="74" t="s">
         <v>701</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="64" t="s">
         <v>695</v>
       </c>
-      <c r="D7" s="26"/>
+      <c r="D7" s="64"/>
       <c r="E7" s="17">
         <v>0</v>
       </c>
@@ -3440,11 +3532,11 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="31"/>
-      <c r="C8" s="26" t="s">
+      <c r="B8" s="75"/>
+      <c r="C8" s="64" t="s">
         <v>696</v>
       </c>
-      <c r="D8" s="26"/>
+      <c r="D8" s="64"/>
       <c r="E8" s="17">
         <v>0</v>
       </c>
@@ -3501,11 +3593,11 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="31"/>
-      <c r="C9" s="26" t="s">
+      <c r="B9" s="75"/>
+      <c r="C9" s="64" t="s">
         <v>697</v>
       </c>
-      <c r="D9" s="26"/>
+      <c r="D9" s="64"/>
       <c r="E9" s="17">
         <v>0</v>
       </c>
@@ -3562,103 +3654,103 @@
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="71" t="s">
         <v>698</v>
       </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="37">
+      <c r="D10" s="71"/>
+      <c r="E10" s="79">
         <f>SUM(E3:G3)</f>
         <v>8</v>
       </c>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="39">
+      <c r="F10" s="80"/>
+      <c r="G10" s="80"/>
+      <c r="H10" s="65">
         <f>SUM(H3:J3)</f>
         <v>13</v>
       </c>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="40">
+      <c r="I10" s="65"/>
+      <c r="J10" s="65"/>
+      <c r="K10" s="70">
         <f>SUM(K3:M3)</f>
         <v>14</v>
       </c>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40">
+      <c r="L10" s="70"/>
+      <c r="M10" s="70"/>
+      <c r="N10" s="70">
         <f>SUM(N3:P3)</f>
         <v>7</v>
       </c>
-      <c r="O10" s="40"/>
-      <c r="P10" s="40"/>
-      <c r="Q10" s="41">
+      <c r="O10" s="70"/>
+      <c r="P10" s="70"/>
+      <c r="Q10" s="66">
         <f>SUM(Q7:S7)</f>
         <v>25</v>
       </c>
-      <c r="R10" s="41"/>
-      <c r="S10" s="41"/>
-      <c r="T10" s="42">
+      <c r="R10" s="66"/>
+      <c r="S10" s="66"/>
+      <c r="T10" s="78">
         <f>SUM(T7:V7)</f>
         <v>19</v>
       </c>
-      <c r="U10" s="42"/>
-      <c r="V10" s="42"/>
+      <c r="U10" s="78"/>
+      <c r="V10" s="78"/>
     </row>
     <row r="11" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="76" t="s">
         <v>702</v>
       </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="35">
+      <c r="D11" s="76"/>
+      <c r="E11" s="67">
         <f>SUM(E10:P10)</f>
         <v>42</v>
       </c>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="35"/>
-      <c r="L11" s="35"/>
-      <c r="M11" s="35"/>
-      <c r="N11" s="35"/>
-      <c r="O11" s="35"/>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="36">
+      <c r="F11" s="67"/>
+      <c r="G11" s="67"/>
+      <c r="H11" s="67"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="67"/>
+      <c r="K11" s="67"/>
+      <c r="L11" s="67"/>
+      <c r="M11" s="67"/>
+      <c r="N11" s="67"/>
+      <c r="O11" s="67"/>
+      <c r="P11" s="67"/>
+      <c r="Q11" s="68">
         <f>SUM(Q10:V10)</f>
         <v>44</v>
       </c>
-      <c r="R11" s="36"/>
-      <c r="S11" s="36"/>
-      <c r="T11" s="36"/>
-      <c r="U11" s="36"/>
-      <c r="V11" s="36"/>
+      <c r="R11" s="68"/>
+      <c r="S11" s="68"/>
+      <c r="T11" s="68"/>
+      <c r="U11" s="68"/>
+      <c r="V11" s="68"/>
     </row>
     <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="71" t="s">
         <v>699</v>
       </c>
-      <c r="D12" s="27"/>
-      <c r="E12" s="34">
+      <c r="D12" s="71"/>
+      <c r="E12" s="77">
         <f>SUM(E10:V10)</f>
         <v>86</v>
       </c>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="34"/>
-      <c r="P12" s="34"/>
-      <c r="Q12" s="34"/>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
-      <c r="U12" s="34"/>
-      <c r="V12" s="34"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="77"/>
+      <c r="J12" s="77"/>
+      <c r="K12" s="77"/>
+      <c r="L12" s="77"/>
+      <c r="M12" s="77"/>
+      <c r="N12" s="77"/>
+      <c r="O12" s="77"/>
+      <c r="P12" s="77"/>
+      <c r="Q12" s="77"/>
+      <c r="R12" s="77"/>
+      <c r="S12" s="77"/>
+      <c r="T12" s="77"/>
+      <c r="U12" s="77"/>
+      <c r="V12" s="77"/>
     </row>
     <row r="13" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E13" s="15"/>
@@ -3692,7 +3784,7 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="44" t="s">
+      <c r="A15" s="25" t="s">
         <v>122</v>
       </c>
       <c r="B15" t="s">
@@ -3704,15 +3796,15 @@
       <c r="D15" t="s">
         <v>608</v>
       </c>
-      <c r="E15" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="53" t="s">
+      <c r="E15" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="34" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="44"/>
+      <c r="A16" s="25"/>
       <c r="B16" t="s">
         <v>11</v>
       </c>
@@ -3722,15 +3814,15 @@
       <c r="D16" t="s">
         <v>609</v>
       </c>
-      <c r="E16" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" s="53" t="s">
+      <c r="E16" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="34" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="44"/>
+      <c r="A17" s="25"/>
       <c r="B17" t="s">
         <v>13</v>
       </c>
@@ -3740,15 +3832,15 @@
       <c r="D17" t="s">
         <v>610</v>
       </c>
-      <c r="E17" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="53" t="s">
+      <c r="E17" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="34" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
+      <c r="A18" s="25"/>
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -3758,21 +3850,21 @@
       <c r="D18" t="s">
         <v>611</v>
       </c>
-      <c r="E18" s="50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="53" t="s">
+      <c r="E18" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="34" t="s">
         <v>707</v>
       </c>
-      <c r="K18" s="59" t="s">
+      <c r="K18" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N18" s="68" t="s">
+      <c r="N18" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+      <c r="A19" s="25"/>
       <c r="B19" t="s">
         <v>17</v>
       </c>
@@ -3782,21 +3874,21 @@
       <c r="D19" t="s">
         <v>612</v>
       </c>
-      <c r="F19" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" s="56" t="s">
+      <c r="F19" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="37" t="s">
         <v>707</v>
       </c>
-      <c r="K19" s="59" t="s">
+      <c r="K19" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N19" s="68" t="s">
+      <c r="N19" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="25"/>
       <c r="B20" t="s">
         <v>19</v>
       </c>
@@ -3806,15 +3898,15 @@
       <c r="D20" t="s">
         <v>613</v>
       </c>
-      <c r="F20" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="56" t="s">
+      <c r="F20" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="37" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="44"/>
+      <c r="A21" s="25"/>
       <c r="B21" t="s">
         <v>21</v>
       </c>
@@ -3824,21 +3916,21 @@
       <c r="D21" t="s">
         <v>614</v>
       </c>
-      <c r="F21" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="56" t="s">
+      <c r="F21" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" s="37" t="s">
         <v>707</v>
       </c>
-      <c r="L21" s="62" t="s">
+      <c r="L21" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="O21" s="71" t="s">
+      <c r="O21" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="44"/>
+      <c r="A22" s="25"/>
       <c r="B22" t="s">
         <v>23</v>
       </c>
@@ -3848,15 +3940,15 @@
       <c r="D22" t="s">
         <v>615</v>
       </c>
-      <c r="F22" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="56" t="s">
+      <c r="F22" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="37" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
+      <c r="A23" s="25"/>
       <c r="B23" t="s">
         <v>25</v>
       </c>
@@ -3866,18 +3958,18 @@
       <c r="D23" t="s">
         <v>617</v>
       </c>
-      <c r="H23" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="K23" s="59" t="s">
+      <c r="H23" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K23" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N23" s="68" t="s">
+      <c r="N23" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
+      <c r="A24" s="25"/>
       <c r="B24" t="s">
         <v>27</v>
       </c>
@@ -3887,18 +3979,18 @@
       <c r="D24" t="s">
         <v>618</v>
       </c>
-      <c r="H24" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="K24" s="59" t="s">
+      <c r="H24" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="K24" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N24" s="68" t="s">
+      <c r="N24" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+      <c r="A25" s="25"/>
       <c r="B25" t="s">
         <v>29</v>
       </c>
@@ -3908,27 +4000,27 @@
       <c r="D25" t="s">
         <v>616</v>
       </c>
-      <c r="H25" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="77" t="s">
+      <c r="H25" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="I25" s="58" t="s">
         <v>707</v>
       </c>
-      <c r="K25" s="59" t="s">
+      <c r="K25" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="L25" s="62" t="s">
+      <c r="L25" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="N25" s="68" t="s">
+      <c r="N25" s="49" t="s">
         <v>707</v>
       </c>
-      <c r="O25" s="71" t="s">
+      <c r="O25" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="44"/>
+      <c r="A26" s="25"/>
       <c r="B26" t="s">
         <v>31</v>
       </c>
@@ -3938,21 +4030,21 @@
       <c r="D26" t="s">
         <v>622</v>
       </c>
-      <c r="H26" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="77" t="s">
+      <c r="H26" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="58" t="s">
         <v>707</v>
       </c>
-      <c r="K26" s="59" t="s">
+      <c r="K26" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N26" s="68" t="s">
+      <c r="N26" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="44"/>
+      <c r="A27" s="25"/>
       <c r="B27" t="s">
         <v>35</v>
       </c>
@@ -3962,21 +4054,21 @@
       <c r="D27" t="s">
         <v>625</v>
       </c>
-      <c r="H27" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="77" t="s">
+      <c r="H27" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="58" t="s">
         <v>707</v>
       </c>
-      <c r="K27" s="59" t="s">
+      <c r="K27" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N27" s="68" t="s">
+      <c r="N27" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
+      <c r="A28" s="25"/>
       <c r="B28" t="s">
         <v>37</v>
       </c>
@@ -3986,21 +4078,21 @@
       <c r="D28" t="s">
         <v>621</v>
       </c>
-      <c r="H28" s="74" t="s">
-        <v>10</v>
-      </c>
-      <c r="I28" s="77" t="s">
+      <c r="H28" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" s="58" t="s">
         <v>707</v>
       </c>
-      <c r="K28" s="59" t="s">
+      <c r="K28" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N28" s="68" t="s">
+      <c r="N28" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
+      <c r="A29" s="25"/>
       <c r="B29" t="s">
         <v>40</v>
       </c>
@@ -4010,21 +4102,21 @@
       <c r="D29" t="s">
         <v>665</v>
       </c>
-      <c r="I29" s="77" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" s="80" t="s">
+      <c r="I29" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="J29" s="61" t="s">
         <v>707</v>
       </c>
-      <c r="K29" s="59" t="s">
+      <c r="K29" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N29" s="68" t="s">
+      <c r="N29" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="25"/>
       <c r="B30" t="s">
         <v>42</v>
       </c>
@@ -4034,21 +4126,21 @@
       <c r="D30" t="s">
         <v>637</v>
       </c>
-      <c r="I30" s="77" t="s">
-        <v>10</v>
-      </c>
-      <c r="J30" s="80" t="s">
+      <c r="I30" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="J30" s="61" t="s">
         <v>707</v>
       </c>
-      <c r="L30" s="62" t="s">
+      <c r="L30" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="O30" s="71" t="s">
+      <c r="O30" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="44"/>
+      <c r="A31" s="25"/>
       <c r="B31" t="s">
         <v>44</v>
       </c>
@@ -4058,21 +4150,21 @@
       <c r="D31" t="s">
         <v>628</v>
       </c>
-      <c r="I31" s="77" t="s">
-        <v>10</v>
-      </c>
-      <c r="J31" s="80" t="s">
+      <c r="I31" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="J31" s="61" t="s">
         <v>707</v>
       </c>
-      <c r="K31" s="59" t="s">
+      <c r="K31" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N31" s="68" t="s">
+      <c r="N31" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="44"/>
+      <c r="A32" s="25"/>
       <c r="B32" t="s">
         <v>46</v>
       </c>
@@ -4082,21 +4174,21 @@
       <c r="D32" t="s">
         <v>629</v>
       </c>
-      <c r="I32" s="77" t="s">
-        <v>10</v>
-      </c>
-      <c r="J32" s="80" t="s">
+      <c r="I32" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="J32" s="61" t="s">
         <v>707</v>
       </c>
-      <c r="K32" s="59" t="s">
+      <c r="K32" s="40" t="s">
         <v>707</v>
       </c>
-      <c r="N32" s="68" t="s">
+      <c r="N32" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="44"/>
+      <c r="A33" s="25"/>
       <c r="B33" t="s">
         <v>48</v>
       </c>
@@ -4106,10 +4198,10 @@
       <c r="D33" t="s">
         <v>644</v>
       </c>
-      <c r="J33" s="80" t="s">
-        <v>10</v>
-      </c>
-      <c r="M33" s="65" t="s">
+      <c r="J33" s="61" t="s">
+        <v>10</v>
+      </c>
+      <c r="M33" s="46" t="s">
         <v>707</v>
       </c>
       <c r="S33" s="8" t="s">
@@ -4117,7 +4209,7 @@
       </c>
     </row>
     <row r="34" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="44"/>
+      <c r="A34" s="25"/>
       <c r="B34" t="s">
         <v>50</v>
       </c>
@@ -4127,16 +4219,16 @@
       <c r="D34" t="s">
         <v>639</v>
       </c>
-      <c r="J34" s="80" t="s">
-        <v>10</v>
-      </c>
-      <c r="L34" s="62" t="s">
+      <c r="J34" s="61" t="s">
+        <v>10</v>
+      </c>
+      <c r="L34" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="M34" s="65" t="s">
+      <c r="M34" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="O34" s="71" t="s">
+      <c r="O34" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S34" s="8" t="s">
@@ -4144,7 +4236,7 @@
       </c>
     </row>
     <row r="35" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="44"/>
+      <c r="A35" s="25"/>
       <c r="B35" t="s">
         <v>52</v>
       </c>
@@ -4154,10 +4246,10 @@
       <c r="D35" t="s">
         <v>647</v>
       </c>
-      <c r="J35" s="80" t="s">
-        <v>10</v>
-      </c>
-      <c r="M35" s="65" t="s">
+      <c r="J35" s="61" t="s">
+        <v>10</v>
+      </c>
+      <c r="M35" s="46" t="s">
         <v>707</v>
       </c>
       <c r="S35" s="8" t="s">
@@ -4165,7 +4257,7 @@
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A36" s="44"/>
+      <c r="A36" s="25"/>
       <c r="B36" t="s">
         <v>54</v>
       </c>
@@ -4175,15 +4267,15 @@
       <c r="D36" t="s">
         <v>632</v>
       </c>
-      <c r="K36" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="N36" s="68" t="s">
+      <c r="K36" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="N36" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A37" s="44"/>
+      <c r="A37" s="25"/>
       <c r="B37" t="s">
         <v>56</v>
       </c>
@@ -4193,15 +4285,15 @@
       <c r="D37" t="s">
         <v>633</v>
       </c>
-      <c r="K37" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="N37" s="68" t="s">
+      <c r="K37" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="N37" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="44"/>
+      <c r="A38" s="25"/>
       <c r="B38" t="s">
         <v>33</v>
       </c>
@@ -4211,15 +4303,15 @@
       <c r="D38" t="s">
         <v>623</v>
       </c>
-      <c r="K38" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="N38" s="68" t="s">
+      <c r="K38" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="N38" s="49" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="44"/>
+      <c r="A39" s="25"/>
       <c r="B39" t="s">
         <v>92</v>
       </c>
@@ -4229,21 +4321,21 @@
       <c r="D39" t="s">
         <v>645</v>
       </c>
-      <c r="K39" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="L39" s="62" t="s">
+      <c r="K39" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="L39" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="N39" s="68" t="s">
+      <c r="N39" s="49" t="s">
         <v>707</v>
       </c>
-      <c r="O39" s="71" t="s">
+      <c r="O39" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A40" s="44"/>
+      <c r="A40" s="25"/>
       <c r="B40" t="s">
         <v>58</v>
       </c>
@@ -4253,21 +4345,21 @@
       <c r="D40" t="s">
         <v>626</v>
       </c>
-      <c r="K40" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="L40" s="62" t="s">
+      <c r="K40" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="L40" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="N40" s="68" t="s">
+      <c r="N40" s="49" t="s">
         <v>707</v>
       </c>
-      <c r="O40" s="71" t="s">
+      <c r="O40" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A41" s="44"/>
+      <c r="A41" s="25"/>
       <c r="B41" t="s">
         <v>62</v>
       </c>
@@ -4277,19 +4369,19 @@
       <c r="D41" t="s">
         <v>620</v>
       </c>
-      <c r="K41" s="59" t="s">
-        <v>10</v>
-      </c>
-      <c r="L41" s="62" t="s">
+      <c r="K41" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="L41" s="43" t="s">
         <v>707</v>
       </c>
-      <c r="M41" s="65" t="s">
+      <c r="M41" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="N41" s="68" t="s">
+      <c r="N41" s="49" t="s">
         <v>707</v>
       </c>
-      <c r="O41" s="71" t="s">
+      <c r="O41" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S41" s="8" t="s">
@@ -4297,7 +4389,7 @@
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A42" s="44"/>
+      <c r="A42" s="25"/>
       <c r="B42" t="s">
         <v>89</v>
       </c>
@@ -4307,13 +4399,13 @@
       <c r="D42" t="s">
         <v>634</v>
       </c>
-      <c r="L42" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="M42" s="65" t="s">
+      <c r="L42" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="M42" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="O42" s="71" t="s">
+      <c r="O42" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S42" s="8" t="s">
@@ -4321,7 +4413,7 @@
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A43" s="44"/>
+      <c r="A43" s="25"/>
       <c r="B43" t="s">
         <v>69</v>
       </c>
@@ -4331,13 +4423,13 @@
       <c r="D43" t="s">
         <v>636</v>
       </c>
-      <c r="L43" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="M43" s="65" t="s">
+      <c r="L43" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="M43" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="O43" s="71" t="s">
+      <c r="O43" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S43" s="8" t="s">
@@ -4345,7 +4437,7 @@
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A44" s="44"/>
+      <c r="A44" s="25"/>
       <c r="B44" t="s">
         <v>71</v>
       </c>
@@ -4355,13 +4447,13 @@
       <c r="D44" t="s">
         <v>638</v>
       </c>
-      <c r="L44" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="M44" s="65" t="s">
+      <c r="L44" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="M44" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="O44" s="71" t="s">
+      <c r="O44" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S44" s="8" t="s">
@@ -4369,7 +4461,7 @@
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A45" s="44"/>
+      <c r="A45" s="25"/>
       <c r="B45" t="s">
         <v>78</v>
       </c>
@@ -4379,13 +4471,13 @@
       <c r="D45" t="s">
         <v>643</v>
       </c>
-      <c r="L45" s="62" t="s">
-        <v>10</v>
-      </c>
-      <c r="M45" s="65" t="s">
+      <c r="L45" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="M45" s="46" t="s">
         <v>707</v>
       </c>
-      <c r="O45" s="71" t="s">
+      <c r="O45" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S45" s="8" t="s">
@@ -4393,7 +4485,7 @@
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A46" s="44"/>
+      <c r="A46" s="25"/>
       <c r="B46" t="s">
         <v>80</v>
       </c>
@@ -4403,7 +4495,7 @@
       <c r="D46" t="s">
         <v>646</v>
       </c>
-      <c r="M46" s="65" t="s">
+      <c r="M46" s="46" t="s">
         <v>10</v>
       </c>
       <c r="S46" s="8" t="s">
@@ -4411,7 +4503,7 @@
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A47" s="44"/>
+      <c r="A47" s="25"/>
       <c r="B47" t="s">
         <v>82</v>
       </c>
@@ -4421,7 +4513,7 @@
       <c r="D47" t="s">
         <v>648</v>
       </c>
-      <c r="M47" s="65" t="s">
+      <c r="M47" s="46" t="s">
         <v>10</v>
       </c>
       <c r="S47" s="8" t="s">
@@ -4429,7 +4521,7 @@
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A48" s="44"/>
+      <c r="A48" s="25"/>
       <c r="B48" t="s">
         <v>84</v>
       </c>
@@ -4439,7 +4531,7 @@
       <c r="D48" t="s">
         <v>649</v>
       </c>
-      <c r="M48" s="65" t="s">
+      <c r="M48" s="46" t="s">
         <v>10</v>
       </c>
       <c r="S48" s="8" t="s">
@@ -4447,7 +4539,7 @@
       </c>
     </row>
     <row r="49" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A49" s="44"/>
+      <c r="A49" s="25"/>
       <c r="B49" t="s">
         <v>86</v>
       </c>
@@ -4457,7 +4549,7 @@
       <c r="D49" t="s">
         <v>650</v>
       </c>
-      <c r="M49" s="65" t="s">
+      <c r="M49" s="46" t="s">
         <v>10</v>
       </c>
       <c r="S49" s="8" t="s">
@@ -4465,7 +4557,7 @@
       </c>
     </row>
     <row r="50" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A50" s="44"/>
+      <c r="A50" s="25"/>
       <c r="B50" t="s">
         <v>64</v>
       </c>
@@ -4475,15 +4567,15 @@
       <c r="D50" t="s">
         <v>627</v>
       </c>
-      <c r="N50" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O50" s="71" t="s">
+      <c r="N50" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O50" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="51" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A51" s="44"/>
+      <c r="A51" s="25"/>
       <c r="B51" t="s">
         <v>712</v>
       </c>
@@ -4493,15 +4585,15 @@
       <c r="D51" t="s">
         <v>631</v>
       </c>
-      <c r="N51" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O51" s="71" t="s">
+      <c r="N51" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O51" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A52" s="44"/>
+      <c r="A52" s="25"/>
       <c r="B52" t="s">
         <v>711</v>
       </c>
@@ -4511,15 +4603,15 @@
       <c r="D52" t="s">
         <v>630</v>
       </c>
-      <c r="N52" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O52" s="71" t="s">
+      <c r="N52" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O52" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A53" s="44"/>
+      <c r="A53" s="25"/>
       <c r="B53" t="s">
         <v>73</v>
       </c>
@@ -4529,10 +4621,10 @@
       <c r="D53" t="s">
         <v>640</v>
       </c>
-      <c r="N53" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O53" s="71" t="s">
+      <c r="N53" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O53" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S53" s="8" t="s">
@@ -4540,7 +4632,7 @@
       </c>
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A54" s="44"/>
+      <c r="A54" s="25"/>
       <c r="B54" t="s">
         <v>75</v>
       </c>
@@ -4550,10 +4642,10 @@
       <c r="D54" t="s">
         <v>641</v>
       </c>
-      <c r="N54" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O54" s="71" t="s">
+      <c r="N54" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O54" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S54" s="8" t="s">
@@ -4561,7 +4653,7 @@
       </c>
     </row>
     <row r="55" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A55" s="44"/>
+      <c r="A55" s="25"/>
       <c r="B55" t="s">
         <v>88</v>
       </c>
@@ -4571,10 +4663,10 @@
       <c r="D55" t="s">
         <v>642</v>
       </c>
-      <c r="N55" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O55" s="71" t="s">
+      <c r="N55" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O55" s="52" t="s">
         <v>707</v>
       </c>
       <c r="S55" s="8" t="s">
@@ -4582,7 +4674,7 @@
       </c>
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A56" s="44"/>
+      <c r="A56" s="25"/>
       <c r="B56" t="s">
         <v>60</v>
       </c>
@@ -4592,39 +4684,39 @@
       <c r="D56" t="s">
         <v>624</v>
       </c>
-      <c r="N56" s="68" t="s">
-        <v>10</v>
-      </c>
-      <c r="O56" s="71" t="s">
+      <c r="N56" s="49" t="s">
+        <v>10</v>
+      </c>
+      <c r="O56" s="52" t="s">
         <v>707</v>
       </c>
     </row>
     <row r="57" spans="1:26" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="43"/>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="43"/>
-      <c r="I57" s="43"/>
-      <c r="J57" s="43"/>
-      <c r="K57" s="43"/>
-      <c r="L57" s="43"/>
-      <c r="M57" s="43"/>
-      <c r="Q57" s="43"/>
-      <c r="R57" s="43"/>
-      <c r="S57" s="43"/>
-      <c r="T57" s="43"/>
-      <c r="U57" s="43"/>
-      <c r="V57" s="43"/>
-      <c r="W57" s="43"/>
-      <c r="X57" s="43"/>
-      <c r="Y57" s="43"/>
-      <c r="Z57" s="43"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="2"/>
+      <c r="M57" s="2"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="2"/>
+      <c r="S57" s="2"/>
+      <c r="T57" s="2"/>
+      <c r="U57" s="2"/>
+      <c r="V57" s="2"/>
+      <c r="W57" s="2"/>
+      <c r="X57" s="2"/>
+      <c r="Y57" s="2"/>
+      <c r="Z57" s="2"/>
     </row>
     <row r="58" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="45" t="s">
+      <c r="A58" s="26" t="s">
         <v>706</v>
       </c>
       <c r="B58" t="s">
@@ -4644,7 +4736,7 @@
       </c>
     </row>
     <row r="59" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A59" s="45"/>
+      <c r="A59" s="26"/>
       <c r="B59" t="s">
         <v>94</v>
       </c>
@@ -4662,7 +4754,7 @@
       </c>
     </row>
     <row r="60" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A60" s="45"/>
+      <c r="A60" s="26"/>
       <c r="B60" t="s">
         <v>95</v>
       </c>
@@ -4680,7 +4772,7 @@
       </c>
     </row>
     <row r="61" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A61" s="45"/>
+      <c r="A61" s="26"/>
       <c r="B61" t="s">
         <v>96</v>
       </c>
@@ -4698,7 +4790,7 @@
       </c>
     </row>
     <row r="62" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A62" s="45"/>
+      <c r="A62" s="26"/>
       <c r="B62" t="s">
         <v>97</v>
       </c>
@@ -4716,7 +4808,7 @@
       </c>
     </row>
     <row r="63" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A63" s="45"/>
+      <c r="A63" s="26"/>
       <c r="B63" t="s">
         <v>98</v>
       </c>
@@ -4734,7 +4826,7 @@
       </c>
     </row>
     <row r="64" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A64" s="45"/>
+      <c r="A64" s="26"/>
       <c r="B64" t="s">
         <v>99</v>
       </c>
@@ -4752,7 +4844,7 @@
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A65" s="45"/>
+      <c r="A65" s="26"/>
       <c r="B65" t="s">
         <v>101</v>
       </c>
@@ -4767,7 +4859,7 @@
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A66" s="45"/>
+      <c r="A66" s="26"/>
       <c r="B66" t="s">
         <v>102</v>
       </c>
@@ -4788,7 +4880,7 @@
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A67" s="45"/>
+      <c r="A67" s="26"/>
       <c r="B67" t="s">
         <v>103</v>
       </c>
@@ -4806,7 +4898,7 @@
       </c>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A68" s="45"/>
+      <c r="A68" s="26"/>
       <c r="B68" t="s">
         <v>104</v>
       </c>
@@ -4824,7 +4916,7 @@
       </c>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A69" s="45"/>
+      <c r="A69" s="26"/>
       <c r="B69" t="s">
         <v>105</v>
       </c>
@@ -4842,7 +4934,7 @@
       </c>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A70" s="45"/>
+      <c r="A70" s="26"/>
       <c r="B70" t="s">
         <v>125</v>
       </c>
@@ -4863,7 +4955,7 @@
       </c>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A71" s="45"/>
+      <c r="A71" s="26"/>
       <c r="B71" t="s">
         <v>127</v>
       </c>
@@ -4881,7 +4973,7 @@
       </c>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A72" s="45"/>
+      <c r="A72" s="26"/>
       <c r="B72" t="s">
         <v>129</v>
       </c>
@@ -4896,7 +4988,7 @@
       </c>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A73" s="45"/>
+      <c r="A73" s="26"/>
       <c r="B73" t="s">
         <v>131</v>
       </c>
@@ -4914,7 +5006,7 @@
       </c>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A74" s="45"/>
+      <c r="A74" s="26"/>
       <c r="B74" t="s">
         <v>133</v>
       </c>
@@ -4932,7 +5024,7 @@
       </c>
     </row>
     <row r="75" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A75" s="45"/>
+      <c r="A75" s="26"/>
       <c r="B75" t="s">
         <v>135</v>
       </c>
@@ -4950,7 +5042,7 @@
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A76" s="45"/>
+      <c r="A76" s="26"/>
       <c r="B76" t="s">
         <v>137</v>
       </c>
@@ -4968,7 +5060,7 @@
       </c>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A77" s="45"/>
+      <c r="A77" s="26"/>
       <c r="B77" t="s">
         <v>139</v>
       </c>
@@ -4983,7 +5075,7 @@
       </c>
     </row>
     <row r="78" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A78" s="45"/>
+      <c r="A78" s="26"/>
       <c r="B78" t="s">
         <v>141</v>
       </c>
@@ -4998,7 +5090,7 @@
       </c>
     </row>
     <row r="79" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A79" s="45"/>
+      <c r="A79" s="26"/>
       <c r="B79" t="s">
         <v>143</v>
       </c>
@@ -5013,7 +5105,7 @@
       </c>
     </row>
     <row r="80" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A80" s="45"/>
+      <c r="A80" s="26"/>
       <c r="B80" t="s">
         <v>145</v>
       </c>
@@ -5028,7 +5120,7 @@
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A81" s="45"/>
+      <c r="A81" s="26"/>
       <c r="B81" t="s">
         <v>146</v>
       </c>
@@ -5043,7 +5135,7 @@
       </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A82" s="45"/>
+      <c r="A82" s="26"/>
       <c r="B82" t="s">
         <v>150</v>
       </c>
@@ -5058,7 +5150,7 @@
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A83" s="45"/>
+      <c r="A83" s="26"/>
       <c r="B83" t="s">
         <v>123</v>
       </c>
@@ -5073,7 +5165,7 @@
       </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A84" s="45"/>
+      <c r="A84" s="26"/>
       <c r="B84" t="s">
         <v>156</v>
       </c>
@@ -5088,7 +5180,7 @@
       </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A85" s="45"/>
+      <c r="A85" s="26"/>
       <c r="B85" t="s">
         <v>157</v>
       </c>
@@ -5103,7 +5195,7 @@
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A86" s="45"/>
+      <c r="A86" s="26"/>
       <c r="B86" t="s">
         <v>160</v>
       </c>
@@ -5118,7 +5210,7 @@
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A87" s="45"/>
+      <c r="A87" s="26"/>
       <c r="B87" t="s">
         <v>162</v>
       </c>
@@ -5133,7 +5225,7 @@
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A88" s="45"/>
+      <c r="A88" s="26"/>
       <c r="B88" t="s">
         <v>164</v>
       </c>
@@ -5151,7 +5243,7 @@
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A89" s="45"/>
+      <c r="A89" s="26"/>
       <c r="B89" t="s">
         <v>165</v>
       </c>
@@ -5169,7 +5261,7 @@
       </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A90" s="45"/>
+      <c r="A90" s="26"/>
       <c r="B90" t="s">
         <v>100</v>
       </c>
@@ -5187,7 +5279,7 @@
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A91" s="45"/>
+      <c r="A91" s="26"/>
       <c r="B91" t="s">
         <v>154</v>
       </c>
@@ -5208,7 +5300,7 @@
       </c>
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A92" s="45"/>
+      <c r="A92" s="26"/>
       <c r="B92" t="s">
         <v>168</v>
       </c>
@@ -5226,7 +5318,7 @@
       </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A93" s="45"/>
+      <c r="A93" s="26"/>
       <c r="B93" t="s">
         <v>170</v>
       </c>
@@ -5244,7 +5336,7 @@
       </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A94" s="45"/>
+      <c r="A94" s="26"/>
       <c r="B94" t="s">
         <v>172</v>
       </c>
@@ -5262,7 +5354,7 @@
       </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A95" s="45"/>
+      <c r="A95" s="26"/>
       <c r="B95" t="s">
         <v>173</v>
       </c>
@@ -5280,7 +5372,7 @@
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A96" s="45"/>
+      <c r="A96" s="26"/>
       <c r="B96" t="s">
         <v>174</v>
       </c>
@@ -5298,7 +5390,7 @@
       </c>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A97" s="45"/>
+      <c r="A97" s="26"/>
       <c r="B97" t="s">
         <v>175</v>
       </c>
@@ -5316,7 +5408,7 @@
       </c>
     </row>
     <row r="98" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A98" s="45"/>
+      <c r="A98" s="26"/>
       <c r="B98" t="s">
         <v>180</v>
       </c>
@@ -5334,7 +5426,7 @@
       </c>
     </row>
     <row r="99" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A99" s="45"/>
+      <c r="A99" s="26"/>
       <c r="B99" t="s">
         <v>182</v>
       </c>
@@ -5349,7 +5441,7 @@
       </c>
     </row>
     <row r="100" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A100" s="45"/>
+      <c r="A100" s="26"/>
       <c r="B100" t="s">
         <v>184</v>
       </c>
@@ -5364,7 +5456,7 @@
       </c>
     </row>
     <row r="101" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A101" s="45"/>
+      <c r="A101" s="26"/>
       <c r="B101" t="s">
         <v>186</v>
       </c>
@@ -5378,23 +5470,167 @@
         <v>10</v>
       </c>
     </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A102" s="62"/>
+      <c r="B102" t="s">
+        <v>713</v>
+      </c>
+      <c r="C102" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="103" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A103" s="62"/>
+      <c r="B103" t="s">
+        <v>714</v>
+      </c>
+      <c r="C103" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A104" s="62"/>
+      <c r="B104" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A105" s="62"/>
+      <c r="B105" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A106" s="62"/>
+      <c r="B106" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A107" s="62"/>
+      <c r="B107" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A108" s="62"/>
+      <c r="B108" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A109" s="62"/>
+      <c r="B109" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A110" s="62"/>
+      <c r="B110" t="s">
+        <v>720</v>
+      </c>
+      <c r="C110" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A111" s="62"/>
+      <c r="B111" t="s">
+        <v>721</v>
+      </c>
+      <c r="C111" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A112" s="62"/>
+      <c r="B112" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="62"/>
+      <c r="B113" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="62"/>
+      <c r="B114" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" s="62"/>
+      <c r="B115" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" s="62"/>
+      <c r="B116" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" s="62"/>
+      <c r="B117" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" s="62"/>
+      <c r="B118" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" s="62"/>
+      <c r="B119" t="s">
+        <v>730</v>
+      </c>
+      <c r="C119" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" s="62"/>
+      <c r="B120" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" s="62"/>
+      <c r="B121" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" s="62"/>
+      <c r="B122" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" s="62"/>
+      <c r="B123" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" s="62"/>
+      <c r="B124" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" s="62"/>
+      <c r="B125" t="s">
+        <v>736</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E12:V12"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="E11:P11"/>
-    <mergeCell ref="Q11:V11"/>
     <mergeCell ref="W1:Y1"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
@@ -5407,6 +5643,21 @@
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="N1:P1"/>
+    <mergeCell ref="E12:V12"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="E11:P11"/>
+    <mergeCell ref="Q11:V11"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished Gym leader warmup and challenge decks
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2678B9D-CF21-474D-8E0A-BBDFCF641016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58549CF0-E6BF-4574-BA97-AF9002341593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14565" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="779">
   <si>
     <t>Opponent</t>
   </si>
@@ -2262,6 +2262,117 @@
   </si>
   <si>
     <t>Cold Water Warmup</t>
+  </si>
+  <si>
+    <t>Static Charge</t>
+  </si>
+  <si>
+    <t>Power Surge</t>
+  </si>
+  <si>
+    <t>Life Draining Pollen</t>
+  </si>
+  <si>
+    <t>Sunbathing</t>
+  </si>
+  <si>
+    <t>Ninja Ambush</t>
+  </si>
+  <si>
+    <t>Koga's Ninja Poison</t>
+  </si>
+  <si>
+    <t>Psychic Uplink</t>
+  </si>
+  <si>
+    <t>Mixed Aura</t>
+  </si>
+  <si>
+    <t>Incinerator</t>
+  </si>
+  <si>
+    <t>Stoke The Flames</t>
+  </si>
+  <si>
+    <t>Burning Slot Machine</t>
+  </si>
+  <si>
+    <t>The Might Of The Boss</t>
+  </si>
+  <si>
+    <t>Kings And Queens</t>
+  </si>
+  <si>
+    <t>Zz Mewtwo Purple</t>
+  </si>
+  <si>
+    <t>Zz Charizard Red</t>
+  </si>
+  <si>
+    <t>ZZ Gengar Silver</t>
+  </si>
+  <si>
+    <t>Zz Espeon Umbreon Silver</t>
+  </si>
+  <si>
+    <t>Zz Venusaur Green</t>
+  </si>
+  <si>
+    <t>Zz Pikachu Gold</t>
+  </si>
+  <si>
+    <t>Zz Blastoise Blue</t>
+  </si>
+  <si>
+    <t>Zz Eevee Brown</t>
+  </si>
+  <si>
+    <t>Energy Fighting Brown</t>
+  </si>
+  <si>
+    <t>Energy Water Blue</t>
+  </si>
+  <si>
+    <t>Energy Lightning Gold</t>
+  </si>
+  <si>
+    <t>Energy Grass Green</t>
+  </si>
+  <si>
+    <t>Energy Psychic Purple</t>
+  </si>
+  <si>
+    <t>Energy Fire Red</t>
+  </si>
+  <si>
+    <t>Energy Colorless Silver</t>
+  </si>
+  <si>
+    <t>Energy Darkness Black</t>
+  </si>
+  <si>
+    <t>Energy Fighting Brown 2</t>
+  </si>
+  <si>
+    <t>Energy Water Blue 2</t>
+  </si>
+  <si>
+    <t>Energy Lightning Gold 2</t>
+  </si>
+  <si>
+    <t>Energy Grass Green 2</t>
+  </si>
+  <si>
+    <t>Energy Colorless Silver 2</t>
+  </si>
+  <si>
+    <t>Energy Psychic Purple 2</t>
+  </si>
+  <si>
+    <t>Energy Fire Red 2</t>
+  </si>
+  <si>
+    <t>Energy Darkness Black 2</t>
   </si>
 </sst>
 </file>
@@ -2692,29 +2803,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2745,6 +2838,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3141,41 +3252,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E1" s="69" t="s">
+      <c r="E1" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69" t="s">
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69" t="s">
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69" t="s">
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69" t="s">
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63" t="s">
         <v>694</v>
       </c>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69" t="s">
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63" t="s">
         <v>694</v>
       </c>
-      <c r="U1" s="69"/>
-      <c r="V1" s="69"/>
-      <c r="W1" s="69" t="s">
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63" t="s">
         <v>694</v>
       </c>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="69"/>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
     </row>
     <row r="2" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E2" s="29" t="s">
@@ -3243,13 +3354,13 @@
       </c>
     </row>
     <row r="3" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="66" t="s">
         <v>700</v>
       </c>
-      <c r="C3" s="63" t="s">
+      <c r="C3" s="80" t="s">
         <v>695</v>
       </c>
-      <c r="D3" s="63"/>
+      <c r="D3" s="80"/>
       <c r="E3" s="30">
         <v>4</v>
       </c>
@@ -3315,11 +3426,11 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="73"/>
-      <c r="C4" s="63" t="s">
+      <c r="B4" s="67"/>
+      <c r="C4" s="80" t="s">
         <v>696</v>
       </c>
-      <c r="D4" s="63"/>
+      <c r="D4" s="80"/>
       <c r="E4" s="30">
         <v>4</v>
       </c>
@@ -3385,11 +3496,11 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="73"/>
-      <c r="C5" s="63" t="s">
+      <c r="B5" s="67"/>
+      <c r="C5" s="80" t="s">
         <v>697</v>
       </c>
-      <c r="D5" s="63"/>
+      <c r="D5" s="80"/>
       <c r="E5" s="30">
         <v>4</v>
       </c>
@@ -3469,7 +3580,7 @@
       <c r="V6" s="15"/>
     </row>
     <row r="7" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="74" t="s">
+      <c r="B7" s="68" t="s">
         <v>701</v>
       </c>
       <c r="C7" s="64" t="s">
@@ -3532,7 +3643,7 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="75"/>
+      <c r="B8" s="69"/>
       <c r="C8" s="64" t="s">
         <v>696</v>
       </c>
@@ -3593,7 +3704,7 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="75"/>
+      <c r="B9" s="69"/>
       <c r="C9" s="64" t="s">
         <v>697</v>
       </c>
@@ -3654,103 +3765,103 @@
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="C10" s="71" t="s">
+      <c r="C10" s="65" t="s">
         <v>698</v>
       </c>
-      <c r="D10" s="71"/>
-      <c r="E10" s="79">
+      <c r="D10" s="65"/>
+      <c r="E10" s="73">
         <f>SUM(E3:G3)</f>
         <v>8</v>
       </c>
-      <c r="F10" s="80"/>
-      <c r="G10" s="80"/>
-      <c r="H10" s="65">
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="76">
         <f>SUM(H3:J3)</f>
         <v>13</v>
       </c>
-      <c r="I10" s="65"/>
-      <c r="J10" s="65"/>
-      <c r="K10" s="70">
+      <c r="I10" s="76"/>
+      <c r="J10" s="76"/>
+      <c r="K10" s="75">
         <f>SUM(K3:M3)</f>
         <v>14</v>
       </c>
-      <c r="L10" s="70"/>
-      <c r="M10" s="70"/>
-      <c r="N10" s="70">
+      <c r="L10" s="75"/>
+      <c r="M10" s="75"/>
+      <c r="N10" s="75">
         <f>SUM(N3:P3)</f>
         <v>7</v>
       </c>
-      <c r="O10" s="70"/>
-      <c r="P10" s="70"/>
-      <c r="Q10" s="66">
+      <c r="O10" s="75"/>
+      <c r="P10" s="75"/>
+      <c r="Q10" s="77">
         <f>SUM(Q7:S7)</f>
         <v>25</v>
       </c>
-      <c r="R10" s="66"/>
-      <c r="S10" s="66"/>
-      <c r="T10" s="78">
+      <c r="R10" s="77"/>
+      <c r="S10" s="77"/>
+      <c r="T10" s="72">
         <f>SUM(T7:V7)</f>
         <v>19</v>
       </c>
-      <c r="U10" s="78"/>
-      <c r="V10" s="78"/>
+      <c r="U10" s="72"/>
+      <c r="V10" s="72"/>
     </row>
     <row r="11" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="76" t="s">
+      <c r="C11" s="70" t="s">
         <v>702</v>
       </c>
-      <c r="D11" s="76"/>
-      <c r="E11" s="67">
+      <c r="D11" s="70"/>
+      <c r="E11" s="78">
         <f>SUM(E10:P10)</f>
         <v>42</v>
       </c>
-      <c r="F11" s="67"/>
-      <c r="G11" s="67"/>
-      <c r="H11" s="67"/>
-      <c r="I11" s="67"/>
-      <c r="J11" s="67"/>
-      <c r="K11" s="67"/>
-      <c r="L11" s="67"/>
-      <c r="M11" s="67"/>
-      <c r="N11" s="67"/>
-      <c r="O11" s="67"/>
-      <c r="P11" s="67"/>
-      <c r="Q11" s="68">
+      <c r="F11" s="78"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="78"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="78"/>
+      <c r="M11" s="78"/>
+      <c r="N11" s="78"/>
+      <c r="O11" s="78"/>
+      <c r="P11" s="78"/>
+      <c r="Q11" s="79">
         <f>SUM(Q10:V10)</f>
         <v>44</v>
       </c>
-      <c r="R11" s="68"/>
-      <c r="S11" s="68"/>
-      <c r="T11" s="68"/>
-      <c r="U11" s="68"/>
-      <c r="V11" s="68"/>
+      <c r="R11" s="79"/>
+      <c r="S11" s="79"/>
+      <c r="T11" s="79"/>
+      <c r="U11" s="79"/>
+      <c r="V11" s="79"/>
     </row>
     <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="71" t="s">
+      <c r="C12" s="65" t="s">
         <v>699</v>
       </c>
-      <c r="D12" s="71"/>
-      <c r="E12" s="77">
+      <c r="D12" s="65"/>
+      <c r="E12" s="71">
         <f>SUM(E10:V10)</f>
         <v>86</v>
       </c>
-      <c r="F12" s="77"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="77"/>
-      <c r="J12" s="77"/>
-      <c r="K12" s="77"/>
-      <c r="L12" s="77"/>
-      <c r="M12" s="77"/>
-      <c r="N12" s="77"/>
-      <c r="O12" s="77"/>
-      <c r="P12" s="77"/>
-      <c r="Q12" s="77"/>
-      <c r="R12" s="77"/>
-      <c r="S12" s="77"/>
-      <c r="T12" s="77"/>
-      <c r="U12" s="77"/>
-      <c r="V12" s="77"/>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
+      <c r="I12" s="71"/>
+      <c r="J12" s="71"/>
+      <c r="K12" s="71"/>
+      <c r="L12" s="71"/>
+      <c r="M12" s="71"/>
+      <c r="N12" s="71"/>
+      <c r="O12" s="71"/>
+      <c r="P12" s="71"/>
+      <c r="Q12" s="71"/>
+      <c r="R12" s="71"/>
+      <c r="S12" s="71"/>
+      <c r="T12" s="71"/>
+      <c r="U12" s="71"/>
+      <c r="V12" s="71"/>
     </row>
     <row r="13" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E13" s="15"/>
@@ -5478,6 +5589,9 @@
       <c r="C102" t="s">
         <v>737</v>
       </c>
+      <c r="D102" t="s">
+        <v>763</v>
+      </c>
     </row>
     <row r="103" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A103" s="62"/>
@@ -5487,42 +5601,81 @@
       <c r="C103" t="s">
         <v>741</v>
       </c>
+      <c r="D103" t="s">
+        <v>764</v>
+      </c>
     </row>
     <row r="104" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A104" s="62"/>
       <c r="B104" t="s">
         <v>723</v>
       </c>
+      <c r="C104" t="s">
+        <v>742</v>
+      </c>
+      <c r="D104" t="s">
+        <v>765</v>
+      </c>
     </row>
     <row r="105" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A105" s="62"/>
       <c r="B105" t="s">
         <v>715</v>
       </c>
+      <c r="C105" t="s">
+        <v>745</v>
+      </c>
+      <c r="D105" t="s">
+        <v>766</v>
+      </c>
     </row>
     <row r="106" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A106" s="62"/>
       <c r="B106" t="s">
         <v>716</v>
       </c>
+      <c r="C106" t="s">
+        <v>746</v>
+      </c>
+      <c r="D106" t="s">
+        <v>769</v>
+      </c>
     </row>
     <row r="107" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A107" s="62"/>
       <c r="B107" t="s">
         <v>717</v>
       </c>
+      <c r="C107" t="s">
+        <v>748</v>
+      </c>
+      <c r="D107" t="s">
+        <v>767</v>
+      </c>
     </row>
     <row r="108" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A108" s="62"/>
       <c r="B108" t="s">
         <v>718</v>
       </c>
+      <c r="C108" t="s">
+        <v>752</v>
+      </c>
+      <c r="D108" t="s">
+        <v>768</v>
+      </c>
     </row>
     <row r="109" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A109" s="62"/>
       <c r="B109" t="s">
         <v>719</v>
       </c>
+      <c r="C109" t="s">
+        <v>754</v>
+      </c>
+      <c r="D109" t="s">
+        <v>770</v>
+      </c>
     </row>
     <row r="110" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A110" s="62"/>
@@ -5532,6 +5685,9 @@
       <c r="C110" t="s">
         <v>738</v>
       </c>
+      <c r="D110" t="s">
+        <v>771</v>
+      </c>
     </row>
     <row r="111" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A111" s="62"/>
@@ -5541,50 +5697,92 @@
       <c r="C111" t="s">
         <v>739</v>
       </c>
+      <c r="D111" t="s">
+        <v>772</v>
+      </c>
     </row>
     <row r="112" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A112" s="62"/>
       <c r="B112" t="s">
         <v>722</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C112" t="s">
+        <v>743</v>
+      </c>
+      <c r="D112" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="62"/>
       <c r="B113" t="s">
         <v>724</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C113" t="s">
+        <v>744</v>
+      </c>
+      <c r="D113" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="62"/>
       <c r="B114" t="s">
         <v>725</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C114" t="s">
+        <v>747</v>
+      </c>
+      <c r="D114" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="62"/>
       <c r="B115" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
+        <v>749</v>
+      </c>
+      <c r="D115" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="62"/>
       <c r="B116" t="s">
         <v>727</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C116" t="s">
+        <v>751</v>
+      </c>
+      <c r="D116" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="62"/>
       <c r="B117" t="s">
         <v>728</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
+        <v>753</v>
+      </c>
+      <c r="D117" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="62"/>
       <c r="B118" t="s">
         <v>729</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D118" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="62"/>
       <c r="B119" t="s">
         <v>730</v>
@@ -5592,45 +5790,80 @@
       <c r="C119" t="s">
         <v>740</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D119" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="62"/>
       <c r="B120" t="s">
         <v>731</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D120" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="62"/>
       <c r="B121" t="s">
         <v>732</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D121" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="62"/>
       <c r="B122" t="s">
         <v>733</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D122" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="62"/>
       <c r="B123" t="s">
         <v>734</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D123" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="62"/>
       <c r="B124" t="s">
         <v>735</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C124" t="s">
+        <v>750</v>
+      </c>
+      <c r="D124" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="62"/>
       <c r="B125" t="s">
         <v>736</v>
       </c>
+      <c r="D125" t="s">
+        <v>755</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="E11:P11"/>
+    <mergeCell ref="Q11:V11"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="K10:M10"/>
     <mergeCell ref="W1:Y1"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
@@ -5647,17 +5880,6 @@
     <mergeCell ref="T10:V10"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="N10:P10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="E11:P11"/>
-    <mergeCell ref="Q11:V11"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6596,7 +6818,7 @@
       </c>
       <c r="B103" t="str">
         <f>_xlfn.XLOOKUP(A103, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Koga</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -6605,7 +6827,7 @@
       </c>
       <c r="B104" t="str">
         <f>_xlfn.XLOOKUP(A104, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Giovanni</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -6614,7 +6836,7 @@
       </c>
       <c r="B105" t="str">
         <f>_xlfn.XLOOKUP(A105, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Giovanni</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -6650,7 +6872,7 @@
       </c>
       <c r="B109" t="str">
         <f>_xlfn.XLOOKUP(A109, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Brock</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -6659,7 +6881,7 @@
       </c>
       <c r="B110" t="str">
         <f>_xlfn.XLOOKUP(A110, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Brock</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -6668,7 +6890,7 @@
       </c>
       <c r="B111" t="str">
         <f>_xlfn.XLOOKUP(A111, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Blaine</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -6677,7 +6899,7 @@
       </c>
       <c r="B112" t="str">
         <f>_xlfn.XLOOKUP(A112, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Blaine</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -6686,7 +6908,7 @@
       </c>
       <c r="B113" t="str">
         <f>_xlfn.XLOOKUP(A113, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Erika</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -6695,7 +6917,7 @@
       </c>
       <c r="B114" t="str">
         <f>_xlfn.XLOOKUP(A114, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Erika</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -6704,7 +6926,7 @@
       </c>
       <c r="B115" t="str">
         <f>_xlfn.XLOOKUP(A115, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Lt. Surge</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -6713,7 +6935,7 @@
       </c>
       <c r="B116" t="str">
         <f>_xlfn.XLOOKUP(A116, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Lt. Surge</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -6731,7 +6953,7 @@
       </c>
       <c r="B118" t="str">
         <f>_xlfn.XLOOKUP(A118, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Sabrina</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -6740,7 +6962,7 @@
       </c>
       <c r="B119" t="str">
         <f>_xlfn.XLOOKUP(A119, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Sabrina</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -6749,7 +6971,7 @@
       </c>
       <c r="B120" t="str">
         <f>_xlfn.XLOOKUP(A120, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Ex Gym Leader Misty</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -6758,7 +6980,7 @@
       </c>
       <c r="B121" t="str">
         <f>_xlfn.XLOOKUP(A121, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Gym Hero Misty</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -8999,7 +9221,7 @@
       </c>
       <c r="B370" t="str">
         <f>_xlfn.XLOOKUP(A370, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Misty</v>
       </c>
     </row>
     <row r="371" spans="1:2" x14ac:dyDescent="0.25">
@@ -9017,7 +9239,7 @@
       </c>
       <c r="B372" t="str">
         <f>_xlfn.XLOOKUP(A372, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Blaine</v>
       </c>
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.25">
@@ -9053,7 +9275,7 @@
       </c>
       <c r="B376" t="str">
         <f>_xlfn.XLOOKUP(A376, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Brock</v>
       </c>
     </row>
     <row r="377" spans="1:2" x14ac:dyDescent="0.25">
@@ -9062,7 +9284,7 @@
       </c>
       <c r="B377" t="str">
         <f>_xlfn.XLOOKUP(A377, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Koga</v>
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.25">
@@ -9089,7 +9311,7 @@
       </c>
       <c r="B380" t="str">
         <f>_xlfn.XLOOKUP(A380, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Sabrina</v>
       </c>
     </row>
     <row r="381" spans="1:2" x14ac:dyDescent="0.25">
@@ -9161,7 +9383,7 @@
       </c>
       <c r="B388" t="str">
         <f>_xlfn.XLOOKUP(A388, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Giovanni</v>
       </c>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.25">
@@ -9215,7 +9437,7 @@
       </c>
       <c r="B394" t="str">
         <f>_xlfn.XLOOKUP(A394, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Lt. Surge</v>
       </c>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.25">
@@ -9305,7 +9527,7 @@
       </c>
       <c r="B404" t="str">
         <f>_xlfn.XLOOKUP(A404, opponents_table!D:D, opponents_table!B:B, "", 0)</f>
-        <v/>
+        <v>Erika</v>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added best of 3 matches for card elders and ready for gym leaders
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AA6C61-EFB8-4005-BF24-B4C2CFEEBC0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2EAB90-046D-4614-BEBD-0E75D3668764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="777">
   <si>
     <t>Opponent</t>
   </si>
@@ -2110,9 +2110,6 @@
   </si>
   <si>
     <t>Hypno Gold</t>
-  </si>
-  <si>
-    <t>CH / VERDANT FOREST</t>
   </si>
   <si>
     <t>New opponents added</t>
@@ -2367,9 +2364,6 @@
   </si>
   <si>
     <t xml:space="preserve">Night 3 </t>
-  </si>
-  <si>
-    <t>CELESTE / VERDANT</t>
   </si>
   <si>
     <t>GYM PLAZA / HALL</t>
@@ -2379,7 +2373,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2405,6 +2399,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2604,7 +2606,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2621,11 +2623,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2637,100 +2650,13 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2826,9 +2752,6 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2868,6 +2791,117 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2896,6 +2930,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFF9D1FB"/>
       <color rgb="FFF8BFF9"/>
       <color rgb="FFFEE7B8"/>
       <color rgb="FFC9E5FF"/>
@@ -2905,7 +2940,6 @@
       <color rgb="FF9FE1FF"/>
       <color rgb="FFB9E9FF"/>
       <color rgb="FFF7C2FA"/>
-      <color rgb="FFF9D1FB"/>
     </mruColors>
   </colors>
   <extLst>
@@ -3262,150 +3296,162 @@
     <col min="5" max="10" width="7.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="E1" s="68" t="s">
+    <row r="1" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E1" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68" t="s">
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68" t="s">
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68" t="s">
-        <v>777</v>
-      </c>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68" t="s">
-        <v>777</v>
-      </c>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68" t="s">
-        <v>703</v>
-      </c>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68" t="s">
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70" t="s">
+        <v>121</v>
+      </c>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70" t="s">
+        <v>702</v>
+      </c>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70" t="s">
+        <v>702</v>
+      </c>
+      <c r="U1" s="70"/>
+      <c r="V1" s="70"/>
+      <c r="W1" s="70" t="s">
+        <v>702</v>
+      </c>
+      <c r="X1" s="70"/>
+      <c r="Y1" s="70"/>
+    </row>
+    <row r="2" spans="1:25" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E2" s="71" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="72" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="73" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="74" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="77" t="s">
+        <v>89</v>
+      </c>
+      <c r="L2" s="78" t="s">
+        <v>90</v>
+      </c>
+      <c r="M2" s="79" t="s">
+        <v>775</v>
+      </c>
+      <c r="N2" s="80" t="s">
+        <v>118</v>
+      </c>
+      <c r="O2" s="81" t="s">
+        <v>119</v>
+      </c>
+      <c r="P2" s="82" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q2" s="83" t="s">
+        <v>150</v>
+      </c>
+      <c r="R2" s="84" t="s">
+        <v>151</v>
+      </c>
+      <c r="S2" s="85" t="s">
+        <v>152</v>
+      </c>
+      <c r="T2" s="86" t="s">
+        <v>699</v>
+      </c>
+      <c r="U2" s="87" t="s">
+        <v>700</v>
+      </c>
+      <c r="V2" s="88" t="s">
+        <v>701</v>
+      </c>
+      <c r="W2" s="86" t="s">
+        <v>704</v>
+      </c>
+      <c r="X2" s="87" t="s">
+        <v>705</v>
+      </c>
+      <c r="Y2" s="88" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="41" t="s">
+        <v>696</v>
+      </c>
+      <c r="C3" s="33" t="s">
         <v>692</v>
       </c>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-    </row>
-    <row r="2" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E2" s="15" t="s">
+      <c r="D3" s="33"/>
+      <c r="E3" s="52">
+        <f>COUNTIF(E11:E400,"✅")</f>
+        <v>4</v>
+      </c>
+      <c r="F3" s="53">
+        <f t="shared" ref="F3:P3" si="0">COUNTIF(F11:F400,"✅")</f>
+        <v>4</v>
+      </c>
+      <c r="G3" s="54">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H3" s="55">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I3" s="56">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="J3" s="57">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K3" s="58">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="L3" s="59">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="M3" s="60">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N3" s="61">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="O3" s="62">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F2" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="33" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="M2" s="25" t="s">
-        <v>776</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="O2" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="P2" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>700</v>
-      </c>
-      <c r="U2" s="9" t="s">
-        <v>701</v>
-      </c>
-      <c r="V2" s="10" t="s">
-        <v>702</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>705</v>
-      </c>
-      <c r="X2" s="9" t="s">
-        <v>706</v>
-      </c>
-      <c r="Y2" s="10" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="71" t="s">
-        <v>697</v>
-      </c>
-      <c r="C3" s="62" t="s">
-        <v>693</v>
-      </c>
-      <c r="D3" s="62"/>
-      <c r="E3" s="16">
-        <v>4</v>
-      </c>
-      <c r="F3" s="18">
-        <v>4</v>
-      </c>
-      <c r="G3" s="20">
-        <v>0</v>
-      </c>
-      <c r="H3" s="32">
-        <v>6</v>
-      </c>
-      <c r="I3" s="34">
-        <v>4</v>
-      </c>
-      <c r="J3" s="36">
-        <v>3</v>
-      </c>
-      <c r="K3" s="22">
-        <v>5</v>
-      </c>
-      <c r="L3" s="24">
-        <v>5</v>
-      </c>
-      <c r="M3" s="26">
-        <v>3</v>
-      </c>
-      <c r="N3" s="28">
-        <v>8</v>
-      </c>
-      <c r="O3" s="30">
-        <v>0</v>
-      </c>
-      <c r="P3" s="14">
+      <c r="P3" s="63">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q3" s="4">
@@ -3437,106 +3483,127 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="72"/>
-      <c r="C4" s="62" t="s">
-        <v>694</v>
-      </c>
-      <c r="D4" s="62"/>
-      <c r="E4" s="16">
+      <c r="B4" s="42"/>
+      <c r="C4" s="33" t="s">
+        <v>693</v>
+      </c>
+      <c r="D4" s="33"/>
+      <c r="E4" s="52">
+        <f>COUNTIF(E11:E400,"✅")+COUNTIF(E11:E400,"✔️")</f>
         <v>4</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="53">
+        <f t="shared" ref="F4:P4" si="1">COUNTIF(F11:F400,"✅")+COUNTIF(F11:F400,"✔️")</f>
         <v>8</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="54">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="H4" s="32">
+      <c r="H4" s="55">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="I4" s="34">
+      <c r="I4" s="56">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="57">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="58">
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="L4" s="24">
+      <c r="L4" s="59">
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="M4" s="26">
+      <c r="M4" s="60">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N4" s="28">
+      <c r="N4" s="61">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="O4" s="62">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="P4" s="63">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="Q4" s="64">
+        <f t="shared" ref="Q4:Y4" si="2">COUNTIF(Q11:Q400,"✅")+COUNTIF(Q11:Q400,"✔️")</f>
+        <v>27</v>
+      </c>
+      <c r="R4" s="65">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="S4" s="66">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="T4" s="67">
+        <f t="shared" si="2"/>
+        <v>19</v>
+      </c>
+      <c r="U4" s="68">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="V4" s="69">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="W4" s="67">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="O4" s="30">
+      <c r="X4" s="68">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="P4" s="14">
+      <c r="Y4" s="69">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Q4" s="37">
-        <v>21</v>
-      </c>
-      <c r="R4" s="38">
-        <v>18</v>
-      </c>
-      <c r="S4" s="39">
-        <v>10</v>
-      </c>
-      <c r="T4" s="40">
-        <v>19</v>
-      </c>
-      <c r="U4" s="41">
-        <v>10</v>
-      </c>
-      <c r="V4" s="42">
-        <v>11</v>
-      </c>
-      <c r="W4" s="4">
-        <v>0</v>
-      </c>
-      <c r="X4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="4">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" spans="1:25" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="11"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="43"/>
-      <c r="Q5" s="43"/>
-      <c r="R5" s="43"/>
-      <c r="S5" s="43"/>
-      <c r="T5" s="43"/>
-      <c r="U5" s="43"/>
-      <c r="V5" s="43"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
     </row>
     <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="73" t="s">
-        <v>698</v>
-      </c>
-      <c r="C6" s="63" t="s">
-        <v>693</v>
-      </c>
-      <c r="D6" s="63"/>
+      <c r="B6" s="43" t="s">
+        <v>697</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>692</v>
+      </c>
+      <c r="D6" s="34"/>
       <c r="E6" s="4">
         <v>0</v>
       </c>
@@ -3573,22 +3640,22 @@
       <c r="P6" s="4">
         <v>0</v>
       </c>
-      <c r="Q6" s="37">
+      <c r="Q6" s="8">
         <v>12</v>
       </c>
-      <c r="R6" s="38">
+      <c r="R6" s="9">
         <v>7</v>
       </c>
-      <c r="S6" s="39">
+      <c r="S6" s="10">
         <v>6</v>
       </c>
-      <c r="T6" s="40">
-        <v>9</v>
-      </c>
-      <c r="U6" s="41">
+      <c r="T6" s="11">
+        <v>9</v>
+      </c>
+      <c r="U6" s="12">
         <v>7</v>
       </c>
-      <c r="V6" s="42">
+      <c r="V6" s="13">
         <v>3</v>
       </c>
       <c r="W6" s="4">
@@ -3602,11 +3669,11 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="74"/>
-      <c r="C7" s="63" t="s">
-        <v>694</v>
-      </c>
-      <c r="D7" s="63"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="34" t="s">
+        <v>693</v>
+      </c>
+      <c r="D7" s="34"/>
       <c r="E7" s="4">
         <v>0</v>
       </c>
@@ -3643,22 +3710,22 @@
       <c r="P7" s="4">
         <v>0</v>
       </c>
-      <c r="Q7" s="37">
+      <c r="Q7" s="8">
         <v>12</v>
       </c>
-      <c r="R7" s="38">
+      <c r="R7" s="9">
         <v>11</v>
       </c>
-      <c r="S7" s="39">
+      <c r="S7" s="10">
         <v>10</v>
       </c>
-      <c r="T7" s="40">
+      <c r="T7" s="11">
         <v>19</v>
       </c>
-      <c r="U7" s="41">
+      <c r="U7" s="12">
         <v>10</v>
       </c>
-      <c r="V7" s="42">
+      <c r="V7" s="13">
         <v>11</v>
       </c>
       <c r="W7" s="4">
@@ -3672,129 +3739,129 @@
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="C8" s="70" t="s">
-        <v>695</v>
-      </c>
-      <c r="D8" s="70"/>
-      <c r="E8" s="78">
+      <c r="C8" s="40" t="s">
+        <v>694</v>
+      </c>
+      <c r="D8" s="40"/>
+      <c r="E8" s="48">
         <f>SUM(E3:G3)</f>
         <v>8</v>
       </c>
-      <c r="F8" s="79"/>
-      <c r="G8" s="79"/>
-      <c r="H8" s="64">
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="35">
         <f>SUM(H3:J3)</f>
         <v>13</v>
       </c>
-      <c r="I8" s="64"/>
-      <c r="J8" s="64"/>
-      <c r="K8" s="69">
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="39">
         <f>SUM(K3:M3)</f>
         <v>13</v>
       </c>
-      <c r="L8" s="69"/>
-      <c r="M8" s="69"/>
-      <c r="N8" s="69">
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
+      <c r="N8" s="39">
         <f>SUM(N3:P3)</f>
         <v>8</v>
       </c>
-      <c r="O8" s="69"/>
-      <c r="P8" s="69"/>
-      <c r="Q8" s="65">
+      <c r="O8" s="39"/>
+      <c r="P8" s="39"/>
+      <c r="Q8" s="36">
         <f>SUM(Q6:S6)</f>
         <v>25</v>
       </c>
-      <c r="R8" s="65"/>
-      <c r="S8" s="65"/>
-      <c r="T8" s="77">
+      <c r="R8" s="36"/>
+      <c r="S8" s="36"/>
+      <c r="T8" s="47">
         <f>SUM(T6:V6)</f>
         <v>19</v>
       </c>
-      <c r="U8" s="77"/>
-      <c r="V8" s="77"/>
+      <c r="U8" s="47"/>
+      <c r="V8" s="47"/>
     </row>
     <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="75" t="s">
-        <v>699</v>
-      </c>
-      <c r="D9" s="75"/>
-      <c r="E9" s="66">
+      <c r="C9" s="45" t="s">
+        <v>698</v>
+      </c>
+      <c r="D9" s="45"/>
+      <c r="E9" s="37">
         <f>SUM(E8:P8)</f>
         <v>42</v>
       </c>
-      <c r="F9" s="66"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="66"/>
-      <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="66"/>
-      <c r="L9" s="66"/>
-      <c r="M9" s="66"/>
-      <c r="N9" s="66"/>
-      <c r="O9" s="66"/>
-      <c r="P9" s="66"/>
-      <c r="Q9" s="67">
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="37"/>
+      <c r="Q9" s="38">
         <f>SUM(Q8:V8)</f>
         <v>44</v>
       </c>
-      <c r="R9" s="67"/>
-      <c r="S9" s="67"/>
-      <c r="T9" s="67"/>
-      <c r="U9" s="67"/>
-      <c r="V9" s="67"/>
+      <c r="R9" s="38"/>
+      <c r="S9" s="38"/>
+      <c r="T9" s="38"/>
+      <c r="U9" s="38"/>
+      <c r="V9" s="38"/>
     </row>
     <row r="10" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="70" t="s">
-        <v>696</v>
-      </c>
-      <c r="D10" s="70"/>
-      <c r="E10" s="76">
+      <c r="C10" s="40" t="s">
+        <v>695</v>
+      </c>
+      <c r="D10" s="40"/>
+      <c r="E10" s="46">
         <f>SUM(E8:V8)</f>
         <v>86</v>
       </c>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="76"/>
-      <c r="K10" s="76"/>
-      <c r="L10" s="76"/>
-      <c r="M10" s="76"/>
-      <c r="N10" s="76"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="76"/>
-      <c r="Q10" s="76"/>
-      <c r="R10" s="76"/>
-      <c r="S10" s="76"/>
-      <c r="T10" s="76"/>
-      <c r="U10" s="76"/>
-      <c r="V10" s="76"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46"/>
+      <c r="P10" s="46"/>
+      <c r="Q10" s="46"/>
+      <c r="R10" s="46"/>
+      <c r="S10" s="46"/>
+      <c r="T10" s="46"/>
+      <c r="U10" s="46"/>
+      <c r="V10" s="46"/>
     </row>
     <row r="11" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="43"/>
-      <c r="R11" s="43"/>
-      <c r="S11" s="43"/>
-      <c r="T11" s="43"/>
-      <c r="U11" s="43"/>
-      <c r="V11" s="43"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="14"/>
+      <c r="S11" s="14"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="14"/>
+      <c r="V11" s="14"/>
     </row>
     <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="6" t="s">
         <v>121</v>
       </c>
       <c r="B12" t="s">
@@ -3806,18 +3873,18 @@
       <c r="D12" t="s">
         <v>606</v>
       </c>
-      <c r="E12" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="45" t="s">
-        <v>704</v>
-      </c>
-      <c r="H12" s="53" t="s">
-        <v>704</v>
+      <c r="E12" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
+      <c r="A13" s="6"/>
       <c r="B13" t="s">
         <v>10</v>
       </c>
@@ -3827,18 +3894,18 @@
       <c r="D13" t="s">
         <v>607</v>
       </c>
-      <c r="E13" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" s="45" t="s">
-        <v>704</v>
-      </c>
-      <c r="I13" s="54" t="s">
-        <v>704</v>
+      <c r="E13" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="I13" s="25" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
+      <c r="A14" s="6"/>
       <c r="B14" t="s">
         <v>12</v>
       </c>
@@ -3848,18 +3915,18 @@
       <c r="D14" t="s">
         <v>608</v>
       </c>
-      <c r="E14" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="45" t="s">
-        <v>704</v>
-      </c>
-      <c r="H14" s="53" t="s">
-        <v>704</v>
+      <c r="E14" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
+      <c r="A15" s="6"/>
       <c r="B15" t="s">
         <v>14</v>
       </c>
@@ -3869,24 +3936,24 @@
       <c r="D15" t="s">
         <v>609</v>
       </c>
-      <c r="E15" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="45" t="s">
-        <v>704</v>
-      </c>
-      <c r="K15" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q15" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R15" s="38" t="s">
-        <v>704</v>
+      <c r="E15" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q15" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R15" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
+      <c r="A16" s="6"/>
       <c r="B16" t="s">
         <v>16</v>
       </c>
@@ -3896,21 +3963,21 @@
       <c r="D16" t="s">
         <v>610</v>
       </c>
-      <c r="F16" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="G16" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="K16" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="N16" s="49" t="s">
-        <v>704</v>
+      <c r="F16" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="N16" s="20" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
+      <c r="A17" s="6"/>
       <c r="B17" t="s">
         <v>18</v>
       </c>
@@ -3920,18 +3987,18 @@
       <c r="D17" t="s">
         <v>611</v>
       </c>
-      <c r="F17" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="G17" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="L17" s="50" t="s">
-        <v>704</v>
+      <c r="F17" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="L17" s="21" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
+      <c r="A18" s="6"/>
       <c r="B18" t="s">
         <v>20</v>
       </c>
@@ -3941,30 +4008,30 @@
       <c r="D18" t="s">
         <v>612</v>
       </c>
-      <c r="F18" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="L18" s="50" t="s">
-        <v>704</v>
-      </c>
-      <c r="O18" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="P18" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="R18" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S18" s="39" t="s">
-        <v>704</v>
+      <c r="F18" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>703</v>
+      </c>
+      <c r="O18" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="R18" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S18" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
+      <c r="A19" s="6"/>
       <c r="B19" t="s">
         <v>22</v>
       </c>
@@ -3974,18 +4041,18 @@
       <c r="D19" t="s">
         <v>613</v>
       </c>
-      <c r="F19" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="48" t="s">
-        <v>704</v>
-      </c>
-      <c r="I19" s="54" t="s">
-        <v>704</v>
+      <c r="F19" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>703</v>
+      </c>
+      <c r="I19" s="25" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
+      <c r="A20" s="6"/>
       <c r="B20" t="s">
         <v>24</v>
       </c>
@@ -3995,18 +4062,18 @@
       <c r="D20" t="s">
         <v>615</v>
       </c>
-      <c r="H20" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="K20" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q20" s="47" t="s">
-        <v>704</v>
+      <c r="H20" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K20" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q20" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
+      <c r="A21" s="6"/>
       <c r="B21" t="s">
         <v>26</v>
       </c>
@@ -4016,18 +4083,18 @@
       <c r="D21" t="s">
         <v>616</v>
       </c>
-      <c r="H21" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="K21" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q21" s="47" t="s">
-        <v>704</v>
+      <c r="H21" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q21" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
+      <c r="A22" s="6"/>
       <c r="B22" t="s">
         <v>28</v>
       </c>
@@ -4037,29 +4104,29 @@
       <c r="D22" t="s">
         <v>614</v>
       </c>
-      <c r="H22" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="I22" s="54" t="s">
-        <v>704</v>
+      <c r="H22" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I22" s="25" t="s">
+        <v>703</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
-      <c r="N22" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="O22" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q22" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R22" s="38" t="s">
-        <v>704</v>
+      <c r="N22" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="O22" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q22" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R22" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
+      <c r="A23" s="6"/>
       <c r="B23" t="s">
         <v>30</v>
       </c>
@@ -4069,19 +4136,19 @@
       <c r="D23" t="s">
         <v>620</v>
       </c>
-      <c r="H23" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="I23" s="54" t="s">
-        <v>704</v>
+      <c r="H23" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I23" s="25" t="s">
+        <v>703</v>
       </c>
       <c r="K23" s="1"/>
-      <c r="N23" s="49" t="s">
-        <v>704</v>
+      <c r="N23" s="20" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
+      <c r="A24" s="6"/>
       <c r="B24" t="s">
         <v>34</v>
       </c>
@@ -4091,24 +4158,21 @@
       <c r="D24" t="s">
         <v>623</v>
       </c>
-      <c r="H24" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="I24" s="54" t="s">
-        <v>704</v>
-      </c>
-      <c r="K24" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="N24" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q24" s="47" t="s">
-        <v>704</v>
+      <c r="H24" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I24" s="25" t="s">
+        <v>703</v>
+      </c>
+      <c r="K24" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q24" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
+      <c r="A25" s="6"/>
       <c r="B25" t="s">
         <v>36</v>
       </c>
@@ -4118,22 +4182,22 @@
       <c r="D25" t="s">
         <v>619</v>
       </c>
-      <c r="H25" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="I25" s="54" t="s">
-        <v>704</v>
+      <c r="H25" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>703</v>
       </c>
       <c r="K25" s="1"/>
-      <c r="N25" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q25" s="47" t="s">
-        <v>704</v>
+      <c r="N25" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q25" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12"/>
+      <c r="A26" s="6"/>
       <c r="B26" t="s">
         <v>39</v>
       </c>
@@ -4143,24 +4207,24 @@
       <c r="D26" t="s">
         <v>663</v>
       </c>
-      <c r="I26" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="J26" s="55" t="s">
-        <v>704</v>
-      </c>
-      <c r="K26" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="N26" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q26" s="47" t="s">
-        <v>704</v>
+      <c r="I26" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J26" s="26" t="s">
+        <v>703</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="N26" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q26" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
+      <c r="A27" s="6"/>
       <c r="B27" t="s">
         <v>41</v>
       </c>
@@ -4170,21 +4234,21 @@
       <c r="D27" t="s">
         <v>635</v>
       </c>
-      <c r="I27" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="J27" s="55" t="s">
-        <v>704</v>
-      </c>
-      <c r="O27" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="R27" s="38" t="s">
-        <v>704</v>
+      <c r="I27" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J27" s="26" t="s">
+        <v>703</v>
+      </c>
+      <c r="O27" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="R27" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
+      <c r="A28" s="6"/>
       <c r="B28" t="s">
         <v>43</v>
       </c>
@@ -4194,24 +4258,24 @@
       <c r="D28" t="s">
         <v>626</v>
       </c>
-      <c r="I28" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="J28" s="55" t="s">
-        <v>704</v>
-      </c>
-      <c r="K28" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="N28" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q28" s="47" t="s">
-        <v>704</v>
+      <c r="I28" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J28" s="26" t="s">
+        <v>703</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="N28" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q28" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12"/>
+      <c r="A29" s="6"/>
       <c r="B29" t="s">
         <v>45</v>
       </c>
@@ -4221,24 +4285,24 @@
       <c r="D29" t="s">
         <v>627</v>
       </c>
-      <c r="I29" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="J29" s="55" t="s">
-        <v>704</v>
-      </c>
-      <c r="K29" s="46" t="s">
-        <v>704</v>
-      </c>
-      <c r="N29" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q29" s="47" t="s">
-        <v>704</v>
+      <c r="I29" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J29" s="26" t="s">
+        <v>703</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="N29" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q29" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12"/>
+      <c r="A30" s="6"/>
       <c r="B30" t="s">
         <v>47</v>
       </c>
@@ -4248,18 +4312,18 @@
       <c r="D30" t="s">
         <v>642</v>
       </c>
-      <c r="J30" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="P30" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="S30" s="39" t="s">
-        <v>704</v>
+      <c r="J30" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="P30" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="S30" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
+      <c r="A31" s="6"/>
       <c r="B31" t="s">
         <v>49</v>
       </c>
@@ -4269,30 +4333,30 @@
       <c r="D31" t="s">
         <v>637</v>
       </c>
-      <c r="J31" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="L31" s="50" t="s">
-        <v>704</v>
-      </c>
-      <c r="M31" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="O31" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="P31" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="R31" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S31" s="39" t="s">
-        <v>704</v>
+      <c r="J31" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="L31" s="21" t="s">
+        <v>703</v>
+      </c>
+      <c r="M31" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="O31" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="P31" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="R31" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S31" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12"/>
+      <c r="A32" s="6"/>
       <c r="B32" t="s">
         <v>51</v>
       </c>
@@ -4302,18 +4366,18 @@
       <c r="D32" t="s">
         <v>645</v>
       </c>
-      <c r="J32" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="P32" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="S32" s="39" t="s">
-        <v>704</v>
+      <c r="J32" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="P32" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="S32" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
+      <c r="A33" s="6"/>
       <c r="B33" t="s">
         <v>53</v>
       </c>
@@ -4323,18 +4387,18 @@
       <c r="D33" t="s">
         <v>630</v>
       </c>
-      <c r="K33" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="N33" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q33" s="47" t="s">
-        <v>704</v>
+      <c r="K33" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="N33" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q33" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A34" s="12"/>
+      <c r="A34" s="6"/>
       <c r="B34" t="s">
         <v>55</v>
       </c>
@@ -4344,18 +4408,18 @@
       <c r="D34" t="s">
         <v>631</v>
       </c>
-      <c r="K34" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="N34" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q34" s="47" t="s">
-        <v>704</v>
+      <c r="K34" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="N34" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q34" s="18" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12"/>
+      <c r="A35" s="6"/>
       <c r="B35" t="s">
         <v>91</v>
       </c>
@@ -4365,27 +4429,27 @@
       <c r="D35" t="s">
         <v>643</v>
       </c>
-      <c r="K35" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="L35" s="50" t="s">
-        <v>704</v>
-      </c>
-      <c r="N35" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="O35" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q35" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R35" s="38" t="s">
-        <v>704</v>
+      <c r="K35" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="L35" s="21" t="s">
+        <v>703</v>
+      </c>
+      <c r="N35" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="O35" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q35" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R35" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A36" s="12"/>
+      <c r="A36" s="6"/>
       <c r="B36" t="s">
         <v>57</v>
       </c>
@@ -4395,27 +4459,27 @@
       <c r="D36" t="s">
         <v>624</v>
       </c>
-      <c r="K36" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="L36" s="50" t="s">
-        <v>704</v>
-      </c>
-      <c r="N36" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="O36" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q36" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R36" s="38" t="s">
-        <v>704</v>
+      <c r="K36" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="L36" s="21" t="s">
+        <v>703</v>
+      </c>
+      <c r="N36" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="O36" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q36" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R36" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A37" s="12"/>
+      <c r="A37" s="6"/>
       <c r="B37" t="s">
         <v>61</v>
       </c>
@@ -4425,36 +4489,36 @@
       <c r="D37" t="s">
         <v>618</v>
       </c>
-      <c r="K37" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="L37" s="50" t="s">
-        <v>704</v>
-      </c>
-      <c r="M37" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="N37" s="49" t="s">
-        <v>704</v>
-      </c>
-      <c r="O37" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="P37" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="Q37" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R37" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S37" s="39" t="s">
-        <v>704</v>
+      <c r="K37" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="L37" s="21" t="s">
+        <v>703</v>
+      </c>
+      <c r="M37" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="N37" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="O37" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="P37" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q37" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R37" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S37" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A38" s="12"/>
+      <c r="A38" s="6"/>
       <c r="B38" t="s">
         <v>88</v>
       </c>
@@ -4464,21 +4528,21 @@
       <c r="D38" t="s">
         <v>632</v>
       </c>
-      <c r="L38" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="M38" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="R38" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S38" s="39" t="s">
-        <v>704</v>
+      <c r="L38" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M38" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="R38" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S38" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A39" s="12"/>
+      <c r="A39" s="6"/>
       <c r="B39" t="s">
         <v>68</v>
       </c>
@@ -4488,21 +4552,21 @@
       <c r="D39" t="s">
         <v>634</v>
       </c>
-      <c r="L39" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="M39" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="R39" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S39" s="39" t="s">
-        <v>704</v>
+      <c r="L39" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M39" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="R39" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S39" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A40" s="12"/>
+      <c r="A40" s="6"/>
       <c r="B40" t="s">
         <v>70</v>
       </c>
@@ -4512,27 +4576,21 @@
       <c r="D40" t="s">
         <v>636</v>
       </c>
-      <c r="L40" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="M40" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="O40" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="P40" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="R40" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S40" s="39" t="s">
-        <v>704</v>
+      <c r="L40" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M40" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="R40" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S40" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A41" s="12"/>
+      <c r="A41" s="6"/>
       <c r="B41" t="s">
         <v>77</v>
       </c>
@@ -4542,27 +4600,21 @@
       <c r="D41" t="s">
         <v>641</v>
       </c>
-      <c r="L41" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="M41" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="O41" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="P41" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="R41" s="38" t="s">
-        <v>704</v>
-      </c>
-      <c r="S41" s="39" t="s">
-        <v>704</v>
+      <c r="L41" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M41" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="R41" s="9" t="s">
+        <v>703</v>
+      </c>
+      <c r="S41" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A42" s="12"/>
+      <c r="A42" s="6"/>
       <c r="B42" t="s">
         <v>79</v>
       </c>
@@ -4572,18 +4624,18 @@
       <c r="D42" t="s">
         <v>644</v>
       </c>
-      <c r="L42" s="50" t="s">
-        <v>9</v>
-      </c>
-      <c r="M42" s="51" t="s">
-        <v>704</v>
-      </c>
-      <c r="S42" s="39" t="s">
-        <v>704</v>
+      <c r="L42" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M42" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="S42" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A43" s="12"/>
+      <c r="A43" s="6"/>
       <c r="B43" t="s">
         <v>81</v>
       </c>
@@ -4593,18 +4645,18 @@
       <c r="D43" t="s">
         <v>646</v>
       </c>
-      <c r="M43" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="P43" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="S43" s="39" t="s">
-        <v>704</v>
+      <c r="M43" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="P43" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="S43" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A44" s="12"/>
+      <c r="A44" s="6"/>
       <c r="B44" t="s">
         <v>83</v>
       </c>
@@ -4614,18 +4666,18 @@
       <c r="D44" t="s">
         <v>647</v>
       </c>
-      <c r="M44" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="P44" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="S44" s="39" t="s">
-        <v>704</v>
+      <c r="M44" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="P44" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="S44" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
+      <c r="A45" s="6"/>
       <c r="B45" t="s">
         <v>85</v>
       </c>
@@ -4635,18 +4687,18 @@
       <c r="D45" t="s">
         <v>648</v>
       </c>
-      <c r="M45" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="P45" s="14" t="s">
-        <v>704</v>
-      </c>
-      <c r="S45" s="39" t="s">
-        <v>704</v>
+      <c r="M45" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="P45" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="S45" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A46" s="12"/>
+      <c r="A46" s="6"/>
       <c r="B46" t="s">
         <v>63</v>
       </c>
@@ -4657,20 +4709,20 @@
         <v>625</v>
       </c>
       <c r="L46" s="1"/>
-      <c r="N46" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O46" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="R46" s="61" t="s">
+      <c r="N46" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O46" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="R46" s="32" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A47" s="12"/>
+      <c r="A47" s="6"/>
       <c r="B47" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C47" t="s">
         <v>65</v>
@@ -4679,20 +4731,20 @@
         <v>629</v>
       </c>
       <c r="L47" s="1"/>
-      <c r="N47" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O47" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="R47" s="61" t="s">
+      <c r="N47" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O47" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="R47" s="32" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A48" s="12"/>
+      <c r="A48" s="6"/>
       <c r="B48" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C48" t="s">
         <v>66</v>
@@ -4701,18 +4753,18 @@
         <v>628</v>
       </c>
       <c r="L48" s="1"/>
-      <c r="N48" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O48" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="R48" s="61" t="s">
+      <c r="N48" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O48" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="R48" s="32" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A49" s="12"/>
+      <c r="A49" s="6"/>
       <c r="B49" t="s">
         <v>59</v>
       </c>
@@ -4722,15 +4774,15 @@
       <c r="D49" t="s">
         <v>622</v>
       </c>
-      <c r="N49" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O49" s="52" t="s">
-        <v>704</v>
+      <c r="N49" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O49" s="23" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="50" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A50" s="12"/>
+      <c r="A50" s="6"/>
       <c r="B50" t="s">
         <v>72</v>
       </c>
@@ -4741,18 +4793,18 @@
         <v>638</v>
       </c>
       <c r="M50" s="1"/>
-      <c r="N50" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O50" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="S50" s="39" t="s">
-        <v>704</v>
+      <c r="N50" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O50" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="S50" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="51" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A51" s="12"/>
+      <c r="A51" s="6"/>
       <c r="B51" t="s">
         <v>74</v>
       </c>
@@ -4762,18 +4814,18 @@
       <c r="D51" t="s">
         <v>639</v>
       </c>
-      <c r="N51" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O51" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="S51" s="39" t="s">
-        <v>704</v>
+      <c r="N51" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O51" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="S51" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A52" s="12"/>
+      <c r="A52" s="6"/>
       <c r="B52" t="s">
         <v>87</v>
       </c>
@@ -4783,18 +4835,18 @@
       <c r="D52" t="s">
         <v>640</v>
       </c>
-      <c r="N52" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="O52" s="52" t="s">
-        <v>704</v>
-      </c>
-      <c r="S52" s="39" t="s">
-        <v>704</v>
+      <c r="N52" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O52" s="23" t="s">
+        <v>703</v>
+      </c>
+      <c r="S52" s="10" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A53" s="12"/>
+      <c r="A53" s="6"/>
       <c r="B53" t="s">
         <v>32</v>
       </c>
@@ -4806,14 +4858,14 @@
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
-      <c r="O53" s="52" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q53" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="R53" s="38" t="s">
-        <v>704</v>
+      <c r="O53" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q53" s="18" t="s">
+        <v>703</v>
+      </c>
+      <c r="R53" s="9" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="54" spans="1:26" ht="6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4841,8 +4893,8 @@
       <c r="Z54" s="2"/>
     </row>
     <row r="55" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="80" t="s">
-        <v>703</v>
+      <c r="A55" s="50" t="s">
+        <v>702</v>
       </c>
       <c r="B55" t="s">
         <v>92</v>
@@ -4853,15 +4905,15 @@
       <c r="D55" t="s">
         <v>649</v>
       </c>
-      <c r="N55" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q55" s="56" t="s">
+      <c r="Q55" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T55" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A56" s="80"/>
+      <c r="A56" s="50"/>
       <c r="B56" t="s">
         <v>93</v>
       </c>
@@ -4871,15 +4923,15 @@
       <c r="D56" t="s">
         <v>650</v>
       </c>
-      <c r="N56" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q56" s="56" t="s">
+      <c r="Q56" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T56" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="57" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A57" s="80"/>
+      <c r="A57" s="50"/>
       <c r="B57" t="s">
         <v>94</v>
       </c>
@@ -4889,15 +4941,15 @@
       <c r="D57" t="s">
         <v>651</v>
       </c>
-      <c r="N57" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q57" s="56" t="s">
+      <c r="Q57" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T57" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A58" s="80"/>
+      <c r="A58" s="50"/>
       <c r="B58" t="s">
         <v>95</v>
       </c>
@@ -4907,15 +4959,15 @@
       <c r="D58" t="s">
         <v>652</v>
       </c>
-      <c r="N58" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q58" s="56" t="s">
+      <c r="Q58" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T58" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A59" s="80"/>
+      <c r="A59" s="50"/>
       <c r="B59" t="s">
         <v>96</v>
       </c>
@@ -4925,15 +4977,15 @@
       <c r="D59" t="s">
         <v>653</v>
       </c>
-      <c r="N59" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q59" s="56" t="s">
+      <c r="Q59" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T59" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="60" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A60" s="80"/>
+      <c r="A60" s="50"/>
       <c r="B60" t="s">
         <v>97</v>
       </c>
@@ -4943,15 +4995,15 @@
       <c r="D60" t="s">
         <v>654</v>
       </c>
-      <c r="N60" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q60" s="56" t="s">
+      <c r="Q60" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T60" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A61" s="80"/>
+      <c r="A61" s="50"/>
       <c r="B61" t="s">
         <v>98</v>
       </c>
@@ -4961,15 +5013,15 @@
       <c r="D61" t="s">
         <v>633</v>
       </c>
-      <c r="N61" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q61" s="56" t="s">
+      <c r="Q61" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="T61" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="62" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A62" s="80"/>
+      <c r="A62" s="50"/>
       <c r="B62" t="s">
         <v>100</v>
       </c>
@@ -4979,12 +5031,12 @@
       <c r="D62" t="s">
         <v>656</v>
       </c>
-      <c r="N62" s="47" t="s">
+      <c r="Q62" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="63" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A63" s="80"/>
+      <c r="A63" s="50"/>
       <c r="B63" t="s">
         <v>101</v>
       </c>
@@ -4994,15 +5046,15 @@
       <c r="D63" t="s">
         <v>657</v>
       </c>
-      <c r="N63" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="O63" s="57" t="s">
+      <c r="Q63" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="R63" s="28" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A64" s="80"/>
+      <c r="A64" s="50"/>
       <c r="B64" t="s">
         <v>102</v>
       </c>
@@ -5012,12 +5064,12 @@
       <c r="D64" t="s">
         <v>658</v>
       </c>
-      <c r="N64" s="47" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A65" s="80"/>
+      <c r="Q64" s="18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A65" s="50"/>
       <c r="B65" t="s">
         <v>103</v>
       </c>
@@ -5027,15 +5079,15 @@
       <c r="D65" t="s">
         <v>659</v>
       </c>
-      <c r="N65" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="O65" s="57" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A66" s="80"/>
+      <c r="Q65" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="R65" s="28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A66" s="50"/>
       <c r="B66" t="s">
         <v>104</v>
       </c>
@@ -5045,15 +5097,15 @@
       <c r="D66" t="s">
         <v>660</v>
       </c>
-      <c r="N66" s="47" t="s">
-        <v>9</v>
-      </c>
-      <c r="O66" s="57" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A67" s="80"/>
+      <c r="Q66" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="R66" s="28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A67" s="50"/>
       <c r="B67" t="s">
         <v>124</v>
       </c>
@@ -5063,18 +5115,18 @@
       <c r="D67" t="s">
         <v>662</v>
       </c>
-      <c r="O67" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="P67" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q67" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A68" s="80"/>
+      <c r="R67" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="S67" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="T67" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A68" s="50"/>
       <c r="B68" t="s">
         <v>126</v>
       </c>
@@ -5084,15 +5136,15 @@
       <c r="D68" t="s">
         <v>664</v>
       </c>
-      <c r="O68" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q68" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A69" s="80"/>
+      <c r="R68" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="T68" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A69" s="50"/>
       <c r="B69" t="s">
         <v>128</v>
       </c>
@@ -5102,12 +5154,12 @@
       <c r="D69" t="s">
         <v>665</v>
       </c>
-      <c r="O69" s="57" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A70" s="80"/>
+      <c r="R69" s="28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A70" s="50"/>
       <c r="B70" t="s">
         <v>130</v>
       </c>
@@ -5117,15 +5169,15 @@
       <c r="D70" t="s">
         <v>681</v>
       </c>
-      <c r="O70" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="P70" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A71" s="80"/>
+      <c r="R70" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="S70" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A71" s="50"/>
       <c r="B71" t="s">
         <v>132</v>
       </c>
@@ -5135,15 +5187,15 @@
       <c r="D71" t="s">
         <v>682</v>
       </c>
-      <c r="O71" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="P71" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A72" s="80"/>
+      <c r="R71" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="S71" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A72" s="50"/>
       <c r="B72" t="s">
         <v>134</v>
       </c>
@@ -5153,15 +5205,15 @@
       <c r="D72" t="s">
         <v>666</v>
       </c>
-      <c r="O72" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q72" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A73" s="80"/>
+      <c r="R72" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="T72" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A73" s="50"/>
       <c r="B73" t="s">
         <v>136</v>
       </c>
@@ -5171,15 +5223,15 @@
       <c r="D73" t="s">
         <v>689</v>
       </c>
-      <c r="O73" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="P73" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A74" s="80"/>
+      <c r="R73" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="S73" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A74" s="50"/>
       <c r="B74" t="s">
         <v>138</v>
       </c>
@@ -5189,12 +5241,12 @@
       <c r="D74" t="s">
         <v>685</v>
       </c>
-      <c r="P74" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A75" s="80"/>
+      <c r="S74" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A75" s="50"/>
       <c r="B75" t="s">
         <v>140</v>
       </c>
@@ -5204,12 +5256,12 @@
       <c r="D75" t="s">
         <v>686</v>
       </c>
-      <c r="P75" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A76" s="80"/>
+      <c r="S75" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A76" s="50"/>
       <c r="B76" t="s">
         <v>142</v>
       </c>
@@ -5219,12 +5271,12 @@
       <c r="D76" t="s">
         <v>687</v>
       </c>
-      <c r="P76" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A77" s="80"/>
+      <c r="S76" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A77" s="50"/>
       <c r="B77" t="s">
         <v>144</v>
       </c>
@@ -5234,12 +5286,12 @@
       <c r="D77" t="s">
         <v>688</v>
       </c>
-      <c r="P77" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A78" s="80"/>
+      <c r="S77" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A78" s="50"/>
       <c r="B78" t="s">
         <v>145</v>
       </c>
@@ -5249,12 +5301,12 @@
       <c r="D78" t="s">
         <v>683</v>
       </c>
-      <c r="P78" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A79" s="80"/>
+      <c r="S78" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A79" s="50"/>
       <c r="B79" t="s">
         <v>149</v>
       </c>
@@ -5264,12 +5316,12 @@
       <c r="D79" t="s">
         <v>690</v>
       </c>
-      <c r="P79" s="58" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A80" s="80"/>
+      <c r="S79" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A80" s="50"/>
       <c r="B80" t="s">
         <v>122</v>
       </c>
@@ -5279,12 +5331,12 @@
       <c r="D80" t="s">
         <v>661</v>
       </c>
-      <c r="Q80" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A81" s="80"/>
+      <c r="T80" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A81" s="50"/>
       <c r="B81" t="s">
         <v>155</v>
       </c>
@@ -5294,12 +5346,12 @@
       <c r="D81" t="s">
         <v>668</v>
       </c>
-      <c r="Q81" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A82" s="80"/>
+      <c r="T81" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A82" s="50"/>
       <c r="B82" t="s">
         <v>156</v>
       </c>
@@ -5309,12 +5361,12 @@
       <c r="D82" t="s">
         <v>669</v>
       </c>
-      <c r="Q82" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A83" s="80"/>
+      <c r="T82" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A83" s="50"/>
       <c r="B83" t="s">
         <v>159</v>
       </c>
@@ -5324,12 +5376,12 @@
       <c r="D83" t="s">
         <v>670</v>
       </c>
-      <c r="Q83" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A84" s="80"/>
+      <c r="T83" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A84" s="50"/>
       <c r="B84" t="s">
         <v>161</v>
       </c>
@@ -5339,12 +5391,12 @@
       <c r="D84" t="s">
         <v>671</v>
       </c>
-      <c r="Q84" s="56" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A85" s="80"/>
+      <c r="T84" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A85" s="50"/>
       <c r="B85" t="s">
         <v>163</v>
       </c>
@@ -5354,15 +5406,15 @@
       <c r="D85" t="s">
         <v>672</v>
       </c>
-      <c r="Q85" s="56" t="s">
-        <v>9</v>
-      </c>
-      <c r="R85" s="59" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A86" s="80"/>
+      <c r="T85" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="U85" s="30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A86" s="50"/>
       <c r="B86" t="s">
         <v>164</v>
       </c>
@@ -5372,15 +5424,15 @@
       <c r="D86" t="s">
         <v>673</v>
       </c>
-      <c r="Q86" s="56" t="s">
-        <v>9</v>
-      </c>
-      <c r="R86" s="59" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A87" s="80"/>
+      <c r="T86" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="U86" s="30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A87" s="50"/>
       <c r="B87" t="s">
         <v>99</v>
       </c>
@@ -5390,18 +5442,18 @@
       <c r="D87" t="s">
         <v>655</v>
       </c>
-      <c r="O87" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q87" s="56" t="s">
-        <v>9</v>
-      </c>
-      <c r="R87" s="59" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A88" s="80"/>
+      <c r="R87" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="T87" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="U87" s="30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A88" s="50"/>
       <c r="B88" t="s">
         <v>153</v>
       </c>
@@ -5411,18 +5463,18 @@
       <c r="D88" t="s">
         <v>667</v>
       </c>
-      <c r="Q88" s="56" t="s">
-        <v>9</v>
-      </c>
-      <c r="R88" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S88" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A89" s="80"/>
+      <c r="T88" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="U88" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V88" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A89" s="50"/>
       <c r="B89" t="s">
         <v>167</v>
       </c>
@@ -5432,15 +5484,15 @@
       <c r="D89" t="s">
         <v>675</v>
       </c>
-      <c r="R89" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S89" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A90" s="80"/>
+      <c r="U89" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V89" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A90" s="50"/>
       <c r="B90" t="s">
         <v>169</v>
       </c>
@@ -5450,15 +5502,15 @@
       <c r="D90" t="s">
         <v>674</v>
       </c>
-      <c r="R90" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S90" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A91" s="80"/>
+      <c r="U90" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V90" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A91" s="50"/>
       <c r="B91" t="s">
         <v>171</v>
       </c>
@@ -5468,15 +5520,15 @@
       <c r="D91" t="s">
         <v>676</v>
       </c>
-      <c r="R91" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S91" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A92" s="80"/>
+      <c r="U91" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V91" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A92" s="50"/>
       <c r="B92" t="s">
         <v>172</v>
       </c>
@@ -5486,15 +5538,15 @@
       <c r="D92" t="s">
         <v>677</v>
       </c>
-      <c r="R92" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S92" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A93" s="80"/>
+      <c r="U92" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V92" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A93" s="50"/>
       <c r="B93" t="s">
         <v>173</v>
       </c>
@@ -5504,15 +5556,15 @@
       <c r="D93" t="s">
         <v>679</v>
       </c>
-      <c r="R93" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S93" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A94" s="80"/>
+      <c r="U93" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V93" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A94" s="50"/>
       <c r="B94" t="s">
         <v>174</v>
       </c>
@@ -5522,15 +5574,15 @@
       <c r="D94" t="s">
         <v>678</v>
       </c>
-      <c r="R94" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S94" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A95" s="80"/>
+      <c r="U94" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V94" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A95" s="50"/>
       <c r="B95" t="s">
         <v>179</v>
       </c>
@@ -5540,15 +5592,15 @@
       <c r="D95" t="s">
         <v>680</v>
       </c>
-      <c r="R95" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="S95" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A96" s="80"/>
+      <c r="U95" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="V95" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A96" s="50"/>
       <c r="B96" t="s">
         <v>181</v>
       </c>
@@ -5558,12 +5610,12 @@
       <c r="D96" t="s">
         <v>681</v>
       </c>
-      <c r="S96" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A97" s="80"/>
+      <c r="V96" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A97" s="50"/>
       <c r="B97" t="s">
         <v>183</v>
       </c>
@@ -5573,12 +5625,12 @@
       <c r="D97" t="s">
         <v>691</v>
       </c>
-      <c r="S97" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A98" s="80"/>
+      <c r="V97" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A98" s="50"/>
       <c r="B98" t="s">
         <v>185</v>
       </c>
@@ -5588,281 +5640,281 @@
       <c r="D98" t="s">
         <v>684</v>
       </c>
-      <c r="S98" s="60" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="99" spans="1:19" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A100" s="81" t="s">
-        <v>778</v>
+      <c r="V98" s="31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:22" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A100" s="51" t="s">
+        <v>776</v>
       </c>
       <c r="B100" t="s">
+        <v>709</v>
+      </c>
+      <c r="C100" t="s">
+        <v>733</v>
+      </c>
+      <c r="D100" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A101" s="51"/>
+      <c r="B101" t="s">
         <v>710</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C101" t="s">
+        <v>737</v>
+      </c>
+      <c r="D101" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A102" s="51"/>
+      <c r="B102" t="s">
+        <v>719</v>
+      </c>
+      <c r="C102" t="s">
+        <v>738</v>
+      </c>
+      <c r="D102" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="103" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A103" s="51"/>
+      <c r="B103" t="s">
+        <v>711</v>
+      </c>
+      <c r="C103" t="s">
+        <v>741</v>
+      </c>
+      <c r="D103" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A104" s="51"/>
+      <c r="B104" t="s">
+        <v>712</v>
+      </c>
+      <c r="C104" t="s">
+        <v>742</v>
+      </c>
+      <c r="D104" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A105" s="51"/>
+      <c r="B105" t="s">
+        <v>713</v>
+      </c>
+      <c r="C105" t="s">
+        <v>744</v>
+      </c>
+      <c r="D105" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A106" s="51"/>
+      <c r="B106" t="s">
+        <v>714</v>
+      </c>
+      <c r="C106" t="s">
+        <v>748</v>
+      </c>
+      <c r="D106" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A107" s="51"/>
+      <c r="B107" t="s">
+        <v>715</v>
+      </c>
+      <c r="C107" t="s">
+        <v>750</v>
+      </c>
+      <c r="D107" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A108" s="51"/>
+      <c r="B108" t="s">
+        <v>716</v>
+      </c>
+      <c r="C108" t="s">
         <v>734</v>
       </c>
-      <c r="D100" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A101" s="81"/>
-      <c r="B101" t="s">
-        <v>711</v>
-      </c>
-      <c r="C101" t="s">
-        <v>738</v>
-      </c>
-      <c r="D101" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A102" s="81"/>
-      <c r="B102" t="s">
+      <c r="D108" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A109" s="51"/>
+      <c r="B109" t="s">
+        <v>717</v>
+      </c>
+      <c r="C109" t="s">
+        <v>735</v>
+      </c>
+      <c r="D109" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A110" s="51"/>
+      <c r="B110" t="s">
+        <v>718</v>
+      </c>
+      <c r="C110" t="s">
+        <v>739</v>
+      </c>
+      <c r="D110" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A111" s="51"/>
+      <c r="B111" t="s">
         <v>720</v>
       </c>
-      <c r="C102" t="s">
-        <v>739</v>
-      </c>
-      <c r="D102" t="s">
-        <v>762</v>
-      </c>
-    </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A103" s="81"/>
-      <c r="B103" t="s">
-        <v>712</v>
-      </c>
-      <c r="C103" t="s">
-        <v>742</v>
-      </c>
-      <c r="D103" t="s">
-        <v>763</v>
-      </c>
-    </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A104" s="81"/>
-      <c r="B104" t="s">
-        <v>713</v>
-      </c>
-      <c r="C104" t="s">
+      <c r="C111" t="s">
+        <v>740</v>
+      </c>
+      <c r="D111" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A112" s="51"/>
+      <c r="B112" t="s">
+        <v>721</v>
+      </c>
+      <c r="C112" t="s">
         <v>743</v>
       </c>
-      <c r="D104" t="s">
-        <v>766</v>
-      </c>
-    </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A105" s="81"/>
-      <c r="B105" t="s">
-        <v>714</v>
-      </c>
-      <c r="C105" t="s">
+      <c r="D112" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="51"/>
+      <c r="B113" t="s">
+        <v>722</v>
+      </c>
+      <c r="C113" t="s">
         <v>745</v>
       </c>
-      <c r="D105" t="s">
-        <v>764</v>
-      </c>
-    </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A106" s="81"/>
-      <c r="B106" t="s">
-        <v>715</v>
-      </c>
-      <c r="C106" t="s">
+      <c r="D113" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="51"/>
+      <c r="B114" t="s">
+        <v>723</v>
+      </c>
+      <c r="C114" t="s">
+        <v>747</v>
+      </c>
+      <c r="D114" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="51"/>
+      <c r="B115" t="s">
+        <v>724</v>
+      </c>
+      <c r="C115" t="s">
         <v>749</v>
       </c>
-      <c r="D106" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A107" s="81"/>
-      <c r="B107" t="s">
-        <v>716</v>
-      </c>
-      <c r="C107" t="s">
+      <c r="D115" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="51"/>
+      <c r="B116" t="s">
+        <v>725</v>
+      </c>
+      <c r="D116" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="51"/>
+      <c r="B117" t="s">
+        <v>726</v>
+      </c>
+      <c r="C117" t="s">
+        <v>736</v>
+      </c>
+      <c r="D117" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="51"/>
+      <c r="B118" t="s">
+        <v>727</v>
+      </c>
+      <c r="D118" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="51"/>
+      <c r="B119" t="s">
+        <v>728</v>
+      </c>
+      <c r="D119" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="51"/>
+      <c r="B120" t="s">
+        <v>729</v>
+      </c>
+      <c r="D120" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="51"/>
+      <c r="B121" t="s">
+        <v>730</v>
+      </c>
+      <c r="D121" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="51"/>
+      <c r="B122" t="s">
+        <v>731</v>
+      </c>
+      <c r="C122" t="s">
+        <v>746</v>
+      </c>
+      <c r="D122" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="51"/>
+      <c r="B123" t="s">
+        <v>732</v>
+      </c>
+      <c r="D123" t="s">
         <v>751</v>
-      </c>
-      <c r="D107" t="s">
-        <v>767</v>
-      </c>
-    </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A108" s="81"/>
-      <c r="B108" t="s">
-        <v>717</v>
-      </c>
-      <c r="C108" t="s">
-        <v>735</v>
-      </c>
-      <c r="D108" t="s">
-        <v>768</v>
-      </c>
-    </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A109" s="81"/>
-      <c r="B109" t="s">
-        <v>718</v>
-      </c>
-      <c r="C109" t="s">
-        <v>736</v>
-      </c>
-      <c r="D109" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A110" s="81"/>
-      <c r="B110" t="s">
-        <v>719</v>
-      </c>
-      <c r="C110" t="s">
-        <v>740</v>
-      </c>
-      <c r="D110" t="s">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A111" s="81"/>
-      <c r="B111" t="s">
-        <v>721</v>
-      </c>
-      <c r="C111" t="s">
-        <v>741</v>
-      </c>
-      <c r="D111" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A112" s="81"/>
-      <c r="B112" t="s">
-        <v>722</v>
-      </c>
-      <c r="C112" t="s">
-        <v>744</v>
-      </c>
-      <c r="D112" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" s="81"/>
-      <c r="B113" t="s">
-        <v>723</v>
-      </c>
-      <c r="C113" t="s">
-        <v>746</v>
-      </c>
-      <c r="D113" t="s">
-        <v>773</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="81"/>
-      <c r="B114" t="s">
-        <v>724</v>
-      </c>
-      <c r="C114" t="s">
-        <v>748</v>
-      </c>
-      <c r="D114" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="81"/>
-      <c r="B115" t="s">
-        <v>725</v>
-      </c>
-      <c r="C115" t="s">
-        <v>750</v>
-      </c>
-      <c r="D115" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="81"/>
-      <c r="B116" t="s">
-        <v>726</v>
-      </c>
-      <c r="D116" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" s="81"/>
-      <c r="B117" t="s">
-        <v>727</v>
-      </c>
-      <c r="C117" t="s">
-        <v>737</v>
-      </c>
-      <c r="D117" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="81"/>
-      <c r="B118" t="s">
-        <v>728</v>
-      </c>
-      <c r="D118" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" s="81"/>
-      <c r="B119" t="s">
-        <v>729</v>
-      </c>
-      <c r="D119" t="s">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" s="81"/>
-      <c r="B120" t="s">
-        <v>730</v>
-      </c>
-      <c r="D120" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="81"/>
-      <c r="B121" t="s">
-        <v>731</v>
-      </c>
-      <c r="D121" t="s">
-        <v>754</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="81"/>
-      <c r="B122" t="s">
-        <v>732</v>
-      </c>
-      <c r="C122" t="s">
-        <v>747</v>
-      </c>
-      <c r="D122" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="81"/>
-      <c r="B123" t="s">
-        <v>733</v>
-      </c>
-      <c r="D123" t="s">
-        <v>752</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added All ex gym leader opponents into map with deck restrictions, rewards and marked in tracker
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9DD1ED-4F86-43CE-9833-84758C142FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440BFEF5-5621-4613-AC37-59BDF8BA9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="796">
   <si>
     <t>CELESTE HARBOUR</t>
   </si>
@@ -4475,11 +4475,11 @@
       </c>
       <c r="AB7" s="166">
         <f>COUNTIF(AB55:AB108,"✅")+COUNTIF(AB55:AB108,"✔️")</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AC7" s="50">
         <f>COUNTIF(AC55:AC108,"✅")+COUNTIF(AC55:AC108,"✔️")</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AD7" s="167">
         <f>COUNTIF(AD55:AD108,"✅")+COUNTIF(AD55:AD108,"✔️")</f>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="D100" s="1">
         <f>COUNTIF(G100:AAA100,"✅")+COUNTIF(G100:AAA100,"✔️")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E100" t="s">
         <v>289</v>
@@ -7475,12 +7475,6 @@
         <v>31</v>
       </c>
       <c r="AA100" s="160" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB100" s="166" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC100" s="50" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Map Update: Split out all Opponents into the new 4 timelots updated cheat keys
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783D9178-324F-44FB-8F8B-5327D30DE239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B93CB40-9DEF-4EC1-A3A4-43DA8F3CF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2186" uniqueCount="836">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2300" uniqueCount="857">
   <si>
     <t>CELESTE HARBOUR</t>
   </si>
@@ -2562,6 +2562,70 @@
   <si>
     <t>GYM CHALLENGE
 14</t>
+  </si>
+  <si>
+    <t>GYM CHALLENGE
+15</t>
+  </si>
+  <si>
+    <t>Morn 11</t>
+  </si>
+  <si>
+    <t>After 11</t>
+  </si>
+  <si>
+    <t>Eve 11</t>
+  </si>
+  <si>
+    <t>Nite 11</t>
+  </si>
+  <si>
+    <t>Morn12</t>
+  </si>
+  <si>
+    <t>After 12</t>
+  </si>
+  <si>
+    <t>Eve 12</t>
+  </si>
+  <si>
+    <t>Nite 12</t>
+  </si>
+  <si>
+    <t>Morn13</t>
+  </si>
+  <si>
+    <t>After 13</t>
+  </si>
+  <si>
+    <t>Eve 13</t>
+  </si>
+  <si>
+    <t>Nite 13</t>
+  </si>
+  <si>
+    <t>Morn14</t>
+  </si>
+  <si>
+    <t>After 14</t>
+  </si>
+  <si>
+    <t>Eve 14</t>
+  </si>
+  <si>
+    <t>Nite 14</t>
+  </si>
+  <si>
+    <t>Morn 15</t>
+  </si>
+  <si>
+    <t>After 15</t>
+  </si>
+  <si>
+    <t>Eve 15</t>
+  </si>
+  <si>
+    <t>Nite 15</t>
   </si>
 </sst>
 </file>
@@ -3208,7 +3272,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="203">
+  <cellXfs count="204">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3524,14 +3588,131 @@
     <xf numFmtId="0" fontId="4" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3579,18 +3760,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="29" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3609,120 +3779,17 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="28" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="28" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4109,7 +4176,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BJ133"/>
+  <dimension ref="A1:BN133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -4142,95 +4209,103 @@
     <col min="52" max="53" width="6.5703125" customWidth="1"/>
     <col min="54" max="54" width="6.5703125" style="52" customWidth="1"/>
     <col min="55" max="62" width="6.5703125" customWidth="1"/>
+    <col min="63" max="63" width="6.5703125" style="62" customWidth="1"/>
+    <col min="64" max="66" width="6.5703125" style="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G1" s="121" t="s">
+    <row r="1" spans="1:66" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="170" t="s">
         <v>771</v>
       </c>
-      <c r="H1" s="122"/>
-      <c r="I1" s="122"/>
-      <c r="J1" s="123"/>
-      <c r="K1" s="180" t="s">
+      <c r="H1" s="171"/>
+      <c r="I1" s="171"/>
+      <c r="J1" s="172"/>
+      <c r="K1" s="149" t="s">
         <v>770</v>
       </c>
-      <c r="L1" s="181"/>
-      <c r="M1" s="181"/>
-      <c r="N1" s="182"/>
-      <c r="O1" s="190" t="s">
+      <c r="L1" s="150"/>
+      <c r="M1" s="150"/>
+      <c r="N1" s="151"/>
+      <c r="O1" s="161" t="s">
         <v>769</v>
       </c>
-      <c r="P1" s="191"/>
-      <c r="Q1" s="191"/>
-      <c r="R1" s="192"/>
-      <c r="S1" s="183" t="s">
+      <c r="P1" s="162"/>
+      <c r="Q1" s="162"/>
+      <c r="R1" s="163"/>
+      <c r="S1" s="152" t="s">
         <v>768</v>
       </c>
-      <c r="T1" s="184"/>
-      <c r="U1" s="184"/>
-      <c r="V1" s="185"/>
-      <c r="W1" s="124" t="s">
+      <c r="T1" s="153"/>
+      <c r="U1" s="153"/>
+      <c r="V1" s="154"/>
+      <c r="W1" s="173" t="s">
         <v>765</v>
       </c>
-      <c r="X1" s="125"/>
-      <c r="Y1" s="126"/>
-      <c r="Z1" s="127"/>
-      <c r="AA1" s="152" t="s">
+      <c r="X1" s="174"/>
+      <c r="Y1" s="175"/>
+      <c r="Z1" s="176"/>
+      <c r="AA1" s="196" t="s">
         <v>766</v>
       </c>
-      <c r="AB1" s="153"/>
-      <c r="AC1" s="154"/>
-      <c r="AD1" s="155"/>
-      <c r="AE1" s="148" t="s">
+      <c r="AB1" s="197"/>
+      <c r="AC1" s="198"/>
+      <c r="AD1" s="199"/>
+      <c r="AE1" s="192" t="s">
         <v>767</v>
       </c>
-      <c r="AF1" s="149"/>
-      <c r="AG1" s="150"/>
-      <c r="AH1" s="151"/>
-      <c r="AI1" s="193" t="s">
+      <c r="AF1" s="193"/>
+      <c r="AG1" s="194"/>
+      <c r="AH1" s="195"/>
+      <c r="AI1" s="165" t="s">
         <v>772</v>
       </c>
-      <c r="AJ1" s="194"/>
-      <c r="AK1" s="195"/>
-      <c r="AL1" s="196"/>
-      <c r="AM1" s="166" t="s">
+      <c r="AJ1" s="166"/>
+      <c r="AK1" s="167"/>
+      <c r="AL1" s="168"/>
+      <c r="AM1" s="131" t="s">
         <v>784</v>
       </c>
-      <c r="AN1" s="167"/>
-      <c r="AO1" s="168"/>
-      <c r="AP1" s="169"/>
-      <c r="AQ1" s="166" t="s">
+      <c r="AN1" s="132"/>
+      <c r="AO1" s="133"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="131" t="s">
         <v>827</v>
       </c>
-      <c r="AR1" s="167"/>
-      <c r="AS1" s="168"/>
-      <c r="AT1" s="169"/>
-      <c r="AU1" s="166" t="s">
+      <c r="AR1" s="132"/>
+      <c r="AS1" s="133"/>
+      <c r="AT1" s="134"/>
+      <c r="AU1" s="131" t="s">
         <v>832</v>
       </c>
-      <c r="AV1" s="167"/>
-      <c r="AW1" s="168"/>
-      <c r="AX1" s="169"/>
-      <c r="AY1" s="166" t="s">
+      <c r="AV1" s="132"/>
+      <c r="AW1" s="133"/>
+      <c r="AX1" s="134"/>
+      <c r="AY1" s="131" t="s">
         <v>833</v>
       </c>
-      <c r="AZ1" s="167"/>
-      <c r="BA1" s="168"/>
-      <c r="BB1" s="169"/>
-      <c r="BC1" s="166" t="s">
+      <c r="AZ1" s="132"/>
+      <c r="BA1" s="133"/>
+      <c r="BB1" s="134"/>
+      <c r="BC1" s="131" t="s">
         <v>834</v>
       </c>
-      <c r="BD1" s="167"/>
-      <c r="BE1" s="168"/>
-      <c r="BF1" s="169"/>
-      <c r="BG1" s="166" t="s">
+      <c r="BD1" s="132"/>
+      <c r="BE1" s="133"/>
+      <c r="BF1" s="134"/>
+      <c r="BG1" s="131" t="s">
         <v>835</v>
       </c>
-      <c r="BH1" s="167"/>
-      <c r="BI1" s="168"/>
-      <c r="BJ1" s="169"/>
-    </row>
-    <row r="2" spans="1:62" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="BH1" s="132"/>
+      <c r="BI1" s="133"/>
+      <c r="BJ1" s="134"/>
+      <c r="BK1" s="131" t="s">
+        <v>836</v>
+      </c>
+      <c r="BL1" s="132"/>
+      <c r="BM1" s="133"/>
+      <c r="BN1" s="134"/>
+    </row>
+    <row r="2" spans="1:66" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G2" s="39" t="s">
         <v>787</v>
       </c>
@@ -4352,64 +4427,76 @@
         <v>831</v>
       </c>
       <c r="AU2" s="73" t="s">
-        <v>821</v>
+        <v>837</v>
       </c>
       <c r="AV2" s="25" t="s">
-        <v>826</v>
+        <v>838</v>
       </c>
       <c r="AW2" s="106" t="s">
-        <v>7</v>
+        <v>839</v>
       </c>
       <c r="AX2" s="27" t="s">
-        <v>764</v>
+        <v>840</v>
       </c>
       <c r="AY2" s="78" t="s">
-        <v>822</v>
+        <v>841</v>
       </c>
       <c r="AZ2" s="26" t="s">
-        <v>825</v>
+        <v>842</v>
       </c>
       <c r="BA2" s="26" t="s">
-        <v>773</v>
+        <v>843</v>
       </c>
       <c r="BB2" s="79" t="s">
-        <v>774</v>
+        <v>844</v>
       </c>
       <c r="BC2" s="85" t="s">
-        <v>823</v>
+        <v>845</v>
       </c>
       <c r="BD2" s="87" t="s">
-        <v>824</v>
+        <v>846</v>
       </c>
       <c r="BE2" s="87" t="s">
-        <v>785</v>
+        <v>847</v>
       </c>
       <c r="BF2" s="89" t="s">
-        <v>786</v>
+        <v>848</v>
       </c>
       <c r="BG2" s="85" t="s">
-        <v>828</v>
+        <v>849</v>
       </c>
       <c r="BH2" s="87" t="s">
-        <v>829</v>
+        <v>850</v>
       </c>
       <c r="BI2" s="87" t="s">
-        <v>830</v>
+        <v>851</v>
       </c>
       <c r="BJ2" s="89" t="s">
-        <v>831</v>
-      </c>
-    </row>
-    <row r="3" spans="1:62" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="117" t="s">
+        <v>852</v>
+      </c>
+      <c r="BK2" s="73" t="s">
+        <v>853</v>
+      </c>
+      <c r="BL2" s="25" t="s">
+        <v>854</v>
+      </c>
+      <c r="BM2" s="106" t="s">
+        <v>855</v>
+      </c>
+      <c r="BN2" s="27" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="3" spans="1:66" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="169" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="146" t="s">
+      <c r="D3" s="191" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="118"/>
-      <c r="F3" s="120"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="156"/>
       <c r="G3" s="40">
         <f t="shared" ref="G3:AP3" si="0">COUNTIF(G11:G58,"✅")</f>
         <v>5</v>
@@ -4555,7 +4642,7 @@
         <v>0</v>
       </c>
       <c r="AQ3" s="43">
-        <f t="shared" ref="AQ3:CD3" si="1">COUNTIF(AQ11:AQ58,"✅")</f>
+        <f t="shared" ref="AQ3:BF3" si="1">COUNTIF(AQ11:AQ58,"✅")</f>
         <v>0</v>
       </c>
       <c r="AR3" s="29">
@@ -4619,7 +4706,7 @@
         <v>0</v>
       </c>
       <c r="BG3" s="43">
-        <f t="shared" ref="BG3:BJ3" si="2">COUNTIF(BG11:BG58,"✅")</f>
+        <f t="shared" ref="BG3:BN3" si="2">COUNTIF(BG11:BG58,"✅")</f>
         <v>0</v>
       </c>
       <c r="BH3" s="29">
@@ -4634,15 +4721,31 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="118"/>
+      <c r="BK3" s="43">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BL3" s="29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BM3" s="29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BN3" s="29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="148"/>
       <c r="C4" s="13"/>
-      <c r="D4" s="146" t="s">
+      <c r="D4" s="191" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="118"/>
-      <c r="F4" s="120"/>
+      <c r="E4" s="148"/>
+      <c r="F4" s="156"/>
       <c r="G4" s="40">
         <f t="shared" ref="G4:AP4" si="3">COUNTIF(G11:G58,"✅")+COUNTIF(G11:G58,"✔️")</f>
         <v>5</v>
@@ -4788,7 +4891,7 @@
         <v>9</v>
       </c>
       <c r="AQ4" s="80">
-        <f t="shared" ref="AQ4:CD4" si="4">COUNTIF(AQ11:AQ58,"✅")+COUNTIF(AQ11:AQ58,"✔️")</f>
+        <f t="shared" ref="AQ4:BF4" si="4">COUNTIF(AQ11:AQ58,"✅")+COUNTIF(AQ11:AQ58,"✔️")</f>
         <v>15</v>
       </c>
       <c r="AR4" s="30">
@@ -4852,7 +4955,7 @@
         <v>9</v>
       </c>
       <c r="BG4" s="80">
-        <f t="shared" ref="BG4:BJ4" si="5">COUNTIF(BG11:BG58,"✅")+COUNTIF(BG11:BG58,"✔️")</f>
+        <f t="shared" ref="BG4:BN4" si="5">COUNTIF(BG11:BG58,"✅")+COUNTIF(BG11:BG58,"✔️")</f>
         <v>15</v>
       </c>
       <c r="BH4" s="30">
@@ -4867,8 +4970,24 @@
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:62" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK4" s="74">
+        <f t="shared" si="5"/>
+        <v>12</v>
+      </c>
+      <c r="BL4" s="75">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="BM4" s="107">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="BN4" s="77">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:66" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -4906,16 +5025,16 @@
       <c r="BG5" s="51"/>
       <c r="BJ5" s="52"/>
     </row>
-    <row r="6" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="133" t="s">
+    <row r="6" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="182" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="14"/>
-      <c r="D6" s="119" t="s">
+      <c r="D6" s="155" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="118"/>
-      <c r="F6" s="120"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="156"/>
       <c r="G6" s="43">
         <v>0</v>
       </c>
@@ -5027,8 +5146,8 @@
         <v>0</v>
       </c>
       <c r="AM6" s="86">
-        <f>COUNTIF(AM60:AM120,"✅")</f>
-        <v>4</v>
+        <f>COUNTIF(AM60:AM124,"✅")</f>
+        <v>8</v>
       </c>
       <c r="AN6" s="88">
         <f>COUNTIF(AN60:AN116,"✅")</f>
@@ -5059,7 +5178,7 @@
         <v>0</v>
       </c>
       <c r="AU6" s="74">
-        <f t="shared" ref="AU6:BJ6" si="7">COUNTIF(AU60:AU116,"✅")</f>
+        <f t="shared" ref="AU6:BB6" si="7">COUNTIF(AU60:AU116,"✅")</f>
         <v>0</v>
       </c>
       <c r="AV6" s="75">
@@ -5122,15 +5241,31 @@
         <f>COUNTIF(BJ60:BJ116,"✅")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="118"/>
+      <c r="BK6" s="74">
+        <f t="shared" ref="BK6:BN6" si="8">COUNTIF(BK60:BK116,"✅")</f>
+        <v>0</v>
+      </c>
+      <c r="BL6" s="75">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="BM6" s="107">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="BN6" s="77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="148"/>
       <c r="C7" s="15"/>
-      <c r="D7" s="119" t="s">
+      <c r="D7" s="155" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="118"/>
-      <c r="F7" s="120"/>
+      <c r="E7" s="148"/>
+      <c r="F7" s="156"/>
       <c r="G7" s="43">
         <v>0</v>
       </c>
@@ -5178,353 +5313,379 @@
         <v>0</v>
       </c>
       <c r="W7" s="40">
-        <f>COUNTIF(W60:W116,"✅")+COUNTIF(W60:W116,"✔️")</f>
+        <f t="shared" ref="W7:BJ7" si="9">COUNTIF(W60:W116,"✅")+COUNTIF(W60:W116,"✔️")</f>
         <v>7</v>
       </c>
       <c r="X7" s="41">
-        <f>COUNTIF(X60:X116,"✅")+COUNTIF(X60:X116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>10</v>
       </c>
       <c r="Y7" s="93">
-        <f>COUNTIF(Y60:Y116,"✅")+COUNTIF(Y60:Y116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>8</v>
       </c>
       <c r="Z7" s="53">
-        <f>COUNTIF(Z60:Z116,"✅")+COUNTIF(Z60:Z116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>6</v>
       </c>
       <c r="AA7" s="95">
-        <f>COUNTIF(AA60:AA116,"✅")+COUNTIF(AA60:AA116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>15</v>
       </c>
       <c r="AB7" s="102">
-        <f>COUNTIF(AB60:AB116,"✅")+COUNTIF(AB60:AB116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>19</v>
       </c>
       <c r="AC7" s="99">
-        <f>COUNTIF(AC60:AC116,"✅")+COUNTIF(AC60:AC116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>12</v>
       </c>
       <c r="AD7" s="53">
-        <f>COUNTIF(AD60:AD116,"✅")+COUNTIF(AD60:AD116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>11</v>
       </c>
       <c r="AE7" s="74">
-        <f>COUNTIF(AE60:AE116,"✅")+COUNTIF(AE60:AE116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>15</v>
       </c>
       <c r="AF7" s="75">
-        <f>COUNTIF(AF60:AF116,"✅")+COUNTIF(AF60:AF116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>20</v>
       </c>
       <c r="AG7" s="107">
-        <f>COUNTIF(AG60:AG116,"✅")+COUNTIF(AG60:AG116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>14</v>
       </c>
       <c r="AH7" s="77">
-        <f>COUNTIF(AH60:AH116,"✅")+COUNTIF(AH60:AH116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>16</v>
       </c>
       <c r="AI7" s="80">
-        <f>COUNTIF(AI60:AI116,"✅")+COUNTIF(AI60:AI116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>16</v>
       </c>
       <c r="AJ7" s="30">
-        <f>COUNTIF(AJ60:AJ116,"✅")+COUNTIF(AJ60:AJ116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>21</v>
       </c>
       <c r="AK7" s="30">
-        <f>COUNTIF(AK60:AK116,"✅")+COUNTIF(AK60:AK116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>13</v>
       </c>
       <c r="AL7" s="81">
-        <f>COUNTIF(AL60:AL116,"✅")+COUNTIF(AL60:AL116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>12</v>
       </c>
       <c r="AM7" s="86">
-        <f>COUNTIF(AM60:AM116,"✅")+COUNTIF(AM60:AM116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>16</v>
       </c>
       <c r="AN7" s="88">
-        <f>COUNTIF(AN60:AN116,"✅")+COUNTIF(AN60:AN116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>19</v>
       </c>
       <c r="AO7" s="88">
-        <f>COUNTIF(AO60:AO116,"✅")+COUNTIF(AO60:AO116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>14</v>
       </c>
       <c r="AP7" s="90">
-        <f>COUNTIF(AP60:AP116,"✅")+COUNTIF(AP60:AP116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>14</v>
       </c>
       <c r="AQ7" s="86">
-        <f>COUNTIF(AQ60:AQ116,"✅")+COUNTIF(AQ60:AQ116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>15</v>
       </c>
       <c r="AR7" s="88">
-        <f>COUNTIF(AR60:AR116,"✅")+COUNTIF(AR60:AR116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>18</v>
       </c>
       <c r="AS7" s="88">
-        <f>COUNTIF(AS60:AS116,"✅")+COUNTIF(AS60:AS116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>11</v>
       </c>
       <c r="AT7" s="90">
-        <f>COUNTIF(AT60:AT116,"✅")+COUNTIF(AT60:AT116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>10</v>
       </c>
       <c r="AU7" s="74">
-        <f>COUNTIF(AU60:AU116,"✅")+COUNTIF(AU60:AU116,"✔️")</f>
+        <f t="shared" si="9"/>
+        <v>12</v>
+      </c>
+      <c r="AV7" s="75">
+        <f t="shared" si="9"/>
+        <v>17</v>
+      </c>
+      <c r="AW7" s="107">
+        <f t="shared" si="9"/>
+        <v>10</v>
+      </c>
+      <c r="AX7" s="77">
+        <f t="shared" si="9"/>
+        <v>12</v>
+      </c>
+      <c r="AY7" s="80">
+        <f t="shared" si="9"/>
         <v>13</v>
       </c>
-      <c r="AV7" s="75">
-        <f>COUNTIF(AV60:AV116,"✅")+COUNTIF(AV60:AV116,"✔️")</f>
+      <c r="AZ7" s="30">
+        <f t="shared" si="9"/>
+        <v>17</v>
+      </c>
+      <c r="BA7" s="30">
+        <f t="shared" si="9"/>
+        <v>7</v>
+      </c>
+      <c r="BB7" s="81">
+        <f t="shared" si="9"/>
+        <v>6</v>
+      </c>
+      <c r="BC7" s="86">
+        <f t="shared" si="9"/>
+        <v>16</v>
+      </c>
+      <c r="BD7" s="88">
+        <f t="shared" si="9"/>
+        <v>19</v>
+      </c>
+      <c r="BE7" s="88">
+        <f t="shared" si="9"/>
+        <v>14</v>
+      </c>
+      <c r="BF7" s="90">
+        <f t="shared" si="9"/>
+        <v>14</v>
+      </c>
+      <c r="BG7" s="86">
+        <f t="shared" si="9"/>
+        <v>15</v>
+      </c>
+      <c r="BH7" s="88">
+        <f t="shared" si="9"/>
         <v>18</v>
       </c>
-      <c r="AW7" s="107">
-        <f>COUNTIF(AW60:AW116,"✅")+COUNTIF(AW60:AW116,"✔️")</f>
+      <c r="BI7" s="88">
+        <f t="shared" si="9"/>
         <v>11</v>
       </c>
-      <c r="AX7" s="77">
-        <f>COUNTIF(AX60:AX116,"✅")+COUNTIF(AX60:AX116,"✔️")</f>
-        <v>13</v>
-      </c>
-      <c r="AY7" s="80">
-        <f>COUNTIF(AY60:AY116,"✅")+COUNTIF(AY60:AY116,"✔️")</f>
-        <v>14</v>
-      </c>
-      <c r="AZ7" s="30">
-        <f>COUNTIF(AZ60:AZ116,"✅")+COUNTIF(AZ60:AZ116,"✔️")</f>
-        <v>18</v>
-      </c>
-      <c r="BA7" s="30">
-        <f>COUNTIF(BA60:BA116,"✅")+COUNTIF(BA60:BA116,"✔️")</f>
-        <v>8</v>
-      </c>
-      <c r="BB7" s="81">
-        <f>COUNTIF(BB60:BB116,"✅")+COUNTIF(BB60:BB116,"✔️")</f>
-        <v>7</v>
-      </c>
-      <c r="BC7" s="86">
-        <f>COUNTIF(BC60:BC116,"✅")+COUNTIF(BC60:BC116,"✔️")</f>
-        <v>16</v>
-      </c>
-      <c r="BD7" s="88">
-        <f>COUNTIF(BD60:BD116,"✅")+COUNTIF(BD60:BD116,"✔️")</f>
-        <v>19</v>
-      </c>
-      <c r="BE7" s="88">
-        <f>COUNTIF(BE60:BE116,"✅")+COUNTIF(BE60:BE116,"✔️")</f>
-        <v>14</v>
-      </c>
-      <c r="BF7" s="90">
-        <f>COUNTIF(BF60:BF116,"✅")+COUNTIF(BF60:BF116,"✔️")</f>
-        <v>14</v>
-      </c>
-      <c r="BG7" s="86">
-        <f>COUNTIF(BG60:BG116,"✅")+COUNTIF(BG60:BG116,"✔️")</f>
-        <v>15</v>
-      </c>
-      <c r="BH7" s="88">
-        <f>COUNTIF(BH60:BH116,"✅")+COUNTIF(BH60:BH116,"✔️")</f>
-        <v>18</v>
-      </c>
-      <c r="BI7" s="88">
-        <f>COUNTIF(BI60:BI116,"✅")+COUNTIF(BI60:BI116,"✔️")</f>
-        <v>11</v>
-      </c>
       <c r="BJ7" s="90">
-        <f>COUNTIF(BJ60:BJ116,"✅")+COUNTIF(BJ60:BJ116,"✔️")</f>
+        <f t="shared" si="9"/>
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="D8" s="132" t="s">
+      <c r="BK7" s="74">
+        <f t="shared" ref="BK7:BN7" si="10">COUNTIF(BK60:BK116,"✅")+COUNTIF(BK60:BK116,"✔️")</f>
         <v>12</v>
       </c>
-      <c r="E8" s="118"/>
-      <c r="F8" s="120"/>
-      <c r="G8" s="186">
+      <c r="BL7" s="75">
+        <f t="shared" si="10"/>
+        <v>17</v>
+      </c>
+      <c r="BM7" s="107">
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="BN7" s="77">
+        <f t="shared" si="10"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="D8" s="181" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="148"/>
+      <c r="F8" s="156"/>
+      <c r="G8" s="157">
         <f>SUM(G3:J3)</f>
         <v>9</v>
       </c>
-      <c r="H8" s="187"/>
-      <c r="I8" s="188"/>
-      <c r="J8" s="189"/>
-      <c r="K8" s="174">
+      <c r="H8" s="158"/>
+      <c r="I8" s="159"/>
+      <c r="J8" s="160"/>
+      <c r="K8" s="141">
         <f>SUM(K3:N3)</f>
         <v>14</v>
       </c>
-      <c r="L8" s="175"/>
-      <c r="M8" s="176"/>
-      <c r="N8" s="177"/>
-      <c r="O8" s="128">
+      <c r="L8" s="142"/>
+      <c r="M8" s="143"/>
+      <c r="N8" s="144"/>
+      <c r="O8" s="177">
         <f>SUM(O3:R3)</f>
         <v>14</v>
       </c>
-      <c r="P8" s="129"/>
-      <c r="Q8" s="130"/>
-      <c r="R8" s="131"/>
-      <c r="S8" s="138">
+      <c r="P8" s="178"/>
+      <c r="Q8" s="179"/>
+      <c r="R8" s="180"/>
+      <c r="S8" s="187">
         <f>SUM(S3:V3)</f>
         <v>9</v>
       </c>
-      <c r="T8" s="139"/>
-      <c r="U8" s="140"/>
-      <c r="V8" s="141"/>
-      <c r="W8" s="134">
+      <c r="T8" s="188"/>
+      <c r="U8" s="189"/>
+      <c r="V8" s="190"/>
+      <c r="W8" s="183">
         <f>SUM(W6:Z6)</f>
         <v>16</v>
       </c>
-      <c r="X8" s="135"/>
-      <c r="Y8" s="136"/>
-      <c r="Z8" s="137"/>
-      <c r="AA8" s="160">
+      <c r="X8" s="184"/>
+      <c r="Y8" s="185"/>
+      <c r="Z8" s="186"/>
+      <c r="AA8" s="135">
         <f>SUM(AA6:AD6)</f>
         <v>16</v>
       </c>
-      <c r="AB8" s="161"/>
-      <c r="AC8" s="162"/>
-      <c r="AD8" s="163"/>
-      <c r="AE8" s="156">
+      <c r="AB8" s="136"/>
+      <c r="AC8" s="137"/>
+      <c r="AD8" s="138"/>
+      <c r="AE8" s="119">
         <f>SUM(AE6:AH6)</f>
         <v>15</v>
       </c>
-      <c r="AF8" s="157"/>
-      <c r="AG8" s="158"/>
-      <c r="AH8" s="159"/>
-      <c r="AI8" s="142">
+      <c r="AF8" s="120"/>
+      <c r="AG8" s="121"/>
+      <c r="AH8" s="122"/>
+      <c r="AI8" s="123">
         <f>SUM(AI6:AL6)</f>
         <v>8</v>
       </c>
-      <c r="AJ8" s="143"/>
-      <c r="AK8" s="144"/>
-      <c r="AL8" s="145"/>
-      <c r="AM8" s="170">
+      <c r="AJ8" s="124"/>
+      <c r="AK8" s="125"/>
+      <c r="AL8" s="126"/>
+      <c r="AM8" s="127">
         <f>SUM(AM6:AP6)</f>
-        <v>4</v>
-      </c>
-      <c r="AN8" s="171"/>
-      <c r="AO8" s="172"/>
-      <c r="AP8" s="173"/>
-      <c r="AQ8" s="170">
+        <v>8</v>
+      </c>
+      <c r="AN8" s="128"/>
+      <c r="AO8" s="129"/>
+      <c r="AP8" s="130"/>
+      <c r="AQ8" s="127">
         <f>SUM(AQ6:AT6)</f>
         <v>0</v>
       </c>
-      <c r="AR8" s="171"/>
-      <c r="AS8" s="172"/>
-      <c r="AT8" s="173"/>
-      <c r="AU8" s="156">
+      <c r="AR8" s="128"/>
+      <c r="AS8" s="129"/>
+      <c r="AT8" s="130"/>
+      <c r="AU8" s="119">
         <f>SUM(AU6:AX6)</f>
         <v>0</v>
       </c>
-      <c r="AV8" s="157"/>
-      <c r="AW8" s="158"/>
-      <c r="AX8" s="159"/>
-      <c r="AY8" s="142">
+      <c r="AV8" s="120"/>
+      <c r="AW8" s="121"/>
+      <c r="AX8" s="122"/>
+      <c r="AY8" s="123">
         <f>SUM(AY6:BB6)</f>
         <v>0</v>
       </c>
-      <c r="AZ8" s="143"/>
-      <c r="BA8" s="144"/>
-      <c r="BB8" s="145"/>
-      <c r="BC8" s="170">
+      <c r="AZ8" s="124"/>
+      <c r="BA8" s="125"/>
+      <c r="BB8" s="126"/>
+      <c r="BC8" s="127">
         <f>SUM(BC6:BF6)</f>
         <v>0</v>
       </c>
-      <c r="BD8" s="171"/>
-      <c r="BE8" s="172"/>
-      <c r="BF8" s="173"/>
-      <c r="BG8" s="170">
+      <c r="BD8" s="128"/>
+      <c r="BE8" s="129"/>
+      <c r="BF8" s="130"/>
+      <c r="BG8" s="127">
         <f>SUM(BG6:BJ6)</f>
         <v>0</v>
       </c>
-      <c r="BH8" s="171"/>
-      <c r="BI8" s="172"/>
-      <c r="BJ8" s="173"/>
-    </row>
-    <row r="9" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH8" s="128"/>
+      <c r="BI8" s="129"/>
+      <c r="BJ8" s="130"/>
+      <c r="BK8" s="119">
+        <f>SUM(BK6:BN6)</f>
+        <v>0</v>
+      </c>
+      <c r="BL8" s="120"/>
+      <c r="BM8" s="121"/>
+      <c r="BN8" s="122"/>
+    </row>
+    <row r="9" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D9" s="147" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="118"/>
-      <c r="F9" s="118"/>
-      <c r="G9" s="178">
+      <c r="E9" s="148"/>
+      <c r="F9" s="148"/>
+      <c r="G9" s="145">
         <f>SUM(G8:V8)</f>
         <v>46</v>
       </c>
-      <c r="H9" s="178"/>
-      <c r="I9" s="179"/>
-      <c r="J9" s="179"/>
-      <c r="K9" s="179"/>
-      <c r="L9" s="179"/>
-      <c r="M9" s="179"/>
-      <c r="N9" s="179"/>
-      <c r="O9" s="179"/>
-      <c r="P9" s="179"/>
-      <c r="Q9" s="179"/>
-      <c r="R9" s="179"/>
-      <c r="S9" s="179"/>
-      <c r="T9" s="179"/>
-      <c r="U9" s="179"/>
-      <c r="V9" s="179"/>
-      <c r="W9" s="197">
+      <c r="H9" s="145"/>
+      <c r="I9" s="146"/>
+      <c r="J9" s="146"/>
+      <c r="K9" s="146"/>
+      <c r="L9" s="146"/>
+      <c r="M9" s="146"/>
+      <c r="N9" s="146"/>
+      <c r="O9" s="146"/>
+      <c r="P9" s="146"/>
+      <c r="Q9" s="146"/>
+      <c r="R9" s="146"/>
+      <c r="S9" s="146"/>
+      <c r="T9" s="146"/>
+      <c r="U9" s="146"/>
+      <c r="V9" s="146"/>
+      <c r="W9" s="117">
         <f>SUM(W8:AL8)</f>
         <v>55</v>
       </c>
-      <c r="X9" s="198"/>
-      <c r="Y9" s="198"/>
-      <c r="Z9" s="198"/>
-      <c r="AA9" s="198"/>
-      <c r="AB9" s="198"/>
-      <c r="AC9" s="198"/>
-      <c r="AD9" s="198"/>
-      <c r="AE9" s="198"/>
-      <c r="AF9" s="198"/>
-      <c r="AG9" s="198"/>
-      <c r="AH9" s="198"/>
-      <c r="AI9" s="198"/>
-      <c r="AJ9" s="198"/>
-      <c r="AK9" s="198"/>
-      <c r="AL9" s="199"/>
-      <c r="AM9" s="197">
+      <c r="X9" s="118"/>
+      <c r="Y9" s="118"/>
+      <c r="Z9" s="118"/>
+      <c r="AA9" s="118"/>
+      <c r="AB9" s="118"/>
+      <c r="AC9" s="118"/>
+      <c r="AD9" s="118"/>
+      <c r="AE9" s="118"/>
+      <c r="AF9" s="118"/>
+      <c r="AG9" s="118"/>
+      <c r="AH9" s="118"/>
+      <c r="AI9" s="118"/>
+      <c r="AJ9" s="118"/>
+      <c r="AK9" s="118"/>
+      <c r="AL9" s="164"/>
+      <c r="AM9" s="117">
         <f>SUM(AM8:BB8)</f>
-        <v>4</v>
-      </c>
-      <c r="AN9" s="198"/>
-      <c r="AO9" s="198"/>
-      <c r="AP9" s="198"/>
-      <c r="AQ9" s="198"/>
-      <c r="AR9" s="198"/>
-      <c r="AS9" s="198"/>
-      <c r="AT9" s="198"/>
-      <c r="AU9"/>
-      <c r="AV9"/>
-      <c r="AW9"/>
-      <c r="AX9"/>
-      <c r="AY9"/>
-      <c r="BB9"/>
-      <c r="BC9" s="197">
-        <f>SUM(BC8:BR8)</f>
-        <v>0</v>
-      </c>
-      <c r="BD9" s="198"/>
-      <c r="BE9" s="198"/>
-      <c r="BF9" s="198"/>
-      <c r="BG9" s="198"/>
-      <c r="BH9" s="198"/>
-      <c r="BI9" s="198"/>
-      <c r="BJ9" s="198"/>
-    </row>
-    <row r="10" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="AN9" s="118"/>
+      <c r="AO9" s="118"/>
+      <c r="AP9" s="118"/>
+      <c r="AQ9" s="118"/>
+      <c r="AR9" s="118"/>
+      <c r="AS9" s="118"/>
+      <c r="AT9" s="118"/>
+      <c r="AU9" s="118"/>
+      <c r="AV9" s="118"/>
+      <c r="AW9" s="118"/>
+      <c r="AX9" s="118"/>
+      <c r="AY9" s="118"/>
+      <c r="AZ9" s="118"/>
+      <c r="BA9" s="118"/>
+      <c r="BB9" s="118"/>
+      <c r="BC9" s="118"/>
+      <c r="BD9" s="118"/>
+      <c r="BE9" s="118"/>
+      <c r="BF9" s="118"/>
+      <c r="BG9" s="118"/>
+      <c r="BH9" s="118"/>
+      <c r="BI9" s="118"/>
+      <c r="BJ9" s="118"/>
+      <c r="BK9" s="202"/>
+      <c r="BL9" s="202"/>
+      <c r="BM9" s="202"/>
+      <c r="BN9" s="202"/>
+    </row>
+    <row r="10" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D10" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="118"/>
-      <c r="F10" s="118"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
       <c r="G10" s="200">
-        <f>SUM(G8:AP8)</f>
-        <v>105</v>
+        <f>SUM(G8:BJ8)</f>
+        <v>109</v>
       </c>
       <c r="H10" s="201"/>
       <c r="I10" s="201"/>
@@ -5560,17 +5721,33 @@
       <c r="AM10" s="201"/>
       <c r="AN10" s="201"/>
       <c r="AO10" s="201"/>
-      <c r="AP10" s="202"/>
-      <c r="AQ10" s="51"/>
-      <c r="AU10"/>
-      <c r="AV10"/>
-      <c r="AW10"/>
-      <c r="AX10"/>
-      <c r="AY10"/>
-      <c r="BB10"/>
-      <c r="BG10" s="51"/>
-    </row>
-    <row r="11" spans="1:62" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AP10" s="201"/>
+      <c r="AQ10" s="201"/>
+      <c r="AR10" s="201"/>
+      <c r="AS10" s="201"/>
+      <c r="AT10" s="201"/>
+      <c r="AU10" s="201"/>
+      <c r="AV10" s="201"/>
+      <c r="AW10" s="201"/>
+      <c r="AX10" s="201"/>
+      <c r="AY10" s="201"/>
+      <c r="AZ10" s="201"/>
+      <c r="BA10" s="201"/>
+      <c r="BB10" s="201"/>
+      <c r="BC10" s="201"/>
+      <c r="BD10" s="201"/>
+      <c r="BE10" s="201"/>
+      <c r="BF10" s="201"/>
+      <c r="BG10" s="201"/>
+      <c r="BH10" s="201"/>
+      <c r="BI10" s="201"/>
+      <c r="BJ10" s="201"/>
+      <c r="BK10" s="203"/>
+      <c r="BL10" s="203"/>
+      <c r="BM10" s="203"/>
+      <c r="BN10" s="203"/>
+    </row>
+    <row r="11" spans="1:66" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="7" t="s">
         <v>15</v>
@@ -5616,7 +5793,7 @@
       <c r="BF11" s="31"/>
       <c r="BG11" s="51"/>
     </row>
-    <row r="12" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="96" t="s">
         <v>0</v>
       </c>
@@ -5627,7 +5804,7 @@
         <v>2</v>
       </c>
       <c r="D12" s="5">
-        <f t="shared" ref="D12:D57" si="8">COUNTIF(G12:AAJ12,"✅")+COUNTIF(G12:AAJ12,"✔️")</f>
+        <f t="shared" ref="D12:D57" si="11">COUNTIF(G12:AAN12,"✅")+COUNTIF(G12:AAN12,"✔️")</f>
         <v>3</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -5670,7 +5847,7 @@
       <c r="BI12" s="31"/>
       <c r="BJ12" s="31"/>
     </row>
-    <row r="13" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="97"/>
       <c r="B13" t="s">
         <v>20</v>
@@ -5679,7 +5856,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="E13" t="s">
@@ -5742,7 +5919,7 @@
       <c r="BI13" s="31"/>
       <c r="BJ13" s="31"/>
     </row>
-    <row r="14" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>25</v>
       </c>
@@ -5750,7 +5927,7 @@
         <v>2</v>
       </c>
       <c r="D14" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>13</v>
       </c>
       <c r="E14" t="s">
@@ -5817,7 +5994,7 @@
       <c r="BI14" s="31"/>
       <c r="BJ14" s="31"/>
     </row>
-    <row r="15" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>28</v>
       </c>
@@ -5825,7 +6002,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>14</v>
       </c>
       <c r="E15" t="s">
@@ -5895,7 +6072,7 @@
       <c r="BI15" s="31"/>
       <c r="BJ15" s="31"/>
     </row>
-    <row r="16" spans="1:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>31</v>
       </c>
@@ -5903,8 +6080,8 @@
         <v>4</v>
       </c>
       <c r="D16" s="1">
-        <f t="shared" si="8"/>
-        <v>18</v>
+        <f t="shared" si="11"/>
+        <v>19</v>
       </c>
       <c r="E16" t="s">
         <v>32</v>
@@ -5982,8 +6159,11 @@
       </c>
       <c r="BI16" s="31"/>
       <c r="BJ16" s="31"/>
-    </row>
-    <row r="17" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK16" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>34</v>
       </c>
@@ -5991,8 +6171,8 @@
         <v>4</v>
       </c>
       <c r="D17" s="1">
-        <f t="shared" si="8"/>
-        <v>15</v>
+        <f t="shared" si="11"/>
+        <v>16</v>
       </c>
       <c r="E17" t="s">
         <v>35</v>
@@ -6063,8 +6243,11 @@
       </c>
       <c r="BI17" s="31"/>
       <c r="BJ17" s="31"/>
-    </row>
-    <row r="18" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK17" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>43</v>
       </c>
@@ -6072,7 +6255,7 @@
         <v>2</v>
       </c>
       <c r="D18" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>16</v>
       </c>
       <c r="E18" t="s">
@@ -6146,7 +6329,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>37</v>
       </c>
@@ -6154,8 +6337,8 @@
         <v>3</v>
       </c>
       <c r="D19" s="1">
-        <f t="shared" si="8"/>
-        <v>14</v>
+        <f t="shared" si="11"/>
+        <v>16</v>
       </c>
       <c r="E19" t="s">
         <v>38</v>
@@ -6225,8 +6408,14 @@
       <c r="BJ19" s="53" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="20" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BL19" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM19" s="107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>40</v>
       </c>
@@ -6234,8 +6423,8 @@
         <v>2</v>
       </c>
       <c r="D20" s="1">
-        <f t="shared" si="8"/>
-        <v>20</v>
+        <f t="shared" si="11"/>
+        <v>22</v>
       </c>
       <c r="E20" t="s">
         <v>41</v>
@@ -6319,8 +6508,14 @@
       <c r="BH20" s="31"/>
       <c r="BI20" s="31"/>
       <c r="BJ20" s="31"/>
-    </row>
-    <row r="21" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BL20" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM20" s="107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>794</v>
       </c>
@@ -6328,7 +6523,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="E21" s="2" t="s">
@@ -6365,7 +6560,7 @@
       <c r="BI21" s="31"/>
       <c r="BJ21" s="31"/>
     </row>
-    <row r="22" spans="2:62" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>46</v>
       </c>
@@ -6373,8 +6568,8 @@
         <v>2</v>
       </c>
       <c r="D22" s="1">
-        <f t="shared" si="8"/>
-        <v>20</v>
+        <f t="shared" si="11"/>
+        <v>22</v>
       </c>
       <c r="E22" t="s">
         <v>47</v>
@@ -6458,8 +6653,14 @@
       </c>
       <c r="BI22" s="31"/>
       <c r="BJ22" s="31"/>
-    </row>
-    <row r="23" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BK22" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL22" s="61" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>49</v>
       </c>
@@ -6467,8 +6668,8 @@
         <v>2</v>
       </c>
       <c r="D23" s="1">
-        <f t="shared" si="8"/>
-        <v>20</v>
+        <f t="shared" si="11"/>
+        <v>22</v>
       </c>
       <c r="E23" t="s">
         <v>50</v>
@@ -6552,8 +6753,14 @@
       </c>
       <c r="BI23" s="31"/>
       <c r="BJ23" s="31"/>
-    </row>
-    <row r="24" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK23" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL23" s="61" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>55</v>
       </c>
@@ -6561,7 +6768,7 @@
         <v>4</v>
       </c>
       <c r="D24" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>12</v>
       </c>
       <c r="E24" t="s">
@@ -6627,8 +6834,9 @@
         <v>24</v>
       </c>
       <c r="BJ24" s="31"/>
-    </row>
-    <row r="25" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK24" s="48"/>
+    </row>
+    <row r="25" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>58</v>
       </c>
@@ -6636,8 +6844,8 @@
         <v>4</v>
       </c>
       <c r="D25" s="1">
-        <f t="shared" si="8"/>
-        <v>21</v>
+        <f t="shared" si="11"/>
+        <v>22</v>
       </c>
       <c r="E25" t="s">
         <v>59</v>
@@ -6722,8 +6930,11 @@
       <c r="BJ25" s="53" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK25" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>52</v>
       </c>
@@ -6731,7 +6942,7 @@
         <v>4</v>
       </c>
       <c r="D26" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="E26" t="s">
@@ -6800,8 +7011,11 @@
       <c r="BH26" s="31"/>
       <c r="BI26" s="31"/>
       <c r="BJ26" s="31"/>
-    </row>
-    <row r="27" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK26" s="48"/>
+      <c r="BL26" s="37"/>
+      <c r="BM26" s="37"/>
+    </row>
+    <row r="27" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>61</v>
       </c>
@@ -6809,7 +7023,7 @@
         <v>4</v>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="E27" t="s">
@@ -6872,8 +7086,9 @@
       <c r="BH27" s="31"/>
       <c r="BI27" s="31"/>
       <c r="BJ27" s="31"/>
-    </row>
-    <row r="28" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK27" s="48"/>
+    </row>
+    <row r="28" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>64</v>
       </c>
@@ -6881,8 +7096,8 @@
         <v>4</v>
       </c>
       <c r="D28" s="1">
-        <f t="shared" si="8"/>
-        <v>21</v>
+        <f t="shared" si="11"/>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
         <v>65</v>
@@ -6967,8 +7182,11 @@
       <c r="BH28" s="31"/>
       <c r="BI28" s="31"/>
       <c r="BJ28" s="31"/>
-    </row>
-    <row r="29" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK28" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>67</v>
       </c>
@@ -6976,7 +7194,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="E29" t="s">
@@ -7037,7 +7255,7 @@
       <c r="BI29" s="31"/>
       <c r="BJ29" s="31"/>
     </row>
-    <row r="30" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>70</v>
       </c>
@@ -7045,8 +7263,8 @@
         <v>4</v>
       </c>
       <c r="D30" s="1">
-        <f t="shared" si="8"/>
-        <v>14</v>
+        <f t="shared" si="11"/>
+        <v>15</v>
       </c>
       <c r="E30" t="s">
         <v>71</v>
@@ -7114,8 +7332,11 @@
       <c r="BJ30" s="53" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="31" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK30" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>73</v>
       </c>
@@ -7123,8 +7344,8 @@
         <v>4</v>
       </c>
       <c r="D31" s="1">
-        <f t="shared" si="8"/>
-        <v>14</v>
+        <f t="shared" si="11"/>
+        <v>15</v>
       </c>
       <c r="E31" t="s">
         <v>74</v>
@@ -7192,8 +7413,11 @@
       <c r="BJ31" s="53" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="32" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK31" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>79</v>
       </c>
@@ -7201,8 +7425,8 @@
         <v>6</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" si="8"/>
-        <v>20</v>
+        <f t="shared" si="11"/>
+        <v>23</v>
       </c>
       <c r="E32" t="s">
         <v>80</v>
@@ -7288,8 +7512,17 @@
       <c r="BH32" s="31"/>
       <c r="BI32" s="31"/>
       <c r="BJ32" s="31"/>
-    </row>
-    <row r="33" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BL32" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM32" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN32" s="67" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>76</v>
       </c>
@@ -7297,7 +7530,7 @@
         <v>6</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>7</v>
       </c>
       <c r="E33" t="s">
@@ -7348,7 +7581,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>82</v>
       </c>
@@ -7356,7 +7589,7 @@
         <v>4</v>
       </c>
       <c r="D34" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>7</v>
       </c>
       <c r="E34" t="s">
@@ -7407,7 +7640,7 @@
       <c r="BI34" s="31"/>
       <c r="BJ34" s="31"/>
     </row>
-    <row r="35" spans="2:62" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B35" s="2" t="s">
         <v>795</v>
       </c>
@@ -7415,7 +7648,7 @@
         <v>4</v>
       </c>
       <c r="D35" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>4</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -7461,7 +7694,7 @@
       <c r="BI35" s="31"/>
       <c r="BJ35" s="31"/>
     </row>
-    <row r="36" spans="2:62" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>85</v>
       </c>
@@ -7469,8 +7702,8 @@
         <v>2</v>
       </c>
       <c r="D36" s="1">
-        <f t="shared" si="8"/>
-        <v>9</v>
+        <f t="shared" si="11"/>
+        <v>10</v>
       </c>
       <c r="E36" t="s">
         <v>86</v>
@@ -7525,8 +7758,11 @@
       <c r="BH36" s="31"/>
       <c r="BI36" s="31"/>
       <c r="BJ36" s="31"/>
-    </row>
-    <row r="37" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BK36" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>88</v>
       </c>
@@ -7534,8 +7770,8 @@
         <v>2</v>
       </c>
       <c r="D37" s="1">
-        <f t="shared" si="8"/>
-        <v>9</v>
+        <f t="shared" si="11"/>
+        <v>10</v>
       </c>
       <c r="E37" t="s">
         <v>89</v>
@@ -7590,8 +7826,11 @@
       <c r="BH37" s="31"/>
       <c r="BI37" s="31"/>
       <c r="BJ37" s="31"/>
-    </row>
-    <row r="38" spans="2:62" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK37" s="64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="2:66" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>91</v>
       </c>
@@ -7599,8 +7838,8 @@
         <v>4</v>
       </c>
       <c r="D38" s="1">
-        <f t="shared" si="8"/>
-        <v>21</v>
+        <f t="shared" si="11"/>
+        <v>24</v>
       </c>
       <c r="E38" t="s">
         <v>92</v>
@@ -7687,8 +7926,17 @@
       </c>
       <c r="BI38" s="31"/>
       <c r="BJ38" s="31"/>
-    </row>
-    <row r="39" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BK38" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL38" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM38" s="108" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>94</v>
       </c>
@@ -7696,8 +7944,8 @@
         <v>4</v>
       </c>
       <c r="D39" s="1">
-        <f t="shared" si="8"/>
-        <v>24</v>
+        <f t="shared" si="11"/>
+        <v>27</v>
       </c>
       <c r="E39" t="s">
         <v>95</v>
@@ -7791,8 +8039,17 @@
       <c r="BH39" s="31"/>
       <c r="BI39" s="31"/>
       <c r="BJ39" s="31"/>
-    </row>
-    <row r="40" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BK39" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL39" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM39" s="108" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>100</v>
       </c>
@@ -7800,8 +8057,8 @@
         <v>4</v>
       </c>
       <c r="D40" s="1">
-        <f t="shared" si="8"/>
-        <v>15</v>
+        <f t="shared" si="11"/>
+        <v>18</v>
       </c>
       <c r="E40" t="s">
         <v>101</v>
@@ -7874,8 +8131,17 @@
       <c r="BH40" s="31"/>
       <c r="BI40" s="31"/>
       <c r="BJ40" s="31"/>
-    </row>
-    <row r="41" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BL40" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM40" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN40" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>103</v>
       </c>
@@ -7883,8 +8149,8 @@
         <v>4</v>
       </c>
       <c r="D41" s="1">
-        <f t="shared" si="8"/>
-        <v>15</v>
+        <f t="shared" si="11"/>
+        <v>18</v>
       </c>
       <c r="E41" t="s">
         <v>104</v>
@@ -7957,8 +8223,17 @@
       <c r="BH41" s="31"/>
       <c r="BI41" s="31"/>
       <c r="BJ41" s="31"/>
-    </row>
-    <row r="42" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BL41" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM41" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN41" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>97</v>
       </c>
@@ -7966,8 +8241,8 @@
         <v>6</v>
       </c>
       <c r="D42" s="1">
-        <f t="shared" si="8"/>
-        <v>15</v>
+        <f t="shared" si="11"/>
+        <v>17</v>
       </c>
       <c r="E42" t="s">
         <v>98</v>
@@ -8038,8 +8313,14 @@
       <c r="BH42" s="31"/>
       <c r="BI42" s="31"/>
       <c r="BJ42" s="31"/>
-    </row>
-    <row r="43" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BM42" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN42" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>106</v>
       </c>
@@ -8047,8 +8328,8 @@
         <v>6</v>
       </c>
       <c r="D43" s="1">
-        <f t="shared" si="8"/>
-        <v>12</v>
+        <f t="shared" si="11"/>
+        <v>14</v>
       </c>
       <c r="E43" t="s">
         <v>107</v>
@@ -8112,8 +8393,14 @@
       <c r="BH43" s="31"/>
       <c r="BI43" s="31"/>
       <c r="BJ43" s="31"/>
-    </row>
-    <row r="44" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BM43" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN43" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>109</v>
       </c>
@@ -8121,8 +8408,8 @@
         <v>4</v>
       </c>
       <c r="D44" s="1">
-        <f t="shared" si="8"/>
-        <v>15</v>
+        <f t="shared" si="11"/>
+        <v>17</v>
       </c>
       <c r="E44" t="s">
         <v>110</v>
@@ -8193,8 +8480,14 @@
       <c r="BH44" s="31"/>
       <c r="BI44" s="31"/>
       <c r="BJ44" s="31"/>
-    </row>
-    <row r="45" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BM44" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN44" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>112</v>
       </c>
@@ -8202,8 +8495,8 @@
         <v>6</v>
       </c>
       <c r="D45" s="1">
-        <f t="shared" si="8"/>
-        <v>9</v>
+        <f t="shared" si="11"/>
+        <v>11</v>
       </c>
       <c r="E45" t="s">
         <v>113</v>
@@ -8260,8 +8553,14 @@
       <c r="BH45" s="31"/>
       <c r="BI45" s="31"/>
       <c r="BJ45" s="31"/>
-    </row>
-    <row r="46" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BM45" s="108" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN45" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>115</v>
       </c>
@@ -8269,8 +8568,8 @@
         <v>6</v>
       </c>
       <c r="D46" s="1">
-        <f t="shared" si="8"/>
-        <v>9</v>
+        <f t="shared" si="11"/>
+        <v>10</v>
       </c>
       <c r="E46" t="s">
         <v>116</v>
@@ -8325,8 +8624,11 @@
       <c r="BJ46" s="53" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="47" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BN46" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>118</v>
       </c>
@@ -8334,8 +8636,8 @@
         <v>4</v>
       </c>
       <c r="D47" s="1">
-        <f t="shared" si="8"/>
-        <v>6</v>
+        <f t="shared" si="11"/>
+        <v>7</v>
       </c>
       <c r="E47" t="s">
         <v>119</v>
@@ -8383,8 +8685,11 @@
       <c r="BH47" s="31"/>
       <c r="BI47" s="31"/>
       <c r="BJ47" s="31"/>
-    </row>
-    <row r="48" spans="2:62" x14ac:dyDescent="0.25">
+      <c r="BN47" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="2:66" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>121</v>
       </c>
@@ -8392,8 +8697,8 @@
         <v>4</v>
       </c>
       <c r="D48" s="1">
-        <f t="shared" si="8"/>
-        <v>6</v>
+        <f t="shared" si="11"/>
+        <v>7</v>
       </c>
       <c r="E48" t="s">
         <v>122</v>
@@ -8441,8 +8746,11 @@
       <c r="BH48" s="31"/>
       <c r="BI48" s="31"/>
       <c r="BJ48" s="31"/>
-    </row>
-    <row r="49" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN48" s="68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
         <v>797</v>
       </c>
@@ -8450,7 +8758,7 @@
         <v>4</v>
       </c>
       <c r="D49" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="E49" s="2" t="s">
@@ -8487,7 +8795,7 @@
       <c r="BI49" s="31"/>
       <c r="BJ49" s="31"/>
     </row>
-    <row r="50" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>133</v>
       </c>
@@ -8495,7 +8803,7 @@
         <v>6</v>
       </c>
       <c r="D50" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>9</v>
       </c>
       <c r="E50" t="s">
@@ -8550,7 +8858,7 @@
       <c r="BI50" s="31"/>
       <c r="BJ50" s="31"/>
     </row>
-    <row r="51" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>136</v>
       </c>
@@ -8558,7 +8866,7 @@
         <v>6</v>
       </c>
       <c r="D51" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>27</v>
       </c>
       <c r="E51" t="s">
@@ -8657,8 +8965,9 @@
         <v>24</v>
       </c>
       <c r="BJ51" s="31"/>
-    </row>
-    <row r="52" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN51" s="37"/>
+    </row>
+    <row r="52" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>139</v>
       </c>
@@ -8666,7 +8975,7 @@
         <v>6</v>
       </c>
       <c r="D52" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>27</v>
       </c>
       <c r="E52" t="s">
@@ -8763,7 +9072,7 @@
       </c>
       <c r="BJ52" s="31"/>
     </row>
-    <row r="53" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>142</v>
       </c>
@@ -8771,7 +9080,7 @@
         <v>6</v>
       </c>
       <c r="D53" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>27</v>
       </c>
       <c r="E53" t="s">
@@ -8868,7 +9177,7 @@
       </c>
       <c r="BJ53" s="31"/>
     </row>
-    <row r="54" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>124</v>
       </c>
@@ -8876,7 +9185,7 @@
         <v>6</v>
       </c>
       <c r="D54" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>15</v>
       </c>
       <c r="E54" t="s">
@@ -8950,8 +9259,10 @@
         <v>24</v>
       </c>
       <c r="BJ54" s="31"/>
-    </row>
-    <row r="55" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL54" s="37"/>
+      <c r="BM54" s="37"/>
+    </row>
+    <row r="55" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>127</v>
       </c>
@@ -8959,7 +9270,7 @@
         <v>6</v>
       </c>
       <c r="D55" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>18</v>
       </c>
       <c r="E55" t="s">
@@ -9040,8 +9351,10 @@
       </c>
       <c r="BI55" s="31"/>
       <c r="BJ55" s="31"/>
-    </row>
-    <row r="56" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL55" s="37"/>
+      <c r="BM55" s="37"/>
+    </row>
+    <row r="56" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>130</v>
       </c>
@@ -9049,7 +9362,7 @@
         <v>6</v>
       </c>
       <c r="D56" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>18</v>
       </c>
       <c r="E56" t="s">
@@ -9130,8 +9443,10 @@
       </c>
       <c r="BI56" s="31"/>
       <c r="BJ56" s="31"/>
-    </row>
-    <row r="57" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL56" s="37"/>
+      <c r="BM56" s="37"/>
+    </row>
+    <row r="57" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>145</v>
       </c>
@@ -9139,7 +9454,7 @@
         <v>6</v>
       </c>
       <c r="D57" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>9</v>
       </c>
       <c r="E57" t="s">
@@ -9205,8 +9520,11 @@
       <c r="BH57" s="36"/>
       <c r="BI57" s="36"/>
       <c r="BJ57" s="36"/>
-    </row>
-    <row r="58" spans="1:62" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK57" s="48"/>
+      <c r="BL57" s="37"/>
+      <c r="BM57" s="37"/>
+    </row>
+    <row r="58" spans="1:66" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="9"/>
       <c r="C58" s="17"/>
       <c r="D58" s="9"/>
@@ -9248,8 +9566,12 @@
       <c r="AX58" s="32"/>
       <c r="AY58" s="82"/>
       <c r="BB58" s="83"/>
-    </row>
-    <row r="59" spans="1:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BK58" s="49"/>
+      <c r="BL58" s="32"/>
+      <c r="BM58" s="32"/>
+      <c r="BN58" s="32"/>
+    </row>
+    <row r="59" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="114" t="s">
         <v>148</v>
       </c>
@@ -9260,7 +9582,7 @@
         <v>4</v>
       </c>
       <c r="D59" s="5">
-        <f t="shared" ref="D59:D106" si="9">COUNTIF(G59:AAJ59,"✅")+COUNTIF(G59:AAJ59,"✔️")</f>
+        <f t="shared" ref="D59:D106" si="12">COUNTIF(G59:AAN59,"✅")+COUNTIF(G59:AAN59,"✔️")</f>
         <v>1</v>
       </c>
       <c r="E59" s="2" t="s">
@@ -9297,7 +9619,7 @@
       <c r="BI59" s="31"/>
       <c r="BJ59" s="63"/>
     </row>
-    <row r="60" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A60" s="114"/>
       <c r="B60" t="s">
         <v>149</v>
@@ -9306,8 +9628,8 @@
         <v>1</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E60" t="s">
         <v>150</v>
@@ -9387,8 +9709,14 @@
       </c>
       <c r="BI60" s="31"/>
       <c r="BJ60" s="63"/>
-    </row>
-    <row r="61" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK60" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL60" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A61" s="114"/>
       <c r="B61" t="s">
         <v>152</v>
@@ -9397,8 +9725,8 @@
         <v>1</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E61" t="s">
         <v>153</v>
@@ -9478,8 +9806,14 @@
       </c>
       <c r="BI61" s="31"/>
       <c r="BJ61" s="63"/>
-    </row>
-    <row r="62" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK61" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL61" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A62" s="114"/>
       <c r="B62" t="s">
         <v>155</v>
@@ -9488,8 +9822,8 @@
         <v>1</v>
       </c>
       <c r="D62" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E62" t="s">
         <v>156</v>
@@ -9569,8 +9903,14 @@
       </c>
       <c r="BI62" s="31"/>
       <c r="BJ62" s="63"/>
-    </row>
-    <row r="63" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK62" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL62" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A63" s="114"/>
       <c r="B63" t="s">
         <v>158</v>
@@ -9579,8 +9919,8 @@
         <v>1</v>
       </c>
       <c r="D63" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E63" t="s">
         <v>159</v>
@@ -9660,8 +10000,14 @@
       </c>
       <c r="BI63" s="31"/>
       <c r="BJ63" s="63"/>
-    </row>
-    <row r="64" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK63" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL63" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A64" s="114"/>
       <c r="B64" t="s">
         <v>161</v>
@@ -9670,8 +10016,8 @@
         <v>1</v>
       </c>
       <c r="D64" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E64" t="s">
         <v>162</v>
@@ -9751,8 +10097,14 @@
       </c>
       <c r="BI64" s="31"/>
       <c r="BJ64" s="63"/>
-    </row>
-    <row r="65" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK64" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL64" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A65" s="114"/>
       <c r="B65" t="s">
         <v>164</v>
@@ -9761,8 +10113,8 @@
         <v>1</v>
       </c>
       <c r="D65" s="1">
-        <f t="shared" si="9"/>
-        <v>20</v>
+        <f t="shared" si="12"/>
+        <v>22</v>
       </c>
       <c r="E65" t="s">
         <v>165</v>
@@ -9842,8 +10194,14 @@
       </c>
       <c r="BI65" s="31"/>
       <c r="BJ65" s="63"/>
-    </row>
-    <row r="66" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK65" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL65" s="75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A66" s="114"/>
       <c r="B66" t="s">
         <v>176</v>
@@ -9852,7 +10210,7 @@
         <v>4</v>
       </c>
       <c r="D66" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>9</v>
       </c>
       <c r="E66" t="s">
@@ -9908,8 +10266,9 @@
       <c r="BH66" s="31"/>
       <c r="BI66" s="31"/>
       <c r="BJ66" s="63"/>
-    </row>
-    <row r="67" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK66" s="51"/>
+    </row>
+    <row r="67" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A67" s="114"/>
       <c r="B67" t="s">
         <v>173</v>
@@ -9918,7 +10277,7 @@
         <v>4</v>
       </c>
       <c r="D67" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>13</v>
       </c>
       <c r="E67" t="s">
@@ -9982,8 +10341,9 @@
         <v>24</v>
       </c>
       <c r="BJ67" s="63"/>
-    </row>
-    <row r="68" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK67" s="51"/>
+    </row>
+    <row r="68" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A68" s="114"/>
       <c r="B68" t="s">
         <v>200</v>
@@ -9992,7 +10352,7 @@
         <v>6</v>
       </c>
       <c r="D68" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>8</v>
       </c>
       <c r="E68" t="s">
@@ -10039,8 +10399,10 @@
       </c>
       <c r="BG68" s="62"/>
       <c r="BJ68" s="63"/>
-    </row>
-    <row r="69" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL68"/>
+      <c r="BM68"/>
+    </row>
+    <row r="69" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A69" s="114"/>
       <c r="B69" t="s">
         <v>221</v>
@@ -10049,8 +10411,8 @@
         <v>6</v>
       </c>
       <c r="D69" s="1">
-        <f t="shared" si="9"/>
-        <v>7</v>
+        <f t="shared" si="12"/>
+        <v>8</v>
       </c>
       <c r="E69" t="s">
         <v>222</v>
@@ -10099,8 +10461,11 @@
       <c r="BH69" s="31"/>
       <c r="BI69" s="31"/>
       <c r="BJ69" s="52"/>
-    </row>
-    <row r="70" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN69" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A70" s="114"/>
       <c r="B70" t="s">
         <v>167</v>
@@ -10109,8 +10474,8 @@
         <v>1</v>
       </c>
       <c r="D70" s="1">
-        <f t="shared" si="9"/>
-        <v>19</v>
+        <f t="shared" si="12"/>
+        <v>21</v>
       </c>
       <c r="E70" t="s">
         <v>168</v>
@@ -10187,8 +10552,14 @@
       </c>
       <c r="BI70" s="31"/>
       <c r="BJ70" s="63"/>
-    </row>
-    <row r="71" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK70" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL70" s="102" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A71" s="114"/>
       <c r="B71" t="s">
         <v>257</v>
@@ -10197,8 +10568,8 @@
         <v>6</v>
       </c>
       <c r="D71" s="1">
-        <f t="shared" si="9"/>
-        <v>14</v>
+        <f t="shared" si="12"/>
+        <v>17</v>
       </c>
       <c r="E71" t="s">
         <v>258</v>
@@ -10264,8 +10635,18 @@
       <c r="BH71" s="31"/>
       <c r="BI71" s="31"/>
       <c r="BJ71" s="52"/>
-    </row>
-    <row r="72" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK71" s="51"/>
+      <c r="BL71" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM71" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN71" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A72" s="114"/>
       <c r="B72" t="s">
         <v>260</v>
@@ -10274,8 +10655,8 @@
         <v>6</v>
       </c>
       <c r="D72" s="1">
-        <f t="shared" si="9"/>
-        <v>14</v>
+        <f t="shared" si="12"/>
+        <v>17</v>
       </c>
       <c r="E72" t="s">
         <v>261</v>
@@ -10341,8 +10722,18 @@
       <c r="BH72" s="31"/>
       <c r="BI72" s="31"/>
       <c r="BJ72" s="52"/>
-    </row>
-    <row r="73" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK72" s="51"/>
+      <c r="BL72" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM72" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN72" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A73" s="114"/>
       <c r="B73" t="s">
         <v>266</v>
@@ -10351,8 +10742,8 @@
         <v>6</v>
       </c>
       <c r="D73" s="1">
-        <f t="shared" si="9"/>
-        <v>14</v>
+        <f t="shared" si="12"/>
+        <v>17</v>
       </c>
       <c r="E73" t="s">
         <v>267</v>
@@ -10418,8 +10809,18 @@
       <c r="BH73" s="31"/>
       <c r="BI73" s="31"/>
       <c r="BJ73" s="52"/>
-    </row>
-    <row r="74" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK73" s="51"/>
+      <c r="BL73" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM73" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN73" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A74" s="114"/>
       <c r="B74" t="s">
         <v>263</v>
@@ -10428,8 +10829,8 @@
         <v>6</v>
       </c>
       <c r="D74" s="1">
-        <f t="shared" si="9"/>
-        <v>5</v>
+        <f t="shared" si="12"/>
+        <v>6</v>
       </c>
       <c r="E74" t="s">
         <v>264</v>
@@ -10464,8 +10865,14 @@
       </c>
       <c r="BG74" s="51"/>
       <c r="BJ74" s="52"/>
-    </row>
-    <row r="75" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK74" s="51"/>
+      <c r="BL74"/>
+      <c r="BM74"/>
+      <c r="BN74" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A75" s="114"/>
       <c r="B75" t="s">
         <v>269</v>
@@ -10474,8 +10881,8 @@
         <v>6</v>
       </c>
       <c r="D75" s="1">
-        <f t="shared" si="9"/>
-        <v>5</v>
+        <f t="shared" si="12"/>
+        <v>6</v>
       </c>
       <c r="E75" t="s">
         <v>270</v>
@@ -10510,8 +10917,14 @@
       </c>
       <c r="BG75" s="51"/>
       <c r="BJ75" s="52"/>
-    </row>
-    <row r="76" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK75" s="51"/>
+      <c r="BL75"/>
+      <c r="BM75"/>
+      <c r="BN75" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A76" s="114"/>
       <c r="B76" s="2" t="s">
         <v>811</v>
@@ -10520,7 +10933,7 @@
         <v>4</v>
       </c>
       <c r="D76" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>4</v>
       </c>
       <c r="E76" s="2" t="s">
@@ -10563,8 +10976,11 @@
       <c r="BH76" s="31"/>
       <c r="BI76" s="31"/>
       <c r="BJ76" s="52"/>
-    </row>
-    <row r="77" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL76"/>
+      <c r="BM76"/>
+      <c r="BN76"/>
+    </row>
+    <row r="77" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A77" s="114"/>
       <c r="B77" t="s">
         <v>239</v>
@@ -10573,8 +10989,8 @@
         <v>4</v>
       </c>
       <c r="D77" s="1">
-        <f t="shared" si="9"/>
-        <v>6</v>
+        <f t="shared" si="12"/>
+        <v>7</v>
       </c>
       <c r="E77" t="s">
         <v>240</v>
@@ -10612,8 +11028,14 @@
       </c>
       <c r="BG77" s="62"/>
       <c r="BJ77" s="52"/>
-    </row>
-    <row r="78" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK77" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL77"/>
+      <c r="BM77"/>
+      <c r="BN77"/>
+    </row>
+    <row r="78" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A78" s="114"/>
       <c r="B78" t="s">
         <v>242</v>
@@ -10622,8 +11044,8 @@
         <v>4</v>
       </c>
       <c r="D78" s="1">
-        <f t="shared" si="9"/>
-        <v>6</v>
+        <f t="shared" si="12"/>
+        <v>7</v>
       </c>
       <c r="E78" t="s">
         <v>243</v>
@@ -10661,8 +11083,14 @@
       </c>
       <c r="BG78" s="62"/>
       <c r="BJ78" s="52"/>
-    </row>
-    <row r="79" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK78" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL78"/>
+      <c r="BM78"/>
+      <c r="BN78"/>
+    </row>
+    <row r="79" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A79" s="114"/>
       <c r="B79" t="s">
         <v>185</v>
@@ -10671,7 +11099,7 @@
         <v>6</v>
       </c>
       <c r="D79" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>11</v>
       </c>
       <c r="E79" t="s">
@@ -10729,8 +11157,11 @@
         <v>24</v>
       </c>
       <c r="BJ79" s="52"/>
-    </row>
-    <row r="80" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL79"/>
+      <c r="BM79"/>
+      <c r="BN79"/>
+    </row>
+    <row r="80" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A80" s="114"/>
       <c r="B80" t="s">
         <v>233</v>
@@ -10739,7 +11170,7 @@
         <v>4</v>
       </c>
       <c r="D80" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>6</v>
       </c>
       <c r="E80" t="s">
@@ -10780,8 +11211,12 @@
       </c>
       <c r="BG80" s="62"/>
       <c r="BJ80" s="52"/>
-    </row>
-    <row r="81" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK80" s="51"/>
+      <c r="BL80"/>
+      <c r="BM80"/>
+      <c r="BN80"/>
+    </row>
+    <row r="81" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A81" s="114"/>
       <c r="B81" t="s">
         <v>251</v>
@@ -10790,7 +11225,7 @@
         <v>4</v>
       </c>
       <c r="D81" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>13</v>
       </c>
       <c r="E81" t="s">
@@ -10850,8 +11285,12 @@
         <v>24</v>
       </c>
       <c r="BJ81" s="52"/>
-    </row>
-    <row r="82" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK81" s="51"/>
+      <c r="BL81"/>
+      <c r="BM81"/>
+      <c r="BN81"/>
+    </row>
+    <row r="82" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A82" s="114"/>
       <c r="B82" t="s">
         <v>254</v>
@@ -10860,7 +11299,7 @@
         <v>6</v>
       </c>
       <c r="D82" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>13</v>
       </c>
       <c r="E82" t="s">
@@ -10918,8 +11357,12 @@
         <v>24</v>
       </c>
       <c r="BJ82" s="52"/>
-    </row>
-    <row r="83" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK82" s="51"/>
+      <c r="BL82"/>
+      <c r="BM82"/>
+      <c r="BN82"/>
+    </row>
+    <row r="83" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A83" s="114"/>
       <c r="B83" t="s">
         <v>248</v>
@@ -10928,7 +11371,7 @@
         <v>4</v>
       </c>
       <c r="D83" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>4</v>
       </c>
       <c r="E83" t="s">
@@ -10961,8 +11404,12 @@
       <c r="BJ83" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="84" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK83" s="51"/>
+      <c r="BL83"/>
+      <c r="BM83"/>
+      <c r="BN83"/>
+    </row>
+    <row r="84" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A84" s="114"/>
       <c r="B84" t="s">
         <v>197</v>
@@ -10971,8 +11418,8 @@
         <v>6</v>
       </c>
       <c r="D84" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>12</v>
       </c>
       <c r="E84" t="s">
         <v>198</v>
@@ -11018,8 +11465,15 @@
       <c r="BJ84" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="85" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL84" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM84" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN84"/>
+    </row>
+    <row r="85" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A85" s="114"/>
       <c r="B85" t="s">
         <v>215</v>
@@ -11028,7 +11482,7 @@
         <v>6</v>
       </c>
       <c r="D85" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>9</v>
       </c>
       <c r="E85" t="s">
@@ -11076,8 +11530,9 @@
       <c r="BJ85" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="86" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN85"/>
+    </row>
+    <row r="86" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A86" s="114"/>
       <c r="B86" t="s">
         <v>218</v>
@@ -11086,7 +11541,7 @@
         <v>6</v>
       </c>
       <c r="D86" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>9</v>
       </c>
       <c r="E86" t="s">
@@ -11134,8 +11589,9 @@
       <c r="BJ86" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="87" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN86"/>
+    </row>
+    <row r="87" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A87" s="114"/>
       <c r="B87" t="s">
         <v>274</v>
@@ -11144,7 +11600,7 @@
         <v>6</v>
       </c>
       <c r="D87" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="E87" t="s">
@@ -11180,8 +11636,12 @@
       <c r="BJ87" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="88" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK87" s="51"/>
+      <c r="BL87"/>
+      <c r="BM87"/>
+      <c r="BN87"/>
+    </row>
+    <row r="88" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A88" s="114"/>
       <c r="B88" s="2" t="s">
         <v>816</v>
@@ -11190,8 +11650,8 @@
         <v>4</v>
       </c>
       <c r="D88" s="5">
-        <f t="shared" si="9"/>
-        <v>8</v>
+        <f t="shared" si="12"/>
+        <v>4</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>812</v>
@@ -11219,18 +11679,10 @@
       <c r="AR88" s="31"/>
       <c r="AS88" s="31"/>
       <c r="AT88" s="52"/>
-      <c r="AU88" s="104" t="s">
-        <v>24</v>
-      </c>
-      <c r="AV88" s="115" t="s">
-        <v>24</v>
-      </c>
-      <c r="AW88" s="115" t="s">
-        <v>24</v>
-      </c>
-      <c r="AX88" s="115" t="s">
-        <v>24</v>
-      </c>
+      <c r="AU88" s="51"/>
+      <c r="AV88"/>
+      <c r="AW88"/>
+      <c r="AX88"/>
       <c r="AY88" s="62"/>
       <c r="AZ88" s="31"/>
       <c r="BA88" s="31"/>
@@ -11239,8 +11691,12 @@
       <c r="BH88" s="31"/>
       <c r="BI88" s="31"/>
       <c r="BJ88" s="52"/>
-    </row>
-    <row r="89" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK88" s="51"/>
+      <c r="BL88"/>
+      <c r="BM88"/>
+      <c r="BN88"/>
+    </row>
+    <row r="89" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A89" s="114"/>
       <c r="B89" t="s">
         <v>224</v>
@@ -11249,8 +11705,8 @@
         <v>6</v>
       </c>
       <c r="D89" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>12</v>
       </c>
       <c r="E89" t="s">
         <v>225</v>
@@ -11304,8 +11760,15 @@
       </c>
       <c r="BI89" s="31"/>
       <c r="BJ89" s="63"/>
-    </row>
-    <row r="90" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK89" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL89" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM89"/>
+    </row>
+    <row r="90" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A90" s="114"/>
       <c r="B90" t="s">
         <v>230</v>
@@ -11314,8 +11777,8 @@
         <v>4</v>
       </c>
       <c r="D90" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>12</v>
       </c>
       <c r="E90" t="s">
         <v>231</v>
@@ -11367,8 +11830,15 @@
         <v>24</v>
       </c>
       <c r="BJ90" s="63"/>
-    </row>
-    <row r="91" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK90" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL90" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM90"/>
+    </row>
+    <row r="91" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A91" s="114"/>
       <c r="B91" t="s">
         <v>188</v>
@@ -11377,8 +11847,8 @@
         <v>4</v>
       </c>
       <c r="D91" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>13</v>
       </c>
       <c r="E91" t="s">
         <v>189</v>
@@ -11428,8 +11898,17 @@
       <c r="BF91" s="31"/>
       <c r="BG91" s="62"/>
       <c r="BJ91" s="63"/>
-    </row>
-    <row r="92" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK91" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL91" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM91" s="107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="92" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A92" s="114"/>
       <c r="B92" t="s">
         <v>179</v>
@@ -11438,8 +11917,8 @@
         <v>6</v>
       </c>
       <c r="D92" s="1">
-        <f>COUNTIF(G92:AAJ92,"✅")+COUNTIF(G92:AAJ92,"✔️")</f>
-        <v>8</v>
+        <f>COUNTIF(G92:AAN92,"✅")+COUNTIF(G92:AAN92,"✔️")</f>
+        <v>10</v>
       </c>
       <c r="E92" t="s">
         <v>180</v>
@@ -11479,8 +11958,15 @@
         <v>24</v>
       </c>
       <c r="BJ92" s="52"/>
-    </row>
-    <row r="93" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK92" s="51"/>
+      <c r="BL92" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM92" s="107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="93" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A93" s="114"/>
       <c r="B93" t="s">
         <v>191</v>
@@ -11489,8 +11975,8 @@
         <v>4</v>
       </c>
       <c r="D93" s="1">
-        <f t="shared" si="9"/>
-        <v>14</v>
+        <f t="shared" si="12"/>
+        <v>16</v>
       </c>
       <c r="E93" t="s">
         <v>192</v>
@@ -11550,8 +12036,14 @@
         <v>24</v>
       </c>
       <c r="BJ93" s="63"/>
-    </row>
-    <row r="94" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL93" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM93" s="107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A94" s="114"/>
       <c r="B94" t="s">
         <v>203</v>
@@ -11560,8 +12052,8 @@
         <v>6</v>
       </c>
       <c r="D94" s="1">
-        <f t="shared" si="9"/>
-        <v>12</v>
+        <f t="shared" si="12"/>
+        <v>15</v>
       </c>
       <c r="E94" t="s">
         <v>204</v>
@@ -11613,8 +12105,17 @@
       </c>
       <c r="BG94" s="62"/>
       <c r="BJ94" s="52"/>
-    </row>
-    <row r="95" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BL94" s="75" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM94" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN94" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A95" s="114"/>
       <c r="B95" t="s">
         <v>277</v>
@@ -11623,8 +12124,8 @@
         <v>6</v>
       </c>
       <c r="D95" s="1">
-        <f t="shared" si="9"/>
-        <v>8</v>
+        <f t="shared" si="12"/>
+        <v>10</v>
       </c>
       <c r="E95" t="s">
         <v>278</v>
@@ -11666,8 +12167,15 @@
       </c>
       <c r="BG95" s="51"/>
       <c r="BJ95" s="52"/>
-    </row>
-    <row r="96" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK95" s="51"/>
+      <c r="BM95" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN95" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A96" s="114"/>
       <c r="B96" t="s">
         <v>245</v>
@@ -11676,8 +12184,8 @@
         <v>6</v>
       </c>
       <c r="D96" s="1">
-        <f t="shared" si="9"/>
-        <v>14</v>
+        <f t="shared" si="12"/>
+        <v>16</v>
       </c>
       <c r="E96" t="s">
         <v>246</v>
@@ -11735,8 +12243,14 @@
         <v>24</v>
       </c>
       <c r="BJ96" s="52"/>
-    </row>
-    <row r="97" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BM96" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN96" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="97" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A97" s="114"/>
       <c r="B97" t="s">
         <v>206</v>
@@ -11745,8 +12259,8 @@
         <v>6</v>
       </c>
       <c r="D97" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>11</v>
       </c>
       <c r="E97" t="s">
         <v>207</v>
@@ -11798,8 +12312,11 @@
       <c r="BJ97" s="77" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="98" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN97" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A98" s="114"/>
       <c r="B98" t="s">
         <v>209</v>
@@ -11808,8 +12325,8 @@
         <v>6</v>
       </c>
       <c r="D98" s="1">
-        <f t="shared" si="9"/>
-        <v>10</v>
+        <f t="shared" si="12"/>
+        <v>11</v>
       </c>
       <c r="E98" t="s">
         <v>210</v>
@@ -11861,8 +12378,11 @@
       <c r="BJ98" s="77" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="99" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN98" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A99" s="114"/>
       <c r="B99" t="s">
         <v>212</v>
@@ -11871,8 +12391,8 @@
         <v>6</v>
       </c>
       <c r="D99" s="1">
-        <f t="shared" si="9"/>
-        <v>6</v>
+        <f t="shared" si="12"/>
+        <v>7</v>
       </c>
       <c r="E99" t="s">
         <v>213</v>
@@ -11918,8 +12438,11 @@
       <c r="BJ99" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="100" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BN99" s="77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A100" s="114"/>
       <c r="B100" s="2" t="s">
         <v>817</v>
@@ -11928,8 +12451,8 @@
         <v>4</v>
       </c>
       <c r="D100" s="5">
-        <f t="shared" si="9"/>
-        <v>8</v>
+        <f t="shared" si="12"/>
+        <v>4</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>815</v>
@@ -11959,18 +12482,9 @@
       <c r="AS100" s="31"/>
       <c r="AT100" s="52"/>
       <c r="AU100" s="51"/>
-      <c r="AY100" s="104" t="s">
-        <v>24</v>
-      </c>
-      <c r="AZ100" s="115" t="s">
-        <v>24</v>
-      </c>
-      <c r="BA100" s="115" t="s">
-        <v>24</v>
-      </c>
-      <c r="BB100" s="115" t="s">
-        <v>24</v>
-      </c>
+      <c r="AY100" s="62"/>
+      <c r="AZ100" s="31"/>
+      <c r="BA100" s="31"/>
       <c r="BC100" s="51"/>
       <c r="BD100" s="31"/>
       <c r="BE100" s="31"/>
@@ -11979,8 +12493,9 @@
       <c r="BH100" s="31"/>
       <c r="BI100" s="31"/>
       <c r="BJ100" s="52"/>
-    </row>
-    <row r="101" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK100" s="51"/>
+    </row>
+    <row r="101" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A101" s="114"/>
       <c r="B101" t="s">
         <v>182</v>
@@ -11989,7 +12504,7 @@
         <v>6</v>
       </c>
       <c r="D101" s="1">
-        <f>COUNTIF(G101:AAJ101,"✅")+COUNTIF(G101:AAJ101,"✔️")</f>
+        <f>COUNTIF(G101:AAN101,"✅")+COUNTIF(G101:AAN101,"✔️")</f>
         <v>8</v>
       </c>
       <c r="E101" t="s">
@@ -12040,8 +12555,11 @@
       <c r="BJ101" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="102" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK101" s="51"/>
+      <c r="BL101"/>
+      <c r="BM101"/>
+    </row>
+    <row r="102" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A102" s="114"/>
       <c r="B102" t="s">
         <v>227</v>
@@ -12050,7 +12568,7 @@
         <v>6</v>
       </c>
       <c r="D102" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>12</v>
       </c>
       <c r="E102" t="s">
@@ -12109,8 +12627,9 @@
       <c r="BH102" s="31"/>
       <c r="BI102" s="31"/>
       <c r="BJ102" s="63"/>
-    </row>
-    <row r="103" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK102" s="51"/>
+    </row>
+    <row r="103" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A103" s="114"/>
       <c r="B103" t="s">
         <v>170</v>
@@ -12119,7 +12638,7 @@
         <v>6</v>
       </c>
       <c r="D103" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>10</v>
       </c>
       <c r="E103" t="s">
@@ -12174,8 +12693,9 @@
       </c>
       <c r="BI103" s="31"/>
       <c r="BJ103" s="63"/>
-    </row>
-    <row r="104" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK103" s="51"/>
+    </row>
+    <row r="104" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A104" s="114"/>
       <c r="B104" t="s">
         <v>236</v>
@@ -12184,7 +12704,7 @@
         <v>4</v>
       </c>
       <c r="D104" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>10</v>
       </c>
       <c r="E104" t="s">
@@ -12237,8 +12757,12 @@
         <v>24</v>
       </c>
       <c r="BJ104" s="52"/>
-    </row>
-    <row r="105" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK104" s="51"/>
+      <c r="BL104"/>
+      <c r="BM104"/>
+      <c r="BN104"/>
+    </row>
+    <row r="105" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A105" s="114"/>
       <c r="B105" t="s">
         <v>272</v>
@@ -12247,7 +12771,7 @@
         <v>6</v>
       </c>
       <c r="D105" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>12</v>
       </c>
       <c r="E105" t="s">
@@ -12306,8 +12830,11 @@
       <c r="BJ105" s="81" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="106" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="BK105" s="51"/>
+      <c r="BL105"/>
+      <c r="BM105"/>
+    </row>
+    <row r="106" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A106" s="114"/>
       <c r="B106" t="s">
         <v>194</v>
@@ -12316,7 +12843,7 @@
         <v>6</v>
       </c>
       <c r="D106" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>12</v>
       </c>
       <c r="E106" t="s">
@@ -12373,8 +12900,10 @@
         <v>24</v>
       </c>
       <c r="BJ106" s="52"/>
-    </row>
-    <row r="107" spans="1:62" s="8" customFormat="1" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BL106"/>
+      <c r="BM106"/>
+    </row>
+    <row r="107" spans="1:66" s="8" customFormat="1" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C107" s="18"/>
       <c r="D107" s="10"/>
       <c r="G107" s="50"/>
@@ -12413,9 +12942,13 @@
       <c r="AX107" s="33"/>
       <c r="AY107" s="84"/>
       <c r="BB107" s="83"/>
-    </row>
-    <row r="108" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="A108" s="164" t="s">
+      <c r="BK107" s="66"/>
+      <c r="BL107" s="33"/>
+      <c r="BM107" s="33"/>
+      <c r="BN107" s="33"/>
+    </row>
+    <row r="108" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A108" s="139" t="s">
         <v>775</v>
       </c>
       <c r="B108" t="s">
@@ -12425,7 +12958,7 @@
         <v>6</v>
       </c>
       <c r="D108" s="1">
-        <f t="shared" ref="D108:D115" si="10">COUNTIF(G108:AAJ108,"✅")+COUNTIF(G108:AAJ108,"✔️")</f>
+        <f t="shared" ref="D108:D115" si="13">COUNTIF(G108:AAN108,"✅")+COUNTIF(G108:AAN108,"✔️")</f>
         <v>8</v>
       </c>
       <c r="E108" t="s">
@@ -12471,8 +13004,8 @@
       <c r="BA108" s="31"/>
       <c r="BB108" s="31"/>
     </row>
-    <row r="109" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="A109" s="164"/>
+    <row r="109" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A109" s="139"/>
       <c r="B109" t="s">
         <v>284</v>
       </c>
@@ -12480,7 +13013,7 @@
         <v>6</v>
       </c>
       <c r="D109" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="E109" t="s">
@@ -12514,8 +13047,8 @@
       <c r="BA109" s="31"/>
       <c r="BB109" s="31"/>
     </row>
-    <row r="110" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="A110" s="164"/>
+    <row r="110" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A110" s="139"/>
       <c r="B110" t="s">
         <v>287</v>
       </c>
@@ -12523,7 +13056,7 @@
         <v>6</v>
       </c>
       <c r="D110" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="E110" t="s">
@@ -12557,8 +13090,8 @@
       <c r="BA110" s="31"/>
       <c r="BB110" s="31"/>
     </row>
-    <row r="111" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="A111" s="164"/>
+    <row r="111" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A111" s="139"/>
       <c r="B111" t="s">
         <v>290</v>
       </c>
@@ -12566,7 +13099,7 @@
         <v>6</v>
       </c>
       <c r="D111" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="E111" t="s">
@@ -12600,8 +13133,8 @@
       <c r="BA111" s="31"/>
       <c r="BB111" s="31"/>
     </row>
-    <row r="112" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="A112" s="164"/>
+    <row r="112" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A112" s="139"/>
       <c r="B112" t="s">
         <v>293</v>
       </c>
@@ -12609,7 +13142,7 @@
         <v>6</v>
       </c>
       <c r="D112" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="E112" t="s">
@@ -12643,8 +13176,8 @@
       <c r="BA112" s="31"/>
       <c r="BB112" s="31"/>
     </row>
-    <row r="113" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A113" s="164"/>
+    <row r="113" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A113" s="139"/>
       <c r="B113" t="s">
         <v>296</v>
       </c>
@@ -12652,7 +13185,7 @@
         <v>6</v>
       </c>
       <c r="D113" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="E113" t="s">
@@ -12686,8 +13219,8 @@
       <c r="BA113" s="31"/>
       <c r="BB113" s="31"/>
     </row>
-    <row r="114" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A114" s="164"/>
+    <row r="114" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A114" s="139"/>
       <c r="B114" t="s">
         <v>299</v>
       </c>
@@ -12695,7 +13228,7 @@
         <v>6</v>
       </c>
       <c r="D114" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="E114" t="s">
@@ -12732,8 +13265,8 @@
       <c r="BA114" s="31"/>
       <c r="BB114" s="31"/>
     </row>
-    <row r="115" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A115" s="164"/>
+    <row r="115" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A115" s="139"/>
       <c r="B115" t="s">
         <v>302</v>
       </c>
@@ -12741,7 +13274,7 @@
         <v>6</v>
       </c>
       <c r="D115" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>2</v>
       </c>
       <c r="E115" t="s">
@@ -12769,7 +13302,7 @@
       <c r="BA115" s="31"/>
       <c r="BB115" s="31"/>
     </row>
-    <row r="116" spans="1:61" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:66" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C116" s="18"/>
       <c r="D116" s="10"/>
       <c r="G116" s="50"/>
@@ -12808,17 +13341,21 @@
       <c r="AX116" s="33"/>
       <c r="AY116" s="84"/>
       <c r="BB116" s="83"/>
-    </row>
-    <row r="117" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A117" s="165" t="s">
+      <c r="BK116" s="66"/>
+      <c r="BL116" s="33"/>
+      <c r="BM116" s="33"/>
+      <c r="BN116" s="33"/>
+    </row>
+    <row r="117" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A117" s="140" t="s">
         <v>280</v>
       </c>
       <c r="B117" t="s">
         <v>776</v>
       </c>
       <c r="D117" s="1">
-        <f t="shared" ref="D117:D133" si="11">COUNTIF(G117:AAJ117,"✅")+COUNTIF(G117:AAJ117,"✔️")</f>
-        <v>18</v>
+        <f t="shared" ref="D117:D133" si="14">COUNTIF(G117:AAN117,"✅")+COUNTIF(G117:AAN117,"✔️")</f>
+        <v>21</v>
       </c>
       <c r="E117" t="s">
         <v>306</v>
@@ -12880,15 +13417,24 @@
       <c r="BI117" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="118" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A118" s="165"/>
+      <c r="BK117" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL117" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM117" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="118" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A118" s="140"/>
       <c r="B118" t="s">
         <v>777</v>
       </c>
       <c r="D118" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E118" t="s">
         <v>309</v>
@@ -12950,15 +13496,24 @@
       <c r="BI118" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="119" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A119" s="165"/>
+      <c r="BK118" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL118" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM118" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A119" s="140"/>
       <c r="B119" t="s">
         <v>778</v>
       </c>
       <c r="D119" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E119" t="s">
         <v>312</v>
@@ -13020,15 +13575,24 @@
       <c r="BI119" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="120" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A120" s="165"/>
+      <c r="BK119" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL119" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM119" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="120" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A120" s="140"/>
       <c r="B120" t="s">
         <v>779</v>
       </c>
       <c r="D120" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E120" t="s">
         <v>315</v>
@@ -13090,15 +13654,24 @@
       <c r="BI120" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="121" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A121" s="165"/>
+      <c r="BK120" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL120" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM120" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="121" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A121" s="140"/>
       <c r="B121" t="s">
         <v>780</v>
       </c>
       <c r="D121" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E121" t="s">
         <v>318</v>
@@ -13160,15 +13733,24 @@
       <c r="BI121" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="122" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A122" s="165"/>
+      <c r="BK121" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL121" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM121" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="122" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A122" s="140"/>
       <c r="B122" t="s">
         <v>781</v>
       </c>
       <c r="D122" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E122" t="s">
         <v>321</v>
@@ -13259,15 +13841,25 @@
       <c r="BI122" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="123" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A123" s="165"/>
+      <c r="BK122" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL122" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM122" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN122"/>
+    </row>
+    <row r="123" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A123" s="140"/>
       <c r="B123" t="s">
         <v>782</v>
       </c>
       <c r="D123" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E123" t="s">
         <v>324</v>
@@ -13358,15 +13950,25 @@
       <c r="BI123" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="124" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A124" s="165"/>
+      <c r="BK123" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL123" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM123" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN123"/>
+    </row>
+    <row r="124" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A124" s="140"/>
       <c r="B124" t="s">
         <v>783</v>
       </c>
       <c r="D124" s="1">
-        <f t="shared" si="11"/>
-        <v>18</v>
+        <f t="shared" si="14"/>
+        <v>21</v>
       </c>
       <c r="E124" t="s">
         <v>327</v>
@@ -13457,9 +14059,19 @@
       <c r="BI124" s="30" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="125" spans="1:61" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="165"/>
+      <c r="BK124" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BL124" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BM124" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="BN124"/>
+    </row>
+    <row r="125" spans="1:66" s="8" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="140"/>
       <c r="C125" s="18"/>
       <c r="D125" s="10"/>
       <c r="G125" s="50"/>
@@ -13498,14 +14110,18 @@
       <c r="AX125" s="33"/>
       <c r="AY125" s="84"/>
       <c r="BB125" s="83"/>
-    </row>
-    <row r="126" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A126" s="165"/>
+      <c r="BK125" s="66"/>
+      <c r="BL125" s="33"/>
+      <c r="BM125" s="33"/>
+      <c r="BN125" s="33"/>
+    </row>
+    <row r="126" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A126" s="140"/>
       <c r="B126" t="s">
         <v>305</v>
       </c>
       <c r="D126" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F126" t="s">
@@ -13543,14 +14159,18 @@
       <c r="AV126"/>
       <c r="AW126"/>
       <c r="AX126"/>
-    </row>
-    <row r="127" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A127" s="165"/>
+      <c r="BK126" s="51"/>
+      <c r="BL126"/>
+      <c r="BM126"/>
+      <c r="BN126"/>
+    </row>
+    <row r="127" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A127" s="140"/>
       <c r="B127" t="s">
         <v>308</v>
       </c>
       <c r="D127" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="E127" t="s">
@@ -13591,14 +14211,18 @@
       <c r="AV127"/>
       <c r="AW127"/>
       <c r="AX127"/>
-    </row>
-    <row r="128" spans="1:61" x14ac:dyDescent="0.25">
-      <c r="A128" s="165"/>
+      <c r="BK127" s="51"/>
+      <c r="BL127"/>
+      <c r="BM127"/>
+      <c r="BN127"/>
+    </row>
+    <row r="128" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A128" s="140"/>
       <c r="B128" t="s">
         <v>311</v>
       </c>
       <c r="D128" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F128" t="s">
@@ -13636,14 +14260,18 @@
       <c r="AV128"/>
       <c r="AW128"/>
       <c r="AX128"/>
-    </row>
-    <row r="129" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A129" s="165"/>
+      <c r="BK128" s="51"/>
+      <c r="BL128"/>
+      <c r="BM128"/>
+      <c r="BN128"/>
+    </row>
+    <row r="129" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A129" s="140"/>
       <c r="B129" t="s">
         <v>314</v>
       </c>
       <c r="D129" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F129" t="s">
@@ -13681,14 +14309,18 @@
       <c r="AV129"/>
       <c r="AW129"/>
       <c r="AX129"/>
-    </row>
-    <row r="130" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A130" s="165"/>
+      <c r="BK129" s="51"/>
+      <c r="BL129"/>
+      <c r="BM129"/>
+      <c r="BN129"/>
+    </row>
+    <row r="130" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A130" s="140"/>
       <c r="B130" t="s">
         <v>317</v>
       </c>
       <c r="D130" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F130" t="s">
@@ -13726,14 +14358,18 @@
       <c r="AV130"/>
       <c r="AW130"/>
       <c r="AX130"/>
-    </row>
-    <row r="131" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A131" s="165"/>
+      <c r="BK130" s="51"/>
+      <c r="BL130"/>
+      <c r="BM130"/>
+      <c r="BN130"/>
+    </row>
+    <row r="131" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A131" s="140"/>
       <c r="B131" t="s">
         <v>320</v>
       </c>
       <c r="D131" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F131" t="s">
@@ -13771,14 +14407,18 @@
       <c r="AV131"/>
       <c r="AW131"/>
       <c r="AX131"/>
-    </row>
-    <row r="132" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A132" s="165"/>
+      <c r="BK131" s="51"/>
+      <c r="BL131"/>
+      <c r="BM131"/>
+      <c r="BN131"/>
+    </row>
+    <row r="132" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A132" s="140"/>
       <c r="B132" t="s">
         <v>323</v>
       </c>
       <c r="D132" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="E132" t="s">
@@ -13819,14 +14459,18 @@
       <c r="AV132"/>
       <c r="AW132"/>
       <c r="AX132"/>
-    </row>
-    <row r="133" spans="1:50" x14ac:dyDescent="0.25">
-      <c r="A133" s="165"/>
+      <c r="BK132" s="51"/>
+      <c r="BL132"/>
+      <c r="BM132"/>
+      <c r="BN132"/>
+    </row>
+    <row r="133" spans="1:66" x14ac:dyDescent="0.25">
+      <c r="A133" s="140"/>
       <c r="B133" t="s">
         <v>326</v>
       </c>
       <c r="D133" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F133" t="s">
@@ -13864,24 +14508,27 @@
       <c r="AV133"/>
       <c r="AW133"/>
       <c r="AX133"/>
+      <c r="BK133" s="51"/>
+      <c r="BL133"/>
+      <c r="BM133"/>
+      <c r="BN133"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="BC9:BJ9"/>
-    <mergeCell ref="AU8:AX8"/>
-    <mergeCell ref="AY8:BB8"/>
-    <mergeCell ref="BC8:BF8"/>
-    <mergeCell ref="BG8:BJ8"/>
-    <mergeCell ref="AU1:AX1"/>
-    <mergeCell ref="AY1:BB1"/>
-    <mergeCell ref="BC1:BF1"/>
-    <mergeCell ref="BG1:BJ1"/>
-    <mergeCell ref="AQ1:AT1"/>
-    <mergeCell ref="AQ8:AT8"/>
-    <mergeCell ref="AM9:AT9"/>
-    <mergeCell ref="AE8:AH8"/>
-    <mergeCell ref="AA8:AD8"/>
-    <mergeCell ref="A108:A115"/>
+  <mergeCells count="45">
+    <mergeCell ref="BK1:BN1"/>
+    <mergeCell ref="BK8:BN8"/>
+    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="AM9:BJ9"/>
+    <mergeCell ref="G10:BJ10"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="O8:R8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="W8:Z8"/>
+    <mergeCell ref="S8:V8"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A117:A133"/>
     <mergeCell ref="AM1:AP1"/>
     <mergeCell ref="AM8:AP8"/>
@@ -13898,18 +14545,21 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="G1:J1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="O8:R8"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="W8:Z8"/>
-    <mergeCell ref="S8:V8"/>
+    <mergeCell ref="AQ8:AT8"/>
+    <mergeCell ref="AE8:AH8"/>
+    <mergeCell ref="AA8:AD8"/>
+    <mergeCell ref="A108:A115"/>
     <mergeCell ref="AI8:AL8"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="D3:F3"/>
     <mergeCell ref="D9:F9"/>
-    <mergeCell ref="AE1:AH1"/>
-    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="AU1:AX1"/>
+    <mergeCell ref="AY1:BB1"/>
+    <mergeCell ref="BC1:BF1"/>
+    <mergeCell ref="BG1:BJ1"/>
+    <mergeCell ref="AQ1:AT1"/>
+    <mergeCell ref="AU8:AX8"/>
+    <mergeCell ref="AY8:BB8"/>
+    <mergeCell ref="BC8:BF8"/>
+    <mergeCell ref="BG8:BJ8"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>